<commit_message>
Devis 2027 : blocs serrage, transport, opérateurs, bandeau forfait ; matériel sans note ; affaire sans rig
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Tool_List_Enedril_2027.xlsx
+++ b/devis_2027/Tool_List_Enedril_2027.xlsx
@@ -888,16 +888,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -911,20 +910,18 @@
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
       <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Dans le classeur Devis, onglet « 2 Matériel » : copier B6:E29 (Bannière, Description, Qté, Note) et coller ici en B6. Aucun prix ici.</t>
+          <t>Dans le classeur Devis, onglet « 2 Matériel » : copier B6:D29 (Bannière, Description, Qté) et coller ici en B6. Aucun prix ici.</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
     </row>
     <row r="3" ht="6" customHeight="1">
       <c r="A3" s="4" t="n"/>
@@ -933,7 +930,6 @@
       <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -956,17 +952,12 @@
           <t>Qté</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Note pour la tool list</t>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Lignes</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Lignes</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Cumul</t>
         </is>
@@ -974,439 +965,415 @@
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="7">
-        <f>IF(AND(F6&gt;0,B6&lt;&gt;"Oui"),COUNTIFS(F$6:F6,"&gt;0",B$6:B6,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E6&gt;0,B6&lt;&gt;"Oui"),COUNTIFS(E$6:E6,"&gt;0",B$6:B6,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="9" t="n"/>
       <c r="D6" s="10" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="11">
+      <c r="E6" s="11">
         <f>IF($C6="",0,IF($B6="Oui",1,IF(N($D6)&gt;0,INT($D6),1)))</f>
         <v/>
       </c>
-      <c r="G6" s="12">
-        <f>SUM(F$6:F6)</f>
+      <c r="F6" s="12">
+        <f>SUM(E$6:E6)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="7">
-        <f>IF(AND(F7&gt;0,B7&lt;&gt;"Oui"),COUNTIFS(F$6:F7,"&gt;0",B$6:B7,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E7&gt;0,B7&lt;&gt;"Oui"),COUNTIFS(E$6:E7,"&gt;0",B$6:B7,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B7" s="8" t="n"/>
       <c r="C7" s="9" t="n"/>
       <c r="D7" s="10" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="11">
+      <c r="E7" s="11">
         <f>IF($C7="",0,IF($B7="Oui",1,IF(N($D7)&gt;0,INT($D7),1)))</f>
         <v/>
       </c>
-      <c r="G7" s="12">
-        <f>SUM(F$6:F7)</f>
+      <c r="F7" s="12">
+        <f>SUM(E$6:E7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="7">
-        <f>IF(AND(F8&gt;0,B8&lt;&gt;"Oui"),COUNTIFS(F$6:F8,"&gt;0",B$6:B8,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E8&gt;0,B8&lt;&gt;"Oui"),COUNTIFS(E$6:E8,"&gt;0",B$6:B8,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="10" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="11">
+      <c r="E8" s="11">
         <f>IF($C8="",0,IF($B8="Oui",1,IF(N($D8)&gt;0,INT($D8),1)))</f>
         <v/>
       </c>
-      <c r="G8" s="12">
-        <f>SUM(F$6:F8)</f>
+      <c r="F8" s="12">
+        <f>SUM(E$6:E8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="7">
-        <f>IF(AND(F9&gt;0,B9&lt;&gt;"Oui"),COUNTIFS(F$6:F9,"&gt;0",B$6:B9,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E9&gt;0,B9&lt;&gt;"Oui"),COUNTIFS(E$6:E9,"&gt;0",B$6:B9,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B9" s="8" t="n"/>
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="10" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="11">
+      <c r="E9" s="11">
         <f>IF($C9="",0,IF($B9="Oui",1,IF(N($D9)&gt;0,INT($D9),1)))</f>
         <v/>
       </c>
-      <c r="G9" s="12">
-        <f>SUM(F$6:F9)</f>
+      <c r="F9" s="12">
+        <f>SUM(E$6:E9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="7">
-        <f>IF(AND(F10&gt;0,B10&lt;&gt;"Oui"),COUNTIFS(F$6:F10,"&gt;0",B$6:B10,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E10&gt;0,B10&lt;&gt;"Oui"),COUNTIFS(E$6:E10,"&gt;0",B$6:B10,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="9" t="n"/>
       <c r="D10" s="10" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="11">
+      <c r="E10" s="11">
         <f>IF($C10="",0,IF($B10="Oui",1,IF(N($D10)&gt;0,INT($D10),1)))</f>
         <v/>
       </c>
-      <c r="G10" s="12">
-        <f>SUM(F$6:F10)</f>
+      <c r="F10" s="12">
+        <f>SUM(E$6:E10)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="7">
-        <f>IF(AND(F11&gt;0,B11&lt;&gt;"Oui"),COUNTIFS(F$6:F11,"&gt;0",B$6:B11,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E11&gt;0,B11&lt;&gt;"Oui"),COUNTIFS(E$6:E11,"&gt;0",B$6:B11,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B11" s="8" t="n"/>
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="10" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="11">
+      <c r="E11" s="11">
         <f>IF($C11="",0,IF($B11="Oui",1,IF(N($D11)&gt;0,INT($D11),1)))</f>
         <v/>
       </c>
-      <c r="G11" s="12">
-        <f>SUM(F$6:F11)</f>
+      <c r="F11" s="12">
+        <f>SUM(E$6:E11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="7">
-        <f>IF(AND(F12&gt;0,B12&lt;&gt;"Oui"),COUNTIFS(F$6:F12,"&gt;0",B$6:B12,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E12&gt;0,B12&lt;&gt;"Oui"),COUNTIFS(E$6:E12,"&gt;0",B$6:B12,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="10" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="11">
+      <c r="E12" s="11">
         <f>IF($C12="",0,IF($B12="Oui",1,IF(N($D12)&gt;0,INT($D12),1)))</f>
         <v/>
       </c>
-      <c r="G12" s="12">
-        <f>SUM(F$6:F12)</f>
+      <c r="F12" s="12">
+        <f>SUM(E$6:E12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="7">
-        <f>IF(AND(F13&gt;0,B13&lt;&gt;"Oui"),COUNTIFS(F$6:F13,"&gt;0",B$6:B13,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E13&gt;0,B13&lt;&gt;"Oui"),COUNTIFS(E$6:E13,"&gt;0",B$6:B13,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B13" s="8" t="n"/>
       <c r="C13" s="9" t="n"/>
       <c r="D13" s="10" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="11">
+      <c r="E13" s="11">
         <f>IF($C13="",0,IF($B13="Oui",1,IF(N($D13)&gt;0,INT($D13),1)))</f>
         <v/>
       </c>
-      <c r="G13" s="12">
-        <f>SUM(F$6:F13)</f>
+      <c r="F13" s="12">
+        <f>SUM(E$6:E13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="7">
-        <f>IF(AND(F14&gt;0,B14&lt;&gt;"Oui"),COUNTIFS(F$6:F14,"&gt;0",B$6:B14,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E14&gt;0,B14&lt;&gt;"Oui"),COUNTIFS(E$6:E14,"&gt;0",B$6:B14,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="10" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="11">
+      <c r="E14" s="11">
         <f>IF($C14="",0,IF($B14="Oui",1,IF(N($D14)&gt;0,INT($D14),1)))</f>
         <v/>
       </c>
-      <c r="G14" s="12">
-        <f>SUM(F$6:F14)</f>
+      <c r="F14" s="12">
+        <f>SUM(E$6:E14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="7">
-        <f>IF(AND(F15&gt;0,B15&lt;&gt;"Oui"),COUNTIFS(F$6:F15,"&gt;0",B$6:B15,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E15&gt;0,B15&lt;&gt;"Oui"),COUNTIFS(E$6:E15,"&gt;0",B$6:B15,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B15" s="8" t="n"/>
       <c r="C15" s="9" t="n"/>
       <c r="D15" s="10" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="11">
+      <c r="E15" s="11">
         <f>IF($C15="",0,IF($B15="Oui",1,IF(N($D15)&gt;0,INT($D15),1)))</f>
         <v/>
       </c>
-      <c r="G15" s="12">
-        <f>SUM(F$6:F15)</f>
+      <c r="F15" s="12">
+        <f>SUM(E$6:E15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="7">
-        <f>IF(AND(F16&gt;0,B16&lt;&gt;"Oui"),COUNTIFS(F$6:F16,"&gt;0",B$6:B16,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E16&gt;0,B16&lt;&gt;"Oui"),COUNTIFS(E$6:E16,"&gt;0",B$6:B16,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B16" s="8" t="n"/>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="10" t="n"/>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="11">
+      <c r="E16" s="11">
         <f>IF($C16="",0,IF($B16="Oui",1,IF(N($D16)&gt;0,INT($D16),1)))</f>
         <v/>
       </c>
-      <c r="G16" s="12">
-        <f>SUM(F$6:F16)</f>
+      <c r="F16" s="12">
+        <f>SUM(E$6:E16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="7">
-        <f>IF(AND(F17&gt;0,B17&lt;&gt;"Oui"),COUNTIFS(F$6:F17,"&gt;0",B$6:B17,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E17&gt;0,B17&lt;&gt;"Oui"),COUNTIFS(E$6:E17,"&gt;0",B$6:B17,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B17" s="8" t="n"/>
       <c r="C17" s="9" t="n"/>
       <c r="D17" s="10" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="11">
+      <c r="E17" s="11">
         <f>IF($C17="",0,IF($B17="Oui",1,IF(N($D17)&gt;0,INT($D17),1)))</f>
         <v/>
       </c>
-      <c r="G17" s="12">
-        <f>SUM(F$6:F17)</f>
+      <c r="F17" s="12">
+        <f>SUM(E$6:E17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="7">
-        <f>IF(AND(F18&gt;0,B18&lt;&gt;"Oui"),COUNTIFS(F$6:F18,"&gt;0",B$6:B18,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E18&gt;0,B18&lt;&gt;"Oui"),COUNTIFS(E$6:E18,"&gt;0",B$6:B18,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B18" s="8" t="n"/>
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="10" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="11">
+      <c r="E18" s="11">
         <f>IF($C18="",0,IF($B18="Oui",1,IF(N($D18)&gt;0,INT($D18),1)))</f>
         <v/>
       </c>
-      <c r="G18" s="12">
-        <f>SUM(F$6:F18)</f>
+      <c r="F18" s="12">
+        <f>SUM(E$6:E18)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="7">
-        <f>IF(AND(F19&gt;0,B19&lt;&gt;"Oui"),COUNTIFS(F$6:F19,"&gt;0",B$6:B19,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E19&gt;0,B19&lt;&gt;"Oui"),COUNTIFS(E$6:E19,"&gt;0",B$6:B19,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B19" s="8" t="n"/>
       <c r="C19" s="9" t="n"/>
       <c r="D19" s="10" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="11">
+      <c r="E19" s="11">
         <f>IF($C19="",0,IF($B19="Oui",1,IF(N($D19)&gt;0,INT($D19),1)))</f>
         <v/>
       </c>
-      <c r="G19" s="12">
-        <f>SUM(F$6:F19)</f>
+      <c r="F19" s="12">
+        <f>SUM(E$6:E19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="7">
-        <f>IF(AND(F20&gt;0,B20&lt;&gt;"Oui"),COUNTIFS(F$6:F20,"&gt;0",B$6:B20,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E20&gt;0,B20&lt;&gt;"Oui"),COUNTIFS(E$6:E20,"&gt;0",B$6:B20,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B20" s="8" t="n"/>
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="10" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="11">
+      <c r="E20" s="11">
         <f>IF($C20="",0,IF($B20="Oui",1,IF(N($D20)&gt;0,INT($D20),1)))</f>
         <v/>
       </c>
-      <c r="G20" s="12">
-        <f>SUM(F$6:F20)</f>
+      <c r="F20" s="12">
+        <f>SUM(E$6:E20)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="7">
-        <f>IF(AND(F21&gt;0,B21&lt;&gt;"Oui"),COUNTIFS(F$6:F21,"&gt;0",B$6:B21,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E21&gt;0,B21&lt;&gt;"Oui"),COUNTIFS(E$6:E21,"&gt;0",B$6:B21,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="9" t="n"/>
       <c r="D21" s="10" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="11">
+      <c r="E21" s="11">
         <f>IF($C21="",0,IF($B21="Oui",1,IF(N($D21)&gt;0,INT($D21),1)))</f>
         <v/>
       </c>
-      <c r="G21" s="12">
-        <f>SUM(F$6:F21)</f>
+      <c r="F21" s="12">
+        <f>SUM(E$6:E21)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
       <c r="A22" s="7">
-        <f>IF(AND(F22&gt;0,B22&lt;&gt;"Oui"),COUNTIFS(F$6:F22,"&gt;0",B$6:B22,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E22&gt;0,B22&lt;&gt;"Oui"),COUNTIFS(E$6:E22,"&gt;0",B$6:B22,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="9" t="n"/>
       <c r="D22" s="10" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="11">
+      <c r="E22" s="11">
         <f>IF($C22="",0,IF($B22="Oui",1,IF(N($D22)&gt;0,INT($D22),1)))</f>
         <v/>
       </c>
-      <c r="G22" s="12">
-        <f>SUM(F$6:F22)</f>
+      <c r="F22" s="12">
+        <f>SUM(E$6:E22)</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="21" customHeight="1">
       <c r="A23" s="7">
-        <f>IF(AND(F23&gt;0,B23&lt;&gt;"Oui"),COUNTIFS(F$6:F23,"&gt;0",B$6:B23,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E23&gt;0,B23&lt;&gt;"Oui"),COUNTIFS(E$6:E23,"&gt;0",B$6:B23,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="9" t="n"/>
       <c r="D23" s="10" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="11">
+      <c r="E23" s="11">
         <f>IF($C23="",0,IF($B23="Oui",1,IF(N($D23)&gt;0,INT($D23),1)))</f>
         <v/>
       </c>
-      <c r="G23" s="12">
-        <f>SUM(F$6:F23)</f>
+      <c r="F23" s="12">
+        <f>SUM(E$6:E23)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="21" customHeight="1">
       <c r="A24" s="7">
-        <f>IF(AND(F24&gt;0,B24&lt;&gt;"Oui"),COUNTIFS(F$6:F24,"&gt;0",B$6:B24,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E24&gt;0,B24&lt;&gt;"Oui"),COUNTIFS(E$6:E24,"&gt;0",B$6:B24,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="9" t="n"/>
       <c r="D24" s="10" t="n"/>
-      <c r="E24" s="9" t="n"/>
-      <c r="F24" s="11">
+      <c r="E24" s="11">
         <f>IF($C24="",0,IF($B24="Oui",1,IF(N($D24)&gt;0,INT($D24),1)))</f>
         <v/>
       </c>
-      <c r="G24" s="12">
-        <f>SUM(F$6:F24)</f>
+      <c r="F24" s="12">
+        <f>SUM(E$6:E24)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="21" customHeight="1">
       <c r="A25" s="7">
-        <f>IF(AND(F25&gt;0,B25&lt;&gt;"Oui"),COUNTIFS(F$6:F25,"&gt;0",B$6:B25,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E25&gt;0,B25&lt;&gt;"Oui"),COUNTIFS(E$6:E25,"&gt;0",B$6:B25,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="9" t="n"/>
       <c r="D25" s="10" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="11">
+      <c r="E25" s="11">
         <f>IF($C25="",0,IF($B25="Oui",1,IF(N($D25)&gt;0,INT($D25),1)))</f>
         <v/>
       </c>
-      <c r="G25" s="12">
-        <f>SUM(F$6:F25)</f>
+      <c r="F25" s="12">
+        <f>SUM(E$6:E25)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="21" customHeight="1">
       <c r="A26" s="7">
-        <f>IF(AND(F26&gt;0,B26&lt;&gt;"Oui"),COUNTIFS(F$6:F26,"&gt;0",B$6:B26,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E26&gt;0,B26&lt;&gt;"Oui"),COUNTIFS(E$6:E26,"&gt;0",B$6:B26,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="10" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="11">
+      <c r="E26" s="11">
         <f>IF($C26="",0,IF($B26="Oui",1,IF(N($D26)&gt;0,INT($D26),1)))</f>
         <v/>
       </c>
-      <c r="G26" s="12">
-        <f>SUM(F$6:F26)</f>
+      <c r="F26" s="12">
+        <f>SUM(E$6:E26)</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="21" customHeight="1">
       <c r="A27" s="7">
-        <f>IF(AND(F27&gt;0,B27&lt;&gt;"Oui"),COUNTIFS(F$6:F27,"&gt;0",B$6:B27,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E27&gt;0,B27&lt;&gt;"Oui"),COUNTIFS(E$6:E27,"&gt;0",B$6:B27,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B27" s="8" t="n"/>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="10" t="n"/>
-      <c r="E27" s="9" t="n"/>
-      <c r="F27" s="11">
+      <c r="E27" s="11">
         <f>IF($C27="",0,IF($B27="Oui",1,IF(N($D27)&gt;0,INT($D27),1)))</f>
         <v/>
       </c>
-      <c r="G27" s="12">
-        <f>SUM(F$6:F27)</f>
+      <c r="F27" s="12">
+        <f>SUM(E$6:E27)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="21" customHeight="1">
       <c r="A28" s="7">
-        <f>IF(AND(F28&gt;0,B28&lt;&gt;"Oui"),COUNTIFS(F$6:F28,"&gt;0",B$6:B28,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E28&gt;0,B28&lt;&gt;"Oui"),COUNTIFS(E$6:E28,"&gt;0",B$6:B28,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B28" s="8" t="n"/>
       <c r="C28" s="9" t="n"/>
       <c r="D28" s="10" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="11">
+      <c r="E28" s="11">
         <f>IF($C28="",0,IF($B28="Oui",1,IF(N($D28)&gt;0,INT($D28),1)))</f>
         <v/>
       </c>
-      <c r="G28" s="12">
-        <f>SUM(F$6:F28)</f>
+      <c r="F28" s="12">
+        <f>SUM(E$6:E28)</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="21" customHeight="1">
       <c r="A29" s="7">
-        <f>IF(AND(F29&gt;0,B29&lt;&gt;"Oui"),COUNTIFS(F$6:F29,"&gt;0",B$6:B29,"&lt;&gt;Oui"),"")</f>
+        <f>IF(AND(E29&gt;0,B29&lt;&gt;"Oui"),COUNTIFS(E$6:E29,"&gt;0",B$6:B29,"&lt;&gt;Oui"),"")</f>
         <v/>
       </c>
       <c r="B29" s="8" t="n"/>
       <c r="C29" s="9" t="n"/>
       <c r="D29" s="10" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="11">
+      <c r="E29" s="11">
         <f>IF($C29="",0,IF($B29="Oui",1,IF(N($D29)&gt;0,INT($D29),1)))</f>
         <v/>
       </c>
-      <c r="G29" s="12">
-        <f>SUM(F$6:F29)</f>
+      <c r="F29" s="12">
+        <f>SUM(E$6:E29)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="C31" s="13">
-        <f>SUM(F6:F29)&amp;" ligne(s) sur la tool list"</f>
+        <f>SUM(E6:E29)&amp;" ligne(s) sur la tool list"</f>
         <v/>
       </c>
     </row>
@@ -1418,7 +1385,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A6:E29">
+  <conditionalFormatting sqref="A6:D29">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$B6="Oui"</formula>
     </cfRule>
@@ -1806,7 +1773,7 @@
       <c r="B15" s="27" t="n"/>
       <c r="C15" s="27" t="n"/>
       <c r="D15" s="28">
-        <f>IF(T15="","",IF(V15=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U15)),INDEX('1 Matériel'!$C$6:$C$29,U15)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U15)&gt;1,"  ("&amp;(T15-INDEX('1 Matériel'!$G$6:$G$29,U15)+INDEX('1 Matériel'!$F$6:$F$29,U15))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U15)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U15)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U15),"")))</f>
+        <f>IF(T15="","",IF(V15=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U15)),INDEX('1 Matériel'!$C$6:$C$29,U15)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U15)&gt;1,"  ("&amp;(T15-INDEX('1 Matériel'!$F$6:$F$29,U15)+INDEX('1 Matériel'!$E$6:$E$29,U15))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U15)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E15" s="29" t="n"/>
@@ -1824,11 +1791,11 @@
       <c r="Q15" s="31" t="n"/>
       <c r="R15" s="30" t="n"/>
       <c r="T15" s="32">
-        <f>IF(1&lt;=SUM('1 Matériel'!$F$6:$F$29),1,"")</f>
+        <f>IF(1&lt;=SUM('1 Matériel'!$E$6:$E$29),1,"")</f>
         <v/>
       </c>
       <c r="U15" s="32">
-        <f>IF(T15="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T15)+1)</f>
+        <f>IF(T15="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T15)+1)</f>
         <v/>
       </c>
       <c r="V15" s="32">
@@ -1844,7 +1811,7 @@
       <c r="B16" s="27" t="n"/>
       <c r="C16" s="27" t="n"/>
       <c r="D16" s="28">
-        <f>IF(T16="","",IF(V16=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U16)),INDEX('1 Matériel'!$C$6:$C$29,U16)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U16)&gt;1,"  ("&amp;(T16-INDEX('1 Matériel'!$G$6:$G$29,U16)+INDEX('1 Matériel'!$F$6:$F$29,U16))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U16)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U16)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U16),"")))</f>
+        <f>IF(T16="","",IF(V16=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U16)),INDEX('1 Matériel'!$C$6:$C$29,U16)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U16)&gt;1,"  ("&amp;(T16-INDEX('1 Matériel'!$F$6:$F$29,U16)+INDEX('1 Matériel'!$E$6:$E$29,U16))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U16)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E16" s="29" t="n"/>
@@ -1862,11 +1829,11 @@
       <c r="Q16" s="31" t="n"/>
       <c r="R16" s="30" t="n"/>
       <c r="T16" s="32">
-        <f>IF(2&lt;=SUM('1 Matériel'!$F$6:$F$29),2,"")</f>
+        <f>IF(2&lt;=SUM('1 Matériel'!$E$6:$E$29),2,"")</f>
         <v/>
       </c>
       <c r="U16" s="32">
-        <f>IF(T16="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T16)+1)</f>
+        <f>IF(T16="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T16)+1)</f>
         <v/>
       </c>
       <c r="V16" s="32">
@@ -1882,7 +1849,7 @@
       <c r="B17" s="27" t="n"/>
       <c r="C17" s="27" t="n"/>
       <c r="D17" s="28">
-        <f>IF(T17="","",IF(V17=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U17)),INDEX('1 Matériel'!$C$6:$C$29,U17)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U17)&gt;1,"  ("&amp;(T17-INDEX('1 Matériel'!$G$6:$G$29,U17)+INDEX('1 Matériel'!$F$6:$F$29,U17))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U17)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U17)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U17),"")))</f>
+        <f>IF(T17="","",IF(V17=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U17)),INDEX('1 Matériel'!$C$6:$C$29,U17)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U17)&gt;1,"  ("&amp;(T17-INDEX('1 Matériel'!$F$6:$F$29,U17)+INDEX('1 Matériel'!$E$6:$E$29,U17))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U17)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E17" s="29" t="n"/>
@@ -1900,11 +1867,11 @@
       <c r="Q17" s="31" t="n"/>
       <c r="R17" s="30" t="n"/>
       <c r="T17" s="32">
-        <f>IF(3&lt;=SUM('1 Matériel'!$F$6:$F$29),3,"")</f>
+        <f>IF(3&lt;=SUM('1 Matériel'!$E$6:$E$29),3,"")</f>
         <v/>
       </c>
       <c r="U17" s="32">
-        <f>IF(T17="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T17)+1)</f>
+        <f>IF(T17="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T17)+1)</f>
         <v/>
       </c>
       <c r="V17" s="32">
@@ -1920,7 +1887,7 @@
       <c r="B18" s="27" t="n"/>
       <c r="C18" s="27" t="n"/>
       <c r="D18" s="28">
-        <f>IF(T18="","",IF(V18=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U18)),INDEX('1 Matériel'!$C$6:$C$29,U18)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U18)&gt;1,"  ("&amp;(T18-INDEX('1 Matériel'!$G$6:$G$29,U18)+INDEX('1 Matériel'!$F$6:$F$29,U18))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U18)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U18)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U18),"")))</f>
+        <f>IF(T18="","",IF(V18=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U18)),INDEX('1 Matériel'!$C$6:$C$29,U18)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U18)&gt;1,"  ("&amp;(T18-INDEX('1 Matériel'!$F$6:$F$29,U18)+INDEX('1 Matériel'!$E$6:$E$29,U18))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U18)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E18" s="29" t="n"/>
@@ -1938,11 +1905,11 @@
       <c r="Q18" s="31" t="n"/>
       <c r="R18" s="30" t="n"/>
       <c r="T18" s="32">
-        <f>IF(4&lt;=SUM('1 Matériel'!$F$6:$F$29),4,"")</f>
+        <f>IF(4&lt;=SUM('1 Matériel'!$E$6:$E$29),4,"")</f>
         <v/>
       </c>
       <c r="U18" s="32">
-        <f>IF(T18="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T18)+1)</f>
+        <f>IF(T18="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T18)+1)</f>
         <v/>
       </c>
       <c r="V18" s="32">
@@ -1958,7 +1925,7 @@
       <c r="B19" s="27" t="n"/>
       <c r="C19" s="27" t="n"/>
       <c r="D19" s="28">
-        <f>IF(T19="","",IF(V19=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U19)),INDEX('1 Matériel'!$C$6:$C$29,U19)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U19)&gt;1,"  ("&amp;(T19-INDEX('1 Matériel'!$G$6:$G$29,U19)+INDEX('1 Matériel'!$F$6:$F$29,U19))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U19)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U19)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U19),"")))</f>
+        <f>IF(T19="","",IF(V19=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U19)),INDEX('1 Matériel'!$C$6:$C$29,U19)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U19)&gt;1,"  ("&amp;(T19-INDEX('1 Matériel'!$F$6:$F$29,U19)+INDEX('1 Matériel'!$E$6:$E$29,U19))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U19)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E19" s="29" t="n"/>
@@ -1976,11 +1943,11 @@
       <c r="Q19" s="31" t="n"/>
       <c r="R19" s="30" t="n"/>
       <c r="T19" s="32">
-        <f>IF(5&lt;=SUM('1 Matériel'!$F$6:$F$29),5,"")</f>
+        <f>IF(5&lt;=SUM('1 Matériel'!$E$6:$E$29),5,"")</f>
         <v/>
       </c>
       <c r="U19" s="32">
-        <f>IF(T19="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T19)+1)</f>
+        <f>IF(T19="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T19)+1)</f>
         <v/>
       </c>
       <c r="V19" s="32">
@@ -1996,7 +1963,7 @@
       <c r="B20" s="27" t="n"/>
       <c r="C20" s="27" t="n"/>
       <c r="D20" s="28">
-        <f>IF(T20="","",IF(V20=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U20)),INDEX('1 Matériel'!$C$6:$C$29,U20)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U20)&gt;1,"  ("&amp;(T20-INDEX('1 Matériel'!$G$6:$G$29,U20)+INDEX('1 Matériel'!$F$6:$F$29,U20))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U20)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U20)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U20),"")))</f>
+        <f>IF(T20="","",IF(V20=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U20)),INDEX('1 Matériel'!$C$6:$C$29,U20)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U20)&gt;1,"  ("&amp;(T20-INDEX('1 Matériel'!$F$6:$F$29,U20)+INDEX('1 Matériel'!$E$6:$E$29,U20))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U20)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E20" s="29" t="n"/>
@@ -2014,11 +1981,11 @@
       <c r="Q20" s="31" t="n"/>
       <c r="R20" s="30" t="n"/>
       <c r="T20" s="32">
-        <f>IF(6&lt;=SUM('1 Matériel'!$F$6:$F$29),6,"")</f>
+        <f>IF(6&lt;=SUM('1 Matériel'!$E$6:$E$29),6,"")</f>
         <v/>
       </c>
       <c r="U20" s="32">
-        <f>IF(T20="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T20)+1)</f>
+        <f>IF(T20="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T20)+1)</f>
         <v/>
       </c>
       <c r="V20" s="32">
@@ -2034,7 +2001,7 @@
       <c r="B21" s="27" t="n"/>
       <c r="C21" s="27" t="n"/>
       <c r="D21" s="28">
-        <f>IF(T21="","",IF(V21=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U21)),INDEX('1 Matériel'!$C$6:$C$29,U21)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U21)&gt;1,"  ("&amp;(T21-INDEX('1 Matériel'!$G$6:$G$29,U21)+INDEX('1 Matériel'!$F$6:$F$29,U21))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U21)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U21)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U21),"")))</f>
+        <f>IF(T21="","",IF(V21=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U21)),INDEX('1 Matériel'!$C$6:$C$29,U21)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U21)&gt;1,"  ("&amp;(T21-INDEX('1 Matériel'!$F$6:$F$29,U21)+INDEX('1 Matériel'!$E$6:$E$29,U21))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U21)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E21" s="29" t="n"/>
@@ -2052,11 +2019,11 @@
       <c r="Q21" s="31" t="n"/>
       <c r="R21" s="30" t="n"/>
       <c r="T21" s="32">
-        <f>IF(7&lt;=SUM('1 Matériel'!$F$6:$F$29),7,"")</f>
+        <f>IF(7&lt;=SUM('1 Matériel'!$E$6:$E$29),7,"")</f>
         <v/>
       </c>
       <c r="U21" s="32">
-        <f>IF(T21="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T21)+1)</f>
+        <f>IF(T21="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T21)+1)</f>
         <v/>
       </c>
       <c r="V21" s="32">
@@ -2072,7 +2039,7 @@
       <c r="B22" s="27" t="n"/>
       <c r="C22" s="27" t="n"/>
       <c r="D22" s="28">
-        <f>IF(T22="","",IF(V22=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U22)),INDEX('1 Matériel'!$C$6:$C$29,U22)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U22)&gt;1,"  ("&amp;(T22-INDEX('1 Matériel'!$G$6:$G$29,U22)+INDEX('1 Matériel'!$F$6:$F$29,U22))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U22)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U22)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U22),"")))</f>
+        <f>IF(T22="","",IF(V22=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U22)),INDEX('1 Matériel'!$C$6:$C$29,U22)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U22)&gt;1,"  ("&amp;(T22-INDEX('1 Matériel'!$F$6:$F$29,U22)+INDEX('1 Matériel'!$E$6:$E$29,U22))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U22)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E22" s="29" t="n"/>
@@ -2090,11 +2057,11 @@
       <c r="Q22" s="31" t="n"/>
       <c r="R22" s="30" t="n"/>
       <c r="T22" s="32">
-        <f>IF(8&lt;=SUM('1 Matériel'!$F$6:$F$29),8,"")</f>
+        <f>IF(8&lt;=SUM('1 Matériel'!$E$6:$E$29),8,"")</f>
         <v/>
       </c>
       <c r="U22" s="32">
-        <f>IF(T22="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T22)+1)</f>
+        <f>IF(T22="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T22)+1)</f>
         <v/>
       </c>
       <c r="V22" s="32">
@@ -2110,7 +2077,7 @@
       <c r="B23" s="27" t="n"/>
       <c r="C23" s="27" t="n"/>
       <c r="D23" s="28">
-        <f>IF(T23="","",IF(V23=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U23)),INDEX('1 Matériel'!$C$6:$C$29,U23)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U23)&gt;1,"  ("&amp;(T23-INDEX('1 Matériel'!$G$6:$G$29,U23)+INDEX('1 Matériel'!$F$6:$F$29,U23))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U23)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U23)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U23),"")))</f>
+        <f>IF(T23="","",IF(V23=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U23)),INDEX('1 Matériel'!$C$6:$C$29,U23)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U23)&gt;1,"  ("&amp;(T23-INDEX('1 Matériel'!$F$6:$F$29,U23)+INDEX('1 Matériel'!$E$6:$E$29,U23))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U23)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E23" s="29" t="n"/>
@@ -2128,11 +2095,11 @@
       <c r="Q23" s="31" t="n"/>
       <c r="R23" s="30" t="n"/>
       <c r="T23" s="32">
-        <f>IF(9&lt;=SUM('1 Matériel'!$F$6:$F$29),9,"")</f>
+        <f>IF(9&lt;=SUM('1 Matériel'!$E$6:$E$29),9,"")</f>
         <v/>
       </c>
       <c r="U23" s="32">
-        <f>IF(T23="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T23)+1)</f>
+        <f>IF(T23="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T23)+1)</f>
         <v/>
       </c>
       <c r="V23" s="32">
@@ -2148,7 +2115,7 @@
       <c r="B24" s="27" t="n"/>
       <c r="C24" s="27" t="n"/>
       <c r="D24" s="28">
-        <f>IF(T24="","",IF(V24=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U24)),INDEX('1 Matériel'!$C$6:$C$29,U24)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U24)&gt;1,"  ("&amp;(T24-INDEX('1 Matériel'!$G$6:$G$29,U24)+INDEX('1 Matériel'!$F$6:$F$29,U24))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U24)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U24)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U24),"")))</f>
+        <f>IF(T24="","",IF(V24=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U24)),INDEX('1 Matériel'!$C$6:$C$29,U24)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U24)&gt;1,"  ("&amp;(T24-INDEX('1 Matériel'!$F$6:$F$29,U24)+INDEX('1 Matériel'!$E$6:$E$29,U24))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U24)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E24" s="29" t="n"/>
@@ -2166,11 +2133,11 @@
       <c r="Q24" s="31" t="n"/>
       <c r="R24" s="30" t="n"/>
       <c r="T24" s="32">
-        <f>IF(10&lt;=SUM('1 Matériel'!$F$6:$F$29),10,"")</f>
+        <f>IF(10&lt;=SUM('1 Matériel'!$E$6:$E$29),10,"")</f>
         <v/>
       </c>
       <c r="U24" s="32">
-        <f>IF(T24="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T24)+1)</f>
+        <f>IF(T24="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T24)+1)</f>
         <v/>
       </c>
       <c r="V24" s="32">
@@ -2186,7 +2153,7 @@
       <c r="B25" s="27" t="n"/>
       <c r="C25" s="27" t="n"/>
       <c r="D25" s="28">
-        <f>IF(T25="","",IF(V25=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U25)),INDEX('1 Matériel'!$C$6:$C$29,U25)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U25)&gt;1,"  ("&amp;(T25-INDEX('1 Matériel'!$G$6:$G$29,U25)+INDEX('1 Matériel'!$F$6:$F$29,U25))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U25)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U25)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U25),"")))</f>
+        <f>IF(T25="","",IF(V25=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U25)),INDEX('1 Matériel'!$C$6:$C$29,U25)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U25)&gt;1,"  ("&amp;(T25-INDEX('1 Matériel'!$F$6:$F$29,U25)+INDEX('1 Matériel'!$E$6:$E$29,U25))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U25)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E25" s="29" t="n"/>
@@ -2204,11 +2171,11 @@
       <c r="Q25" s="31" t="n"/>
       <c r="R25" s="30" t="n"/>
       <c r="T25" s="32">
-        <f>IF(11&lt;=SUM('1 Matériel'!$F$6:$F$29),11,"")</f>
+        <f>IF(11&lt;=SUM('1 Matériel'!$E$6:$E$29),11,"")</f>
         <v/>
       </c>
       <c r="U25" s="32">
-        <f>IF(T25="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T25)+1)</f>
+        <f>IF(T25="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T25)+1)</f>
         <v/>
       </c>
       <c r="V25" s="32">
@@ -2224,7 +2191,7 @@
       <c r="B26" s="27" t="n"/>
       <c r="C26" s="27" t="n"/>
       <c r="D26" s="28">
-        <f>IF(T26="","",IF(V26=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U26)),INDEX('1 Matériel'!$C$6:$C$29,U26)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U26)&gt;1,"  ("&amp;(T26-INDEX('1 Matériel'!$G$6:$G$29,U26)+INDEX('1 Matériel'!$F$6:$F$29,U26))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U26)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U26)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U26),"")))</f>
+        <f>IF(T26="","",IF(V26=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U26)),INDEX('1 Matériel'!$C$6:$C$29,U26)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U26)&gt;1,"  ("&amp;(T26-INDEX('1 Matériel'!$F$6:$F$29,U26)+INDEX('1 Matériel'!$E$6:$E$29,U26))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U26)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E26" s="29" t="n"/>
@@ -2242,11 +2209,11 @@
       <c r="Q26" s="31" t="n"/>
       <c r="R26" s="30" t="n"/>
       <c r="T26" s="32">
-        <f>IF(12&lt;=SUM('1 Matériel'!$F$6:$F$29),12,"")</f>
+        <f>IF(12&lt;=SUM('1 Matériel'!$E$6:$E$29),12,"")</f>
         <v/>
       </c>
       <c r="U26" s="32">
-        <f>IF(T26="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T26)+1)</f>
+        <f>IF(T26="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T26)+1)</f>
         <v/>
       </c>
       <c r="V26" s="32">
@@ -2262,7 +2229,7 @@
       <c r="B27" s="27" t="n"/>
       <c r="C27" s="27" t="n"/>
       <c r="D27" s="28">
-        <f>IF(T27="","",IF(V27=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U27)),INDEX('1 Matériel'!$C$6:$C$29,U27)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U27)&gt;1,"  ("&amp;(T27-INDEX('1 Matériel'!$G$6:$G$29,U27)+INDEX('1 Matériel'!$F$6:$F$29,U27))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U27)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U27)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U27),"")))</f>
+        <f>IF(T27="","",IF(V27=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U27)),INDEX('1 Matériel'!$C$6:$C$29,U27)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U27)&gt;1,"  ("&amp;(T27-INDEX('1 Matériel'!$F$6:$F$29,U27)+INDEX('1 Matériel'!$E$6:$E$29,U27))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U27)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E27" s="29" t="n"/>
@@ -2280,11 +2247,11 @@
       <c r="Q27" s="31" t="n"/>
       <c r="R27" s="30" t="n"/>
       <c r="T27" s="32">
-        <f>IF(13&lt;=SUM('1 Matériel'!$F$6:$F$29),13,"")</f>
+        <f>IF(13&lt;=SUM('1 Matériel'!$E$6:$E$29),13,"")</f>
         <v/>
       </c>
       <c r="U27" s="32">
-        <f>IF(T27="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T27)+1)</f>
+        <f>IF(T27="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T27)+1)</f>
         <v/>
       </c>
       <c r="V27" s="32">
@@ -2300,7 +2267,7 @@
       <c r="B28" s="27" t="n"/>
       <c r="C28" s="27" t="n"/>
       <c r="D28" s="28">
-        <f>IF(T28="","",IF(V28=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U28)),INDEX('1 Matériel'!$C$6:$C$29,U28)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U28)&gt;1,"  ("&amp;(T28-INDEX('1 Matériel'!$G$6:$G$29,U28)+INDEX('1 Matériel'!$F$6:$F$29,U28))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U28)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U28)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U28),"")))</f>
+        <f>IF(T28="","",IF(V28=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U28)),INDEX('1 Matériel'!$C$6:$C$29,U28)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U28)&gt;1,"  ("&amp;(T28-INDEX('1 Matériel'!$F$6:$F$29,U28)+INDEX('1 Matériel'!$E$6:$E$29,U28))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U28)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E28" s="29" t="n"/>
@@ -2318,11 +2285,11 @@
       <c r="Q28" s="31" t="n"/>
       <c r="R28" s="30" t="n"/>
       <c r="T28" s="32">
-        <f>IF(14&lt;=SUM('1 Matériel'!$F$6:$F$29),14,"")</f>
+        <f>IF(14&lt;=SUM('1 Matériel'!$E$6:$E$29),14,"")</f>
         <v/>
       </c>
       <c r="U28" s="32">
-        <f>IF(T28="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T28)+1)</f>
+        <f>IF(T28="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T28)+1)</f>
         <v/>
       </c>
       <c r="V28" s="32">
@@ -2338,7 +2305,7 @@
       <c r="B29" s="27" t="n"/>
       <c r="C29" s="27" t="n"/>
       <c r="D29" s="28">
-        <f>IF(T29="","",IF(V29=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U29)),INDEX('1 Matériel'!$C$6:$C$29,U29)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U29)&gt;1,"  ("&amp;(T29-INDEX('1 Matériel'!$G$6:$G$29,U29)+INDEX('1 Matériel'!$F$6:$F$29,U29))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U29)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U29)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U29),"")))</f>
+        <f>IF(T29="","",IF(V29=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U29)),INDEX('1 Matériel'!$C$6:$C$29,U29)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U29)&gt;1,"  ("&amp;(T29-INDEX('1 Matériel'!$F$6:$F$29,U29)+INDEX('1 Matériel'!$E$6:$E$29,U29))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U29)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E29" s="29" t="n"/>
@@ -2356,11 +2323,11 @@
       <c r="Q29" s="31" t="n"/>
       <c r="R29" s="30" t="n"/>
       <c r="T29" s="32">
-        <f>IF(15&lt;=SUM('1 Matériel'!$F$6:$F$29),15,"")</f>
+        <f>IF(15&lt;=SUM('1 Matériel'!$E$6:$E$29),15,"")</f>
         <v/>
       </c>
       <c r="U29" s="32">
-        <f>IF(T29="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T29)+1)</f>
+        <f>IF(T29="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T29)+1)</f>
         <v/>
       </c>
       <c r="V29" s="32">
@@ -2376,7 +2343,7 @@
       <c r="B30" s="27" t="n"/>
       <c r="C30" s="27" t="n"/>
       <c r="D30" s="28">
-        <f>IF(T30="","",IF(V30=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U30)),INDEX('1 Matériel'!$C$6:$C$29,U30)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U30)&gt;1,"  ("&amp;(T30-INDEX('1 Matériel'!$G$6:$G$29,U30)+INDEX('1 Matériel'!$F$6:$F$29,U30))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U30)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U30)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U30),"")))</f>
+        <f>IF(T30="","",IF(V30=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U30)),INDEX('1 Matériel'!$C$6:$C$29,U30)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U30)&gt;1,"  ("&amp;(T30-INDEX('1 Matériel'!$F$6:$F$29,U30)+INDEX('1 Matériel'!$E$6:$E$29,U30))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U30)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E30" s="29" t="n"/>
@@ -2394,11 +2361,11 @@
       <c r="Q30" s="31" t="n"/>
       <c r="R30" s="30" t="n"/>
       <c r="T30" s="32">
-        <f>IF(16&lt;=SUM('1 Matériel'!$F$6:$F$29),16,"")</f>
+        <f>IF(16&lt;=SUM('1 Matériel'!$E$6:$E$29),16,"")</f>
         <v/>
       </c>
       <c r="U30" s="32">
-        <f>IF(T30="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T30)+1)</f>
+        <f>IF(T30="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T30)+1)</f>
         <v/>
       </c>
       <c r="V30" s="32">
@@ -2414,7 +2381,7 @@
       <c r="B31" s="27" t="n"/>
       <c r="C31" s="27" t="n"/>
       <c r="D31" s="28">
-        <f>IF(T31="","",IF(V31=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U31)),INDEX('1 Matériel'!$C$6:$C$29,U31)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U31)&gt;1,"  ("&amp;(T31-INDEX('1 Matériel'!$G$6:$G$29,U31)+INDEX('1 Matériel'!$F$6:$F$29,U31))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U31)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U31)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U31),"")))</f>
+        <f>IF(T31="","",IF(V31=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U31)),INDEX('1 Matériel'!$C$6:$C$29,U31)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U31)&gt;1,"  ("&amp;(T31-INDEX('1 Matériel'!$F$6:$F$29,U31)+INDEX('1 Matériel'!$E$6:$E$29,U31))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U31)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E31" s="29" t="n"/>
@@ -2432,11 +2399,11 @@
       <c r="Q31" s="31" t="n"/>
       <c r="R31" s="30" t="n"/>
       <c r="T31" s="32">
-        <f>IF(17&lt;=SUM('1 Matériel'!$F$6:$F$29),17,"")</f>
+        <f>IF(17&lt;=SUM('1 Matériel'!$E$6:$E$29),17,"")</f>
         <v/>
       </c>
       <c r="U31" s="32">
-        <f>IF(T31="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T31)+1)</f>
+        <f>IF(T31="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T31)+1)</f>
         <v/>
       </c>
       <c r="V31" s="32">
@@ -2452,7 +2419,7 @@
       <c r="B32" s="27" t="n"/>
       <c r="C32" s="27" t="n"/>
       <c r="D32" s="28">
-        <f>IF(T32="","",IF(V32=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U32)),INDEX('1 Matériel'!$C$6:$C$29,U32)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U32)&gt;1,"  ("&amp;(T32-INDEX('1 Matériel'!$G$6:$G$29,U32)+INDEX('1 Matériel'!$F$6:$F$29,U32))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U32)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U32)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U32),"")))</f>
+        <f>IF(T32="","",IF(V32=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U32)),INDEX('1 Matériel'!$C$6:$C$29,U32)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U32)&gt;1,"  ("&amp;(T32-INDEX('1 Matériel'!$F$6:$F$29,U32)+INDEX('1 Matériel'!$E$6:$E$29,U32))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U32)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E32" s="29" t="n"/>
@@ -2470,11 +2437,11 @@
       <c r="Q32" s="31" t="n"/>
       <c r="R32" s="30" t="n"/>
       <c r="T32" s="32">
-        <f>IF(18&lt;=SUM('1 Matériel'!$F$6:$F$29),18,"")</f>
+        <f>IF(18&lt;=SUM('1 Matériel'!$E$6:$E$29),18,"")</f>
         <v/>
       </c>
       <c r="U32" s="32">
-        <f>IF(T32="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T32)+1)</f>
+        <f>IF(T32="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T32)+1)</f>
         <v/>
       </c>
       <c r="V32" s="32">
@@ -2490,7 +2457,7 @@
       <c r="B33" s="27" t="n"/>
       <c r="C33" s="27" t="n"/>
       <c r="D33" s="28">
-        <f>IF(T33="","",IF(V33=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U33)),INDEX('1 Matériel'!$C$6:$C$29,U33)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U33)&gt;1,"  ("&amp;(T33-INDEX('1 Matériel'!$G$6:$G$29,U33)+INDEX('1 Matériel'!$F$6:$F$29,U33))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U33)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U33)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U33),"")))</f>
+        <f>IF(T33="","",IF(V33=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U33)),INDEX('1 Matériel'!$C$6:$C$29,U33)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U33)&gt;1,"  ("&amp;(T33-INDEX('1 Matériel'!$F$6:$F$29,U33)+INDEX('1 Matériel'!$E$6:$E$29,U33))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U33)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E33" s="29" t="n"/>
@@ -2508,11 +2475,11 @@
       <c r="Q33" s="31" t="n"/>
       <c r="R33" s="30" t="n"/>
       <c r="T33" s="32">
-        <f>IF(19&lt;=SUM('1 Matériel'!$F$6:$F$29),19,"")</f>
+        <f>IF(19&lt;=SUM('1 Matériel'!$E$6:$E$29),19,"")</f>
         <v/>
       </c>
       <c r="U33" s="32">
-        <f>IF(T33="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T33)+1)</f>
+        <f>IF(T33="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T33)+1)</f>
         <v/>
       </c>
       <c r="V33" s="32">
@@ -2528,7 +2495,7 @@
       <c r="B34" s="27" t="n"/>
       <c r="C34" s="27" t="n"/>
       <c r="D34" s="28">
-        <f>IF(T34="","",IF(V34=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U34)),INDEX('1 Matériel'!$C$6:$C$29,U34)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U34)&gt;1,"  ("&amp;(T34-INDEX('1 Matériel'!$G$6:$G$29,U34)+INDEX('1 Matériel'!$F$6:$F$29,U34))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U34)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U34)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U34),"")))</f>
+        <f>IF(T34="","",IF(V34=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U34)),INDEX('1 Matériel'!$C$6:$C$29,U34)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U34)&gt;1,"  ("&amp;(T34-INDEX('1 Matériel'!$F$6:$F$29,U34)+INDEX('1 Matériel'!$E$6:$E$29,U34))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U34)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E34" s="29" t="n"/>
@@ -2546,11 +2513,11 @@
       <c r="Q34" s="31" t="n"/>
       <c r="R34" s="30" t="n"/>
       <c r="T34" s="32">
-        <f>IF(20&lt;=SUM('1 Matériel'!$F$6:$F$29),20,"")</f>
+        <f>IF(20&lt;=SUM('1 Matériel'!$E$6:$E$29),20,"")</f>
         <v/>
       </c>
       <c r="U34" s="32">
-        <f>IF(T34="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T34)+1)</f>
+        <f>IF(T34="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T34)+1)</f>
         <v/>
       </c>
       <c r="V34" s="32">
@@ -2566,7 +2533,7 @@
       <c r="B35" s="27" t="n"/>
       <c r="C35" s="27" t="n"/>
       <c r="D35" s="28">
-        <f>IF(T35="","",IF(V35=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U35)),INDEX('1 Matériel'!$C$6:$C$29,U35)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U35)&gt;1,"  ("&amp;(T35-INDEX('1 Matériel'!$G$6:$G$29,U35)+INDEX('1 Matériel'!$F$6:$F$29,U35))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U35)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U35)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U35),"")))</f>
+        <f>IF(T35="","",IF(V35=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U35)),INDEX('1 Matériel'!$C$6:$C$29,U35)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U35)&gt;1,"  ("&amp;(T35-INDEX('1 Matériel'!$F$6:$F$29,U35)+INDEX('1 Matériel'!$E$6:$E$29,U35))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U35)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E35" s="29" t="n"/>
@@ -2584,11 +2551,11 @@
       <c r="Q35" s="31" t="n"/>
       <c r="R35" s="30" t="n"/>
       <c r="T35" s="32">
-        <f>IF(21&lt;=SUM('1 Matériel'!$F$6:$F$29),21,"")</f>
+        <f>IF(21&lt;=SUM('1 Matériel'!$E$6:$E$29),21,"")</f>
         <v/>
       </c>
       <c r="U35" s="32">
-        <f>IF(T35="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T35)+1)</f>
+        <f>IF(T35="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T35)+1)</f>
         <v/>
       </c>
       <c r="V35" s="32">
@@ -2604,7 +2571,7 @@
       <c r="B36" s="27" t="n"/>
       <c r="C36" s="27" t="n"/>
       <c r="D36" s="28">
-        <f>IF(T36="","",IF(V36=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U36)),INDEX('1 Matériel'!$C$6:$C$29,U36)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U36)&gt;1,"  ("&amp;(T36-INDEX('1 Matériel'!$G$6:$G$29,U36)+INDEX('1 Matériel'!$F$6:$F$29,U36))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U36)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U36)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U36),"")))</f>
+        <f>IF(T36="","",IF(V36=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U36)),INDEX('1 Matériel'!$C$6:$C$29,U36)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U36)&gt;1,"  ("&amp;(T36-INDEX('1 Matériel'!$F$6:$F$29,U36)+INDEX('1 Matériel'!$E$6:$E$29,U36))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U36)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E36" s="29" t="n"/>
@@ -2622,11 +2589,11 @@
       <c r="Q36" s="31" t="n"/>
       <c r="R36" s="30" t="n"/>
       <c r="T36" s="32">
-        <f>IF(22&lt;=SUM('1 Matériel'!$F$6:$F$29),22,"")</f>
+        <f>IF(22&lt;=SUM('1 Matériel'!$E$6:$E$29),22,"")</f>
         <v/>
       </c>
       <c r="U36" s="32">
-        <f>IF(T36="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T36)+1)</f>
+        <f>IF(T36="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T36)+1)</f>
         <v/>
       </c>
       <c r="V36" s="32">
@@ -2642,7 +2609,7 @@
       <c r="B37" s="27" t="n"/>
       <c r="C37" s="27" t="n"/>
       <c r="D37" s="28">
-        <f>IF(T37="","",IF(V37=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U37)),INDEX('1 Matériel'!$C$6:$C$29,U37)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U37)&gt;1,"  ("&amp;(T37-INDEX('1 Matériel'!$G$6:$G$29,U37)+INDEX('1 Matériel'!$F$6:$F$29,U37))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U37)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U37)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U37),"")))</f>
+        <f>IF(T37="","",IF(V37=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U37)),INDEX('1 Matériel'!$C$6:$C$29,U37)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U37)&gt;1,"  ("&amp;(T37-INDEX('1 Matériel'!$F$6:$F$29,U37)+INDEX('1 Matériel'!$E$6:$E$29,U37))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U37)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E37" s="29" t="n"/>
@@ -2660,11 +2627,11 @@
       <c r="Q37" s="31" t="n"/>
       <c r="R37" s="30" t="n"/>
       <c r="T37" s="32">
-        <f>IF(23&lt;=SUM('1 Matériel'!$F$6:$F$29),23,"")</f>
+        <f>IF(23&lt;=SUM('1 Matériel'!$E$6:$E$29),23,"")</f>
         <v/>
       </c>
       <c r="U37" s="32">
-        <f>IF(T37="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T37)+1)</f>
+        <f>IF(T37="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T37)+1)</f>
         <v/>
       </c>
       <c r="V37" s="32">
@@ -2680,7 +2647,7 @@
       <c r="B38" s="27" t="n"/>
       <c r="C38" s="27" t="n"/>
       <c r="D38" s="28">
-        <f>IF(T38="","",IF(V38=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U38)),INDEX('1 Matériel'!$C$6:$C$29,U38)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U38)&gt;1,"  ("&amp;(T38-INDEX('1 Matériel'!$G$6:$G$29,U38)+INDEX('1 Matériel'!$F$6:$F$29,U38))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U38)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U38)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U38),"")))</f>
+        <f>IF(T38="","",IF(V38=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U38)),INDEX('1 Matériel'!$C$6:$C$29,U38)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U38)&gt;1,"  ("&amp;(T38-INDEX('1 Matériel'!$F$6:$F$29,U38)+INDEX('1 Matériel'!$E$6:$E$29,U38))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U38)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E38" s="29" t="n"/>
@@ -2698,11 +2665,11 @@
       <c r="Q38" s="31" t="n"/>
       <c r="R38" s="30" t="n"/>
       <c r="T38" s="32">
-        <f>IF(24&lt;=SUM('1 Matériel'!$F$6:$F$29),24,"")</f>
+        <f>IF(24&lt;=SUM('1 Matériel'!$E$6:$E$29),24,"")</f>
         <v/>
       </c>
       <c r="U38" s="32">
-        <f>IF(T38="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T38)+1)</f>
+        <f>IF(T38="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T38)+1)</f>
         <v/>
       </c>
       <c r="V38" s="32">
@@ -2718,7 +2685,7 @@
       <c r="B39" s="27" t="n"/>
       <c r="C39" s="27" t="n"/>
       <c r="D39" s="28">
-        <f>IF(T39="","",IF(V39=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U39)),INDEX('1 Matériel'!$C$6:$C$29,U39)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U39)&gt;1,"  ("&amp;(T39-INDEX('1 Matériel'!$G$6:$G$29,U39)+INDEX('1 Matériel'!$F$6:$F$29,U39))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U39)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U39)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U39),"")))</f>
+        <f>IF(T39="","",IF(V39=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U39)),INDEX('1 Matériel'!$C$6:$C$29,U39)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U39)&gt;1,"  ("&amp;(T39-INDEX('1 Matériel'!$F$6:$F$29,U39)+INDEX('1 Matériel'!$E$6:$E$29,U39))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U39)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E39" s="29" t="n"/>
@@ -2736,11 +2703,11 @@
       <c r="Q39" s="31" t="n"/>
       <c r="R39" s="30" t="n"/>
       <c r="T39" s="32">
-        <f>IF(25&lt;=SUM('1 Matériel'!$F$6:$F$29),25,"")</f>
+        <f>IF(25&lt;=SUM('1 Matériel'!$E$6:$E$29),25,"")</f>
         <v/>
       </c>
       <c r="U39" s="32">
-        <f>IF(T39="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T39)+1)</f>
+        <f>IF(T39="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T39)+1)</f>
         <v/>
       </c>
       <c r="V39" s="32">
@@ -2756,7 +2723,7 @@
       <c r="B40" s="27" t="n"/>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="28">
-        <f>IF(T40="","",IF(V40=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U40)),INDEX('1 Matériel'!$C$6:$C$29,U40)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U40)&gt;1,"  ("&amp;(T40-INDEX('1 Matériel'!$G$6:$G$29,U40)+INDEX('1 Matériel'!$F$6:$F$29,U40))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U40)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U40)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U40),"")))</f>
+        <f>IF(T40="","",IF(V40=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U40)),INDEX('1 Matériel'!$C$6:$C$29,U40)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U40)&gt;1,"  ("&amp;(T40-INDEX('1 Matériel'!$F$6:$F$29,U40)+INDEX('1 Matériel'!$E$6:$E$29,U40))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U40)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E40" s="29" t="n"/>
@@ -2774,11 +2741,11 @@
       <c r="Q40" s="31" t="n"/>
       <c r="R40" s="30" t="n"/>
       <c r="T40" s="32">
-        <f>IF(26&lt;=SUM('1 Matériel'!$F$6:$F$29),26,"")</f>
+        <f>IF(26&lt;=SUM('1 Matériel'!$E$6:$E$29),26,"")</f>
         <v/>
       </c>
       <c r="U40" s="32">
-        <f>IF(T40="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T40)+1)</f>
+        <f>IF(T40="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T40)+1)</f>
         <v/>
       </c>
       <c r="V40" s="32">
@@ -2794,7 +2761,7 @@
       <c r="B41" s="27" t="n"/>
       <c r="C41" s="27" t="n"/>
       <c r="D41" s="28">
-        <f>IF(T41="","",IF(V41=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U41)),INDEX('1 Matériel'!$C$6:$C$29,U41)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U41)&gt;1,"  ("&amp;(T41-INDEX('1 Matériel'!$G$6:$G$29,U41)+INDEX('1 Matériel'!$F$6:$F$29,U41))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U41)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U41)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U41),"")))</f>
+        <f>IF(T41="","",IF(V41=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U41)),INDEX('1 Matériel'!$C$6:$C$29,U41)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U41)&gt;1,"  ("&amp;(T41-INDEX('1 Matériel'!$F$6:$F$29,U41)+INDEX('1 Matériel'!$E$6:$E$29,U41))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U41)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E41" s="29" t="n"/>
@@ -2812,11 +2779,11 @@
       <c r="Q41" s="31" t="n"/>
       <c r="R41" s="30" t="n"/>
       <c r="T41" s="32">
-        <f>IF(27&lt;=SUM('1 Matériel'!$F$6:$F$29),27,"")</f>
+        <f>IF(27&lt;=SUM('1 Matériel'!$E$6:$E$29),27,"")</f>
         <v/>
       </c>
       <c r="U41" s="32">
-        <f>IF(T41="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T41)+1)</f>
+        <f>IF(T41="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T41)+1)</f>
         <v/>
       </c>
       <c r="V41" s="32">
@@ -2832,7 +2799,7 @@
       <c r="B42" s="27" t="n"/>
       <c r="C42" s="27" t="n"/>
       <c r="D42" s="28">
-        <f>IF(T42="","",IF(V42=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U42)),INDEX('1 Matériel'!$C$6:$C$29,U42)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U42)&gt;1,"  ("&amp;(T42-INDEX('1 Matériel'!$G$6:$G$29,U42)+INDEX('1 Matériel'!$F$6:$F$29,U42))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U42)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U42)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U42),"")))</f>
+        <f>IF(T42="","",IF(V42=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U42)),INDEX('1 Matériel'!$C$6:$C$29,U42)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U42)&gt;1,"  ("&amp;(T42-INDEX('1 Matériel'!$F$6:$F$29,U42)+INDEX('1 Matériel'!$E$6:$E$29,U42))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U42)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E42" s="29" t="n"/>
@@ -2850,11 +2817,11 @@
       <c r="Q42" s="31" t="n"/>
       <c r="R42" s="30" t="n"/>
       <c r="T42" s="32">
-        <f>IF(28&lt;=SUM('1 Matériel'!$F$6:$F$29),28,"")</f>
+        <f>IF(28&lt;=SUM('1 Matériel'!$E$6:$E$29),28,"")</f>
         <v/>
       </c>
       <c r="U42" s="32">
-        <f>IF(T42="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T42)+1)</f>
+        <f>IF(T42="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T42)+1)</f>
         <v/>
       </c>
       <c r="V42" s="32">
@@ -2870,7 +2837,7 @@
       <c r="B43" s="27" t="n"/>
       <c r="C43" s="27" t="n"/>
       <c r="D43" s="28">
-        <f>IF(T43="","",IF(V43=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U43)),INDEX('1 Matériel'!$C$6:$C$29,U43)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U43)&gt;1,"  ("&amp;(T43-INDEX('1 Matériel'!$G$6:$G$29,U43)+INDEX('1 Matériel'!$F$6:$F$29,U43))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U43)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U43)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U43),"")))</f>
+        <f>IF(T43="","",IF(V43=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U43)),INDEX('1 Matériel'!$C$6:$C$29,U43)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U43)&gt;1,"  ("&amp;(T43-INDEX('1 Matériel'!$F$6:$F$29,U43)+INDEX('1 Matériel'!$E$6:$E$29,U43))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U43)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E43" s="29" t="n"/>
@@ -2888,11 +2855,11 @@
       <c r="Q43" s="31" t="n"/>
       <c r="R43" s="30" t="n"/>
       <c r="T43" s="32">
-        <f>IF(29&lt;=SUM('1 Matériel'!$F$6:$F$29),29,"")</f>
+        <f>IF(29&lt;=SUM('1 Matériel'!$E$6:$E$29),29,"")</f>
         <v/>
       </c>
       <c r="U43" s="32">
-        <f>IF(T43="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T43)+1)</f>
+        <f>IF(T43="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T43)+1)</f>
         <v/>
       </c>
       <c r="V43" s="32">
@@ -2908,7 +2875,7 @@
       <c r="B44" s="27" t="n"/>
       <c r="C44" s="27" t="n"/>
       <c r="D44" s="28">
-        <f>IF(T44="","",IF(V44=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U44)),INDEX('1 Matériel'!$C$6:$C$29,U44)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U44)&gt;1,"  ("&amp;(T44-INDEX('1 Matériel'!$G$6:$G$29,U44)+INDEX('1 Matériel'!$F$6:$F$29,U44))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U44)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U44)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U44),"")))</f>
+        <f>IF(T44="","",IF(V44=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U44)),INDEX('1 Matériel'!$C$6:$C$29,U44)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U44)&gt;1,"  ("&amp;(T44-INDEX('1 Matériel'!$F$6:$F$29,U44)+INDEX('1 Matériel'!$E$6:$E$29,U44))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U44)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E44" s="29" t="n"/>
@@ -2926,11 +2893,11 @@
       <c r="Q44" s="31" t="n"/>
       <c r="R44" s="30" t="n"/>
       <c r="T44" s="32">
-        <f>IF(30&lt;=SUM('1 Matériel'!$F$6:$F$29),30,"")</f>
+        <f>IF(30&lt;=SUM('1 Matériel'!$E$6:$E$29),30,"")</f>
         <v/>
       </c>
       <c r="U44" s="32">
-        <f>IF(T44="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T44)+1)</f>
+        <f>IF(T44="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T44)+1)</f>
         <v/>
       </c>
       <c r="V44" s="32">
@@ -2946,7 +2913,7 @@
       <c r="B45" s="27" t="n"/>
       <c r="C45" s="27" t="n"/>
       <c r="D45" s="28">
-        <f>IF(T45="","",IF(V45=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U45)),INDEX('1 Matériel'!$C$6:$C$29,U45)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U45)&gt;1,"  ("&amp;(T45-INDEX('1 Matériel'!$G$6:$G$29,U45)+INDEX('1 Matériel'!$F$6:$F$29,U45))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U45)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U45)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U45),"")))</f>
+        <f>IF(T45="","",IF(V45=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U45)),INDEX('1 Matériel'!$C$6:$C$29,U45)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U45)&gt;1,"  ("&amp;(T45-INDEX('1 Matériel'!$F$6:$F$29,U45)+INDEX('1 Matériel'!$E$6:$E$29,U45))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U45)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E45" s="29" t="n"/>
@@ -2964,11 +2931,11 @@
       <c r="Q45" s="31" t="n"/>
       <c r="R45" s="30" t="n"/>
       <c r="T45" s="32">
-        <f>IF(31&lt;=SUM('1 Matériel'!$F$6:$F$29),31,"")</f>
+        <f>IF(31&lt;=SUM('1 Matériel'!$E$6:$E$29),31,"")</f>
         <v/>
       </c>
       <c r="U45" s="32">
-        <f>IF(T45="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T45)+1)</f>
+        <f>IF(T45="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T45)+1)</f>
         <v/>
       </c>
       <c r="V45" s="32">
@@ -2984,7 +2951,7 @@
       <c r="B46" s="27" t="n"/>
       <c r="C46" s="27" t="n"/>
       <c r="D46" s="28">
-        <f>IF(T46="","",IF(V46=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U46)),INDEX('1 Matériel'!$C$6:$C$29,U46)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U46)&gt;1,"  ("&amp;(T46-INDEX('1 Matériel'!$G$6:$G$29,U46)+INDEX('1 Matériel'!$F$6:$F$29,U46))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U46)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U46)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U46),"")))</f>
+        <f>IF(T46="","",IF(V46=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U46)),INDEX('1 Matériel'!$C$6:$C$29,U46)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U46)&gt;1,"  ("&amp;(T46-INDEX('1 Matériel'!$F$6:$F$29,U46)+INDEX('1 Matériel'!$E$6:$E$29,U46))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U46)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E46" s="29" t="n"/>
@@ -3002,11 +2969,11 @@
       <c r="Q46" s="31" t="n"/>
       <c r="R46" s="30" t="n"/>
       <c r="T46" s="32">
-        <f>IF(32&lt;=SUM('1 Matériel'!$F$6:$F$29),32,"")</f>
+        <f>IF(32&lt;=SUM('1 Matériel'!$E$6:$E$29),32,"")</f>
         <v/>
       </c>
       <c r="U46" s="32">
-        <f>IF(T46="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T46)+1)</f>
+        <f>IF(T46="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T46)+1)</f>
         <v/>
       </c>
       <c r="V46" s="32">
@@ -3022,7 +2989,7 @@
       <c r="B47" s="27" t="n"/>
       <c r="C47" s="27" t="n"/>
       <c r="D47" s="28">
-        <f>IF(T47="","",IF(V47=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U47)),INDEX('1 Matériel'!$C$6:$C$29,U47)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U47)&gt;1,"  ("&amp;(T47-INDEX('1 Matériel'!$G$6:$G$29,U47)+INDEX('1 Matériel'!$F$6:$F$29,U47))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U47)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U47)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U47),"")))</f>
+        <f>IF(T47="","",IF(V47=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U47)),INDEX('1 Matériel'!$C$6:$C$29,U47)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U47)&gt;1,"  ("&amp;(T47-INDEX('1 Matériel'!$F$6:$F$29,U47)+INDEX('1 Matériel'!$E$6:$E$29,U47))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U47)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E47" s="29" t="n"/>
@@ -3040,11 +3007,11 @@
       <c r="Q47" s="31" t="n"/>
       <c r="R47" s="30" t="n"/>
       <c r="T47" s="32">
-        <f>IF(33&lt;=SUM('1 Matériel'!$F$6:$F$29),33,"")</f>
+        <f>IF(33&lt;=SUM('1 Matériel'!$E$6:$E$29),33,"")</f>
         <v/>
       </c>
       <c r="U47" s="32">
-        <f>IF(T47="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T47)+1)</f>
+        <f>IF(T47="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T47)+1)</f>
         <v/>
       </c>
       <c r="V47" s="32">
@@ -3060,7 +3027,7 @@
       <c r="B48" s="27" t="n"/>
       <c r="C48" s="27" t="n"/>
       <c r="D48" s="28">
-        <f>IF(T48="","",IF(V48=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U48)),INDEX('1 Matériel'!$C$6:$C$29,U48)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U48)&gt;1,"  ("&amp;(T48-INDEX('1 Matériel'!$G$6:$G$29,U48)+INDEX('1 Matériel'!$F$6:$F$29,U48))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U48)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U48)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U48),"")))</f>
+        <f>IF(T48="","",IF(V48=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U48)),INDEX('1 Matériel'!$C$6:$C$29,U48)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U48)&gt;1,"  ("&amp;(T48-INDEX('1 Matériel'!$F$6:$F$29,U48)+INDEX('1 Matériel'!$E$6:$E$29,U48))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U48)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E48" s="29" t="n"/>
@@ -3078,11 +3045,11 @@
       <c r="Q48" s="31" t="n"/>
       <c r="R48" s="30" t="n"/>
       <c r="T48" s="32">
-        <f>IF(34&lt;=SUM('1 Matériel'!$F$6:$F$29),34,"")</f>
+        <f>IF(34&lt;=SUM('1 Matériel'!$E$6:$E$29),34,"")</f>
         <v/>
       </c>
       <c r="U48" s="32">
-        <f>IF(T48="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T48)+1)</f>
+        <f>IF(T48="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T48)+1)</f>
         <v/>
       </c>
       <c r="V48" s="32">
@@ -3098,7 +3065,7 @@
       <c r="B49" s="27" t="n"/>
       <c r="C49" s="27" t="n"/>
       <c r="D49" s="28">
-        <f>IF(T49="","",IF(V49=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U49)),INDEX('1 Matériel'!$C$6:$C$29,U49)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U49)&gt;1,"  ("&amp;(T49-INDEX('1 Matériel'!$G$6:$G$29,U49)+INDEX('1 Matériel'!$F$6:$F$29,U49))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U49)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U49)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U49),"")))</f>
+        <f>IF(T49="","",IF(V49=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U49)),INDEX('1 Matériel'!$C$6:$C$29,U49)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U49)&gt;1,"  ("&amp;(T49-INDEX('1 Matériel'!$F$6:$F$29,U49)+INDEX('1 Matériel'!$E$6:$E$29,U49))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U49)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E49" s="29" t="n"/>
@@ -3116,11 +3083,11 @@
       <c r="Q49" s="31" t="n"/>
       <c r="R49" s="30" t="n"/>
       <c r="T49" s="32">
-        <f>IF(35&lt;=SUM('1 Matériel'!$F$6:$F$29),35,"")</f>
+        <f>IF(35&lt;=SUM('1 Matériel'!$E$6:$E$29),35,"")</f>
         <v/>
       </c>
       <c r="U49" s="32">
-        <f>IF(T49="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T49)+1)</f>
+        <f>IF(T49="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T49)+1)</f>
         <v/>
       </c>
       <c r="V49" s="32">
@@ -3136,7 +3103,7 @@
       <c r="B50" s="27" t="n"/>
       <c r="C50" s="27" t="n"/>
       <c r="D50" s="28">
-        <f>IF(T50="","",IF(V50=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U50)),INDEX('1 Matériel'!$C$6:$C$29,U50)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U50)&gt;1,"  ("&amp;(T50-INDEX('1 Matériel'!$G$6:$G$29,U50)+INDEX('1 Matériel'!$F$6:$F$29,U50))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U50)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U50)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U50),"")))</f>
+        <f>IF(T50="","",IF(V50=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U50)),INDEX('1 Matériel'!$C$6:$C$29,U50)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U50)&gt;1,"  ("&amp;(T50-INDEX('1 Matériel'!$F$6:$F$29,U50)+INDEX('1 Matériel'!$E$6:$E$29,U50))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U50)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E50" s="29" t="n"/>
@@ -3154,11 +3121,11 @@
       <c r="Q50" s="31" t="n"/>
       <c r="R50" s="30" t="n"/>
       <c r="T50" s="32">
-        <f>IF(36&lt;=SUM('1 Matériel'!$F$6:$F$29),36,"")</f>
+        <f>IF(36&lt;=SUM('1 Matériel'!$E$6:$E$29),36,"")</f>
         <v/>
       </c>
       <c r="U50" s="32">
-        <f>IF(T50="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T50)+1)</f>
+        <f>IF(T50="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T50)+1)</f>
         <v/>
       </c>
       <c r="V50" s="32">
@@ -3174,7 +3141,7 @@
       <c r="B51" s="27" t="n"/>
       <c r="C51" s="27" t="n"/>
       <c r="D51" s="28">
-        <f>IF(T51="","",IF(V51=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U51)),INDEX('1 Matériel'!$C$6:$C$29,U51)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U51)&gt;1,"  ("&amp;(T51-INDEX('1 Matériel'!$G$6:$G$29,U51)+INDEX('1 Matériel'!$F$6:$F$29,U51))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U51)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U51)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U51),"")))</f>
+        <f>IF(T51="","",IF(V51=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U51)),INDEX('1 Matériel'!$C$6:$C$29,U51)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U51)&gt;1,"  ("&amp;(T51-INDEX('1 Matériel'!$F$6:$F$29,U51)+INDEX('1 Matériel'!$E$6:$E$29,U51))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U51)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E51" s="29" t="n"/>
@@ -3192,11 +3159,11 @@
       <c r="Q51" s="31" t="n"/>
       <c r="R51" s="30" t="n"/>
       <c r="T51" s="32">
-        <f>IF(37&lt;=SUM('1 Matériel'!$F$6:$F$29),37,"")</f>
+        <f>IF(37&lt;=SUM('1 Matériel'!$E$6:$E$29),37,"")</f>
         <v/>
       </c>
       <c r="U51" s="32">
-        <f>IF(T51="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T51)+1)</f>
+        <f>IF(T51="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T51)+1)</f>
         <v/>
       </c>
       <c r="V51" s="32">
@@ -3212,7 +3179,7 @@
       <c r="B52" s="27" t="n"/>
       <c r="C52" s="27" t="n"/>
       <c r="D52" s="28">
-        <f>IF(T52="","",IF(V52=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U52)),INDEX('1 Matériel'!$C$6:$C$29,U52)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U52)&gt;1,"  ("&amp;(T52-INDEX('1 Matériel'!$G$6:$G$29,U52)+INDEX('1 Matériel'!$F$6:$F$29,U52))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U52)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U52)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U52),"")))</f>
+        <f>IF(T52="","",IF(V52=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U52)),INDEX('1 Matériel'!$C$6:$C$29,U52)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U52)&gt;1,"  ("&amp;(T52-INDEX('1 Matériel'!$F$6:$F$29,U52)+INDEX('1 Matériel'!$E$6:$E$29,U52))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U52)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E52" s="29" t="n"/>
@@ -3230,11 +3197,11 @@
       <c r="Q52" s="31" t="n"/>
       <c r="R52" s="30" t="n"/>
       <c r="T52" s="32">
-        <f>IF(38&lt;=SUM('1 Matériel'!$F$6:$F$29),38,"")</f>
+        <f>IF(38&lt;=SUM('1 Matériel'!$E$6:$E$29),38,"")</f>
         <v/>
       </c>
       <c r="U52" s="32">
-        <f>IF(T52="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T52)+1)</f>
+        <f>IF(T52="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T52)+1)</f>
         <v/>
       </c>
       <c r="V52" s="32">
@@ -3250,7 +3217,7 @@
       <c r="B53" s="27" t="n"/>
       <c r="C53" s="27" t="n"/>
       <c r="D53" s="28">
-        <f>IF(T53="","",IF(V53=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U53)),INDEX('1 Matériel'!$C$6:$C$29,U53)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U53)&gt;1,"  ("&amp;(T53-INDEX('1 Matériel'!$G$6:$G$29,U53)+INDEX('1 Matériel'!$F$6:$F$29,U53))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U53)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U53)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U53),"")))</f>
+        <f>IF(T53="","",IF(V53=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U53)),INDEX('1 Matériel'!$C$6:$C$29,U53)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U53)&gt;1,"  ("&amp;(T53-INDEX('1 Matériel'!$F$6:$F$29,U53)+INDEX('1 Matériel'!$E$6:$E$29,U53))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U53)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E53" s="29" t="n"/>
@@ -3268,11 +3235,11 @@
       <c r="Q53" s="31" t="n"/>
       <c r="R53" s="30" t="n"/>
       <c r="T53" s="32">
-        <f>IF(39&lt;=SUM('1 Matériel'!$F$6:$F$29),39,"")</f>
+        <f>IF(39&lt;=SUM('1 Matériel'!$E$6:$E$29),39,"")</f>
         <v/>
       </c>
       <c r="U53" s="32">
-        <f>IF(T53="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T53)+1)</f>
+        <f>IF(T53="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T53)+1)</f>
         <v/>
       </c>
       <c r="V53" s="32">
@@ -3288,7 +3255,7 @@
       <c r="B54" s="27" t="n"/>
       <c r="C54" s="27" t="n"/>
       <c r="D54" s="28">
-        <f>IF(T54="","",IF(V54=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U54)),INDEX('1 Matériel'!$C$6:$C$29,U54)&amp;IF(INDEX('1 Matériel'!$F$6:$F$29,U54)&gt;1,"  ("&amp;(T54-INDEX('1 Matériel'!$G$6:$G$29,U54)+INDEX('1 Matériel'!$F$6:$F$29,U54))&amp;"/"&amp;INDEX('1 Matériel'!$F$6:$F$29,U54)&amp;")","")&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U54)&lt;&gt;"",CHAR(10)&amp;"→ "&amp;INDEX('1 Matériel'!$E$6:$E$29,U54),"")))</f>
+        <f>IF(T54="","",IF(V54=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U54)),INDEX('1 Matériel'!$C$6:$C$29,U54)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U54)&gt;1,"  ("&amp;(T54-INDEX('1 Matériel'!$F$6:$F$29,U54)+INDEX('1 Matériel'!$E$6:$E$29,U54))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U54)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E54" s="29" t="n"/>
@@ -3306,11 +3273,11 @@
       <c r="Q54" s="31" t="n"/>
       <c r="R54" s="30" t="n"/>
       <c r="T54" s="32">
-        <f>IF(40&lt;=SUM('1 Matériel'!$F$6:$F$29),40,"")</f>
+        <f>IF(40&lt;=SUM('1 Matériel'!$E$6:$E$29),40,"")</f>
         <v/>
       </c>
       <c r="U54" s="32">
-        <f>IF(T54="","",COUNTIF('1 Matériel'!$G$6:$G$29,"&lt;"&amp;T54)+1)</f>
+        <f>IF(T54="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T54)+1)</f>
         <v/>
       </c>
       <c r="V54" s="32">
@@ -3320,7 +3287,7 @@
     </row>
     <row r="55">
       <c r="A55" s="33">
-        <f>IF(SUM('1 Matériel'!$F$6:$F$29)&gt;20,"⚠  "&amp;(SUM('1 Matériel'!$F$6:$F$29)-20)&amp;" ligne(s) au-delà de la ligne 20 sont masquées : cliquer sur le [+] dans la marge gauche pour les afficher.","")</f>
+        <f>IF(SUM('1 Matériel'!$E$6:$E$29)&gt;20,"⚠  "&amp;(SUM('1 Matériel'!$E$6:$E$29)-20)&amp;" ligne(s) au-delà de la ligne 20 sont masquées : cliquer sur le [+] dans la marge gauche pour les afficher.","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Tool list : préparée par / validée par, colisage sous les items, nombre de serrages, sans avancement ni contrôle
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Tool_List_Enedril_2027.xlsx
+++ b/devis_2027/Tool_List_Enedril_2027.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'2 Tool List'!$A$1:$R$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Tool List'!$A$14:$V$54</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'2 Tool List'!$A$1:$L$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,16 +21,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0;-0;;@"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="dd/mm"/>
-    <numFmt numFmtId="168" formatCode="#,##0.0"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0 &quot;kg&quot;"/>
-    <numFmt numFmtId="170" formatCode="0.000 &quot;m³&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="#,##0.0 &quot;kg&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.000 &quot;m³&quot;"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -162,12 +162,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00E2231A"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="0008203F"/>
       <sz val="10"/>
     </font>
@@ -181,12 +175,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0051647A"/>
-      <sz val="8"/>
     </font>
   </fonts>
   <fills count="8">
@@ -233,7 +221,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -252,58 +240,19 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00D5DEE8"/>
-      </left>
-      <top style="thin">
-        <color rgb="00D5DEE8"/>
-      </top>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="00D5DEE8"/>
-      </top>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="00D5DEE8"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D5DEE8"/>
-      </top>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D5DEE8"/>
-      </left>
-    </border>
-    <border/>
-    <border>
-      <right style="thin">
-        <color rgb="00D5DEE8"/>
-      </right>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D5DEE8"/>
-      </left>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
-        <color rgb="00D5DEE8"/>
+        <color rgb="0000AEEF"/>
       </bottom>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="00D5DEE8"/>
-      </right>
-      <bottom style="thin">
-        <color rgb="00D5DEE8"/>
-      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -381,15 +330,9 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -402,7 +345,7 @@
     <xf numFmtId="1" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -411,34 +354,27 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" indent="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -447,7 +383,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -486,14 +422,6 @@
           <color rgb="00B7DDF2"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00DDF3E4"/>
-          <bgColor rgb="00DDF3E4"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1407,31 +1335,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V75"/>
+  <dimension ref="A1:V72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.5" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="1.5" customWidth="1" min="19" max="19"/>
-    <col width="6" customWidth="1" min="20" max="20"/>
-    <col width="6" customWidth="1" min="21" max="21"/>
-    <col width="6" customWidth="1" min="22" max="22"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1470,12 +1388,6 @@
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n"/>
-      <c r="M3" s="4" t="n"/>
-      <c r="N3" s="4" t="n"/>
-      <c r="O3" s="4" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="4" t="n"/>
-      <c r="R3" s="4" t="n"/>
     </row>
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="15" customHeight="1">
@@ -1494,7 +1406,7 @@
           <t>DOSSIER N° · RIG</t>
         </is>
       </c>
-      <c r="L5" s="17" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>DESTINATION</t>
         </is>
@@ -1510,15 +1422,9 @@
       <c r="G6" s="18" t="n"/>
       <c r="H6" s="19" t="n"/>
       <c r="I6" s="19" t="n"/>
-      <c r="J6" s="19" t="n"/>
+      <c r="J6" s="18" t="n"/>
       <c r="K6" s="19" t="n"/>
-      <c r="L6" s="18" t="n"/>
-      <c r="M6" s="19" t="n"/>
-      <c r="N6" s="19" t="n"/>
-      <c r="O6" s="19" t="n"/>
-      <c r="P6" s="19" t="n"/>
-      <c r="Q6" s="19" t="n"/>
-      <c r="R6" s="19" t="n"/>
+      <c r="L6" s="19" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
@@ -1536,9 +1442,9 @@
           <t>N° DE LISTE</t>
         </is>
       </c>
-      <c r="L7" s="17" t="inlineStr">
-        <is>
-          <t>FAITE PAR</t>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>PRÉPARÉE PAR</t>
         </is>
       </c>
     </row>
@@ -1552,15 +1458,9 @@
       <c r="G8" s="18" t="n"/>
       <c r="H8" s="19" t="n"/>
       <c r="I8" s="19" t="n"/>
-      <c r="J8" s="19" t="n"/>
+      <c r="J8" s="18" t="n"/>
       <c r="K8" s="19" t="n"/>
-      <c r="L8" s="18" t="n"/>
-      <c r="M8" s="19" t="n"/>
-      <c r="N8" s="19" t="n"/>
-      <c r="O8" s="19" t="n"/>
-      <c r="P8" s="19" t="n"/>
-      <c r="Q8" s="19" t="n"/>
-      <c r="R8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
@@ -1568,14 +1468,14 @@
           <t>DESCRIPTION GÉNÉRALE</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>COLISAGE</t>
         </is>
       </c>
-      <c r="L9" s="17" t="inlineStr">
-        <is>
-          <t>RÉVISÉE LE · PAR</t>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>VALIDÉE PAR</t>
         </is>
       </c>
     </row>
@@ -1584,24 +1484,18 @@
       <c r="B10" s="19" t="n"/>
       <c r="C10" s="19" t="n"/>
       <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>A communiquer dès que possible</t>
+        </is>
+      </c>
       <c r="F10" s="19" t="n"/>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>A communiquer dès que possible</t>
-        </is>
-      </c>
+      <c r="G10" s="19" t="n"/>
       <c r="H10" s="19" t="n"/>
       <c r="I10" s="19" t="n"/>
-      <c r="J10" s="19" t="n"/>
+      <c r="J10" s="18" t="n"/>
       <c r="K10" s="19" t="n"/>
-      <c r="L10" s="18" t="n"/>
-      <c r="M10" s="19" t="n"/>
-      <c r="N10" s="19" t="n"/>
-      <c r="O10" s="19" t="n"/>
-      <c r="P10" s="19" t="n"/>
-      <c r="Q10" s="19" t="n"/>
-      <c r="R10" s="19" t="n"/>
+      <c r="L10" s="19" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
@@ -1610,7 +1504,12 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="4" customHeight="1"/>
+    <row r="12" ht="14" customHeight="1">
+      <c r="A12" s="21">
+        <f>IF(SUBTOTAL(103,A15:A54)&lt;MIN(SUM('1 Matériel'!$E$6:$E$29),40),"⚠  Appuyer sur Ctrl + Alt + L pour afficher toutes les lignes de la liste.","")</f>
+        <v/>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
@@ -1637,19 +1536,9 @@
       <c r="K13" s="1" t="n"/>
       <c r="L13" s="23" t="inlineStr">
         <is>
-          <t>AVANCEMENT PRÉPARATION</t>
-        </is>
-      </c>
-      <c r="M13" s="24" t="n"/>
-      <c r="N13" s="24" t="n"/>
-      <c r="O13" s="24" t="n"/>
-      <c r="P13" s="22" t="inlineStr">
-        <is>
-          <t>CONTRÔLE SUPERVISEUR</t>
-        </is>
-      </c>
-      <c r="Q13" s="1" t="n"/>
-      <c r="R13" s="1" t="n"/>
+          <t>COLIS</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="25" t="inlineStr">
@@ -1714,39 +1603,7 @@
       </c>
       <c r="L14" s="25" t="inlineStr">
         <is>
-          <t>Prêt à
-partir</t>
-        </is>
-      </c>
-      <c r="M14" s="25" t="inlineStr">
-        <is>
-          <t>Le</t>
-        </is>
-      </c>
-      <c r="N14" s="25" t="inlineStr">
-        <is>
-          <t>Par</t>
-        </is>
-      </c>
-      <c r="O14" s="25" t="inlineStr">
-        <is>
-          <t>Colisage
-(n° colis)</t>
-        </is>
-      </c>
-      <c r="P14" s="25" t="inlineStr">
-        <is>
-          <t>Contrôle</t>
-        </is>
-      </c>
-      <c r="Q14" s="25" t="inlineStr">
-        <is>
-          <t>Le</t>
-        </is>
-      </c>
-      <c r="R14" s="25" t="inlineStr">
-        <is>
-          <t>Par</t>
+          <t>N° colis</t>
         </is>
       </c>
       <c r="T14" s="26" t="inlineStr">
@@ -1767,13 +1624,13 @@
     </row>
     <row r="15" ht="27" customHeight="1">
       <c r="A15" s="7">
-        <f>IF(OR(T15="",V15=1),"",T15-COUNTIF(V$15:V15,1))</f>
+        <f>IF(OR(T15=0,V15=1),"",T15-COUNTIF(V$15:V15,1))</f>
         <v/>
       </c>
       <c r="B15" s="27" t="n"/>
       <c r="C15" s="27" t="n"/>
       <c r="D15" s="28">
-        <f>IF(T15="","",IF(V15=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U15)),INDEX('1 Matériel'!$C$6:$C$29,U15)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U15)&gt;1,"  ("&amp;(T15-INDEX('1 Matériel'!$F$6:$F$29,U15)+INDEX('1 Matériel'!$E$6:$E$29,U15))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U15)&amp;")","")))</f>
+        <f>IF(T15=0,"",IF(V15=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U15)),INDEX('1 Matériel'!$C$6:$C$29,U15)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U15)&gt;1,"  ("&amp;(T15-INDEX('1 Matériel'!$F$6:$F$29,U15)+INDEX('1 Matériel'!$E$6:$E$29,U15))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U15)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E15" s="29" t="n"/>
@@ -1784,34 +1641,28 @@
       <c r="J15" s="30" t="n"/>
       <c r="K15" s="27" t="n"/>
       <c r="L15" s="30" t="n"/>
-      <c r="M15" s="31" t="n"/>
-      <c r="N15" s="30" t="n"/>
-      <c r="O15" s="30" t="n"/>
-      <c r="P15" s="30" t="n"/>
-      <c r="Q15" s="31" t="n"/>
-      <c r="R15" s="30" t="n"/>
-      <c r="T15" s="32">
-        <f>IF(1&lt;=SUM('1 Matériel'!$E$6:$E$29),1,"")</f>
-        <v/>
-      </c>
-      <c r="U15" s="32">
-        <f>IF(T15="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T15)+1)</f>
-        <v/>
-      </c>
-      <c r="V15" s="32">
+      <c r="T15" s="31">
+        <f>IF(1&lt;=SUM('1 Matériel'!$E$6:$E$29),1,0)</f>
+        <v/>
+      </c>
+      <c r="U15" s="31">
+        <f>IF(T15=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T15)+1)</f>
+        <v/>
+      </c>
+      <c r="V15" s="31">
         <f>IF(U15="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U15)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="27" customHeight="1">
       <c r="A16" s="7">
-        <f>IF(OR(T16="",V16=1),"",T16-COUNTIF(V$15:V16,1))</f>
+        <f>IF(OR(T16=0,V16=1),"",T16-COUNTIF(V$15:V16,1))</f>
         <v/>
       </c>
       <c r="B16" s="27" t="n"/>
       <c r="C16" s="27" t="n"/>
       <c r="D16" s="28">
-        <f>IF(T16="","",IF(V16=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U16)),INDEX('1 Matériel'!$C$6:$C$29,U16)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U16)&gt;1,"  ("&amp;(T16-INDEX('1 Matériel'!$F$6:$F$29,U16)+INDEX('1 Matériel'!$E$6:$E$29,U16))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U16)&amp;")","")))</f>
+        <f>IF(T16=0,"",IF(V16=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U16)),INDEX('1 Matériel'!$C$6:$C$29,U16)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U16)&gt;1,"  ("&amp;(T16-INDEX('1 Matériel'!$F$6:$F$29,U16)+INDEX('1 Matériel'!$E$6:$E$29,U16))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U16)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E16" s="29" t="n"/>
@@ -1822,34 +1673,28 @@
       <c r="J16" s="30" t="n"/>
       <c r="K16" s="27" t="n"/>
       <c r="L16" s="30" t="n"/>
-      <c r="M16" s="31" t="n"/>
-      <c r="N16" s="30" t="n"/>
-      <c r="O16" s="30" t="n"/>
-      <c r="P16" s="30" t="n"/>
-      <c r="Q16" s="31" t="n"/>
-      <c r="R16" s="30" t="n"/>
-      <c r="T16" s="32">
-        <f>IF(2&lt;=SUM('1 Matériel'!$E$6:$E$29),2,"")</f>
-        <v/>
-      </c>
-      <c r="U16" s="32">
-        <f>IF(T16="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T16)+1)</f>
-        <v/>
-      </c>
-      <c r="V16" s="32">
+      <c r="T16" s="31">
+        <f>IF(2&lt;=SUM('1 Matériel'!$E$6:$E$29),2,0)</f>
+        <v/>
+      </c>
+      <c r="U16" s="31">
+        <f>IF(T16=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T16)+1)</f>
+        <v/>
+      </c>
+      <c r="V16" s="31">
         <f>IF(U16="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U16)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="27" customHeight="1">
       <c r="A17" s="7">
-        <f>IF(OR(T17="",V17=1),"",T17-COUNTIF(V$15:V17,1))</f>
+        <f>IF(OR(T17=0,V17=1),"",T17-COUNTIF(V$15:V17,1))</f>
         <v/>
       </c>
       <c r="B17" s="27" t="n"/>
       <c r="C17" s="27" t="n"/>
       <c r="D17" s="28">
-        <f>IF(T17="","",IF(V17=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U17)),INDEX('1 Matériel'!$C$6:$C$29,U17)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U17)&gt;1,"  ("&amp;(T17-INDEX('1 Matériel'!$F$6:$F$29,U17)+INDEX('1 Matériel'!$E$6:$E$29,U17))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U17)&amp;")","")))</f>
+        <f>IF(T17=0,"",IF(V17=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U17)),INDEX('1 Matériel'!$C$6:$C$29,U17)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U17)&gt;1,"  ("&amp;(T17-INDEX('1 Matériel'!$F$6:$F$29,U17)+INDEX('1 Matériel'!$E$6:$E$29,U17))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U17)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E17" s="29" t="n"/>
@@ -1860,34 +1705,28 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="27" t="n"/>
       <c r="L17" s="30" t="n"/>
-      <c r="M17" s="31" t="n"/>
-      <c r="N17" s="30" t="n"/>
-      <c r="O17" s="30" t="n"/>
-      <c r="P17" s="30" t="n"/>
-      <c r="Q17" s="31" t="n"/>
-      <c r="R17" s="30" t="n"/>
-      <c r="T17" s="32">
-        <f>IF(3&lt;=SUM('1 Matériel'!$E$6:$E$29),3,"")</f>
-        <v/>
-      </c>
-      <c r="U17" s="32">
-        <f>IF(T17="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T17)+1)</f>
-        <v/>
-      </c>
-      <c r="V17" s="32">
+      <c r="T17" s="31">
+        <f>IF(3&lt;=SUM('1 Matériel'!$E$6:$E$29),3,0)</f>
+        <v/>
+      </c>
+      <c r="U17" s="31">
+        <f>IF(T17=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T17)+1)</f>
+        <v/>
+      </c>
+      <c r="V17" s="31">
         <f>IF(U17="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U17)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="27" customHeight="1">
       <c r="A18" s="7">
-        <f>IF(OR(T18="",V18=1),"",T18-COUNTIF(V$15:V18,1))</f>
+        <f>IF(OR(T18=0,V18=1),"",T18-COUNTIF(V$15:V18,1))</f>
         <v/>
       </c>
       <c r="B18" s="27" t="n"/>
       <c r="C18" s="27" t="n"/>
       <c r="D18" s="28">
-        <f>IF(T18="","",IF(V18=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U18)),INDEX('1 Matériel'!$C$6:$C$29,U18)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U18)&gt;1,"  ("&amp;(T18-INDEX('1 Matériel'!$F$6:$F$29,U18)+INDEX('1 Matériel'!$E$6:$E$29,U18))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U18)&amp;")","")))</f>
+        <f>IF(T18=0,"",IF(V18=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U18)),INDEX('1 Matériel'!$C$6:$C$29,U18)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U18)&gt;1,"  ("&amp;(T18-INDEX('1 Matériel'!$F$6:$F$29,U18)+INDEX('1 Matériel'!$E$6:$E$29,U18))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U18)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E18" s="29" t="n"/>
@@ -1898,34 +1737,28 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="27" t="n"/>
       <c r="L18" s="30" t="n"/>
-      <c r="M18" s="31" t="n"/>
-      <c r="N18" s="30" t="n"/>
-      <c r="O18" s="30" t="n"/>
-      <c r="P18" s="30" t="n"/>
-      <c r="Q18" s="31" t="n"/>
-      <c r="R18" s="30" t="n"/>
-      <c r="T18" s="32">
-        <f>IF(4&lt;=SUM('1 Matériel'!$E$6:$E$29),4,"")</f>
-        <v/>
-      </c>
-      <c r="U18" s="32">
-        <f>IF(T18="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T18)+1)</f>
-        <v/>
-      </c>
-      <c r="V18" s="32">
+      <c r="T18" s="31">
+        <f>IF(4&lt;=SUM('1 Matériel'!$E$6:$E$29),4,0)</f>
+        <v/>
+      </c>
+      <c r="U18" s="31">
+        <f>IF(T18=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T18)+1)</f>
+        <v/>
+      </c>
+      <c r="V18" s="31">
         <f>IF(U18="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U18)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="27" customHeight="1">
       <c r="A19" s="7">
-        <f>IF(OR(T19="",V19=1),"",T19-COUNTIF(V$15:V19,1))</f>
+        <f>IF(OR(T19=0,V19=1),"",T19-COUNTIF(V$15:V19,1))</f>
         <v/>
       </c>
       <c r="B19" s="27" t="n"/>
       <c r="C19" s="27" t="n"/>
       <c r="D19" s="28">
-        <f>IF(T19="","",IF(V19=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U19)),INDEX('1 Matériel'!$C$6:$C$29,U19)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U19)&gt;1,"  ("&amp;(T19-INDEX('1 Matériel'!$F$6:$F$29,U19)+INDEX('1 Matériel'!$E$6:$E$29,U19))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U19)&amp;")","")))</f>
+        <f>IF(T19=0,"",IF(V19=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U19)),INDEX('1 Matériel'!$C$6:$C$29,U19)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U19)&gt;1,"  ("&amp;(T19-INDEX('1 Matériel'!$F$6:$F$29,U19)+INDEX('1 Matériel'!$E$6:$E$29,U19))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U19)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E19" s="29" t="n"/>
@@ -1936,34 +1769,28 @@
       <c r="J19" s="30" t="n"/>
       <c r="K19" s="27" t="n"/>
       <c r="L19" s="30" t="n"/>
-      <c r="M19" s="31" t="n"/>
-      <c r="N19" s="30" t="n"/>
-      <c r="O19" s="30" t="n"/>
-      <c r="P19" s="30" t="n"/>
-      <c r="Q19" s="31" t="n"/>
-      <c r="R19" s="30" t="n"/>
-      <c r="T19" s="32">
-        <f>IF(5&lt;=SUM('1 Matériel'!$E$6:$E$29),5,"")</f>
-        <v/>
-      </c>
-      <c r="U19" s="32">
-        <f>IF(T19="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T19)+1)</f>
-        <v/>
-      </c>
-      <c r="V19" s="32">
+      <c r="T19" s="31">
+        <f>IF(5&lt;=SUM('1 Matériel'!$E$6:$E$29),5,0)</f>
+        <v/>
+      </c>
+      <c r="U19" s="31">
+        <f>IF(T19=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T19)+1)</f>
+        <v/>
+      </c>
+      <c r="V19" s="31">
         <f>IF(U19="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U19)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="27" customHeight="1">
+    <row r="20" hidden="1" ht="27" customHeight="1">
       <c r="A20" s="7">
-        <f>IF(OR(T20="",V20=1),"",T20-COUNTIF(V$15:V20,1))</f>
+        <f>IF(OR(T20=0,V20=1),"",T20-COUNTIF(V$15:V20,1))</f>
         <v/>
       </c>
       <c r="B20" s="27" t="n"/>
       <c r="C20" s="27" t="n"/>
       <c r="D20" s="28">
-        <f>IF(T20="","",IF(V20=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U20)),INDEX('1 Matériel'!$C$6:$C$29,U20)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U20)&gt;1,"  ("&amp;(T20-INDEX('1 Matériel'!$F$6:$F$29,U20)+INDEX('1 Matériel'!$E$6:$E$29,U20))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U20)&amp;")","")))</f>
+        <f>IF(T20=0,"",IF(V20=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U20)),INDEX('1 Matériel'!$C$6:$C$29,U20)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U20)&gt;1,"  ("&amp;(T20-INDEX('1 Matériel'!$F$6:$F$29,U20)+INDEX('1 Matériel'!$E$6:$E$29,U20))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U20)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E20" s="29" t="n"/>
@@ -1974,34 +1801,28 @@
       <c r="J20" s="30" t="n"/>
       <c r="K20" s="27" t="n"/>
       <c r="L20" s="30" t="n"/>
-      <c r="M20" s="31" t="n"/>
-      <c r="N20" s="30" t="n"/>
-      <c r="O20" s="30" t="n"/>
-      <c r="P20" s="30" t="n"/>
-      <c r="Q20" s="31" t="n"/>
-      <c r="R20" s="30" t="n"/>
-      <c r="T20" s="32">
-        <f>IF(6&lt;=SUM('1 Matériel'!$E$6:$E$29),6,"")</f>
-        <v/>
-      </c>
-      <c r="U20" s="32">
-        <f>IF(T20="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T20)+1)</f>
-        <v/>
-      </c>
-      <c r="V20" s="32">
+      <c r="T20" s="31">
+        <f>IF(6&lt;=SUM('1 Matériel'!$E$6:$E$29),6,0)</f>
+        <v/>
+      </c>
+      <c r="U20" s="31">
+        <f>IF(T20=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T20)+1)</f>
+        <v/>
+      </c>
+      <c r="V20" s="31">
         <f>IF(U20="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U20)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="27" customHeight="1">
+    <row r="21" hidden="1" ht="27" customHeight="1">
       <c r="A21" s="7">
-        <f>IF(OR(T21="",V21=1),"",T21-COUNTIF(V$15:V21,1))</f>
+        <f>IF(OR(T21=0,V21=1),"",T21-COUNTIF(V$15:V21,1))</f>
         <v/>
       </c>
       <c r="B21" s="27" t="n"/>
       <c r="C21" s="27" t="n"/>
       <c r="D21" s="28">
-        <f>IF(T21="","",IF(V21=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U21)),INDEX('1 Matériel'!$C$6:$C$29,U21)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U21)&gt;1,"  ("&amp;(T21-INDEX('1 Matériel'!$F$6:$F$29,U21)+INDEX('1 Matériel'!$E$6:$E$29,U21))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U21)&amp;")","")))</f>
+        <f>IF(T21=0,"",IF(V21=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U21)),INDEX('1 Matériel'!$C$6:$C$29,U21)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U21)&gt;1,"  ("&amp;(T21-INDEX('1 Matériel'!$F$6:$F$29,U21)+INDEX('1 Matériel'!$E$6:$E$29,U21))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U21)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E21" s="29" t="n"/>
@@ -2012,34 +1833,28 @@
       <c r="J21" s="30" t="n"/>
       <c r="K21" s="27" t="n"/>
       <c r="L21" s="30" t="n"/>
-      <c r="M21" s="31" t="n"/>
-      <c r="N21" s="30" t="n"/>
-      <c r="O21" s="30" t="n"/>
-      <c r="P21" s="30" t="n"/>
-      <c r="Q21" s="31" t="n"/>
-      <c r="R21" s="30" t="n"/>
-      <c r="T21" s="32">
-        <f>IF(7&lt;=SUM('1 Matériel'!$E$6:$E$29),7,"")</f>
-        <v/>
-      </c>
-      <c r="U21" s="32">
-        <f>IF(T21="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T21)+1)</f>
-        <v/>
-      </c>
-      <c r="V21" s="32">
+      <c r="T21" s="31">
+        <f>IF(7&lt;=SUM('1 Matériel'!$E$6:$E$29),7,0)</f>
+        <v/>
+      </c>
+      <c r="U21" s="31">
+        <f>IF(T21=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T21)+1)</f>
+        <v/>
+      </c>
+      <c r="V21" s="31">
         <f>IF(U21="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U21)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="27" customHeight="1">
+    <row r="22" hidden="1" ht="27" customHeight="1">
       <c r="A22" s="7">
-        <f>IF(OR(T22="",V22=1),"",T22-COUNTIF(V$15:V22,1))</f>
+        <f>IF(OR(T22=0,V22=1),"",T22-COUNTIF(V$15:V22,1))</f>
         <v/>
       </c>
       <c r="B22" s="27" t="n"/>
       <c r="C22" s="27" t="n"/>
       <c r="D22" s="28">
-        <f>IF(T22="","",IF(V22=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U22)),INDEX('1 Matériel'!$C$6:$C$29,U22)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U22)&gt;1,"  ("&amp;(T22-INDEX('1 Matériel'!$F$6:$F$29,U22)+INDEX('1 Matériel'!$E$6:$E$29,U22))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U22)&amp;")","")))</f>
+        <f>IF(T22=0,"",IF(V22=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U22)),INDEX('1 Matériel'!$C$6:$C$29,U22)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U22)&gt;1,"  ("&amp;(T22-INDEX('1 Matériel'!$F$6:$F$29,U22)+INDEX('1 Matériel'!$E$6:$E$29,U22))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U22)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E22" s="29" t="n"/>
@@ -2050,34 +1865,28 @@
       <c r="J22" s="30" t="n"/>
       <c r="K22" s="27" t="n"/>
       <c r="L22" s="30" t="n"/>
-      <c r="M22" s="31" t="n"/>
-      <c r="N22" s="30" t="n"/>
-      <c r="O22" s="30" t="n"/>
-      <c r="P22" s="30" t="n"/>
-      <c r="Q22" s="31" t="n"/>
-      <c r="R22" s="30" t="n"/>
-      <c r="T22" s="32">
-        <f>IF(8&lt;=SUM('1 Matériel'!$E$6:$E$29),8,"")</f>
-        <v/>
-      </c>
-      <c r="U22" s="32">
-        <f>IF(T22="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T22)+1)</f>
-        <v/>
-      </c>
-      <c r="V22" s="32">
+      <c r="T22" s="31">
+        <f>IF(8&lt;=SUM('1 Matériel'!$E$6:$E$29),8,0)</f>
+        <v/>
+      </c>
+      <c r="U22" s="31">
+        <f>IF(T22=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T22)+1)</f>
+        <v/>
+      </c>
+      <c r="V22" s="31">
         <f>IF(U22="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U22)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="27" customHeight="1">
+    <row r="23" hidden="1" ht="27" customHeight="1">
       <c r="A23" s="7">
-        <f>IF(OR(T23="",V23=1),"",T23-COUNTIF(V$15:V23,1))</f>
+        <f>IF(OR(T23=0,V23=1),"",T23-COUNTIF(V$15:V23,1))</f>
         <v/>
       </c>
       <c r="B23" s="27" t="n"/>
       <c r="C23" s="27" t="n"/>
       <c r="D23" s="28">
-        <f>IF(T23="","",IF(V23=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U23)),INDEX('1 Matériel'!$C$6:$C$29,U23)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U23)&gt;1,"  ("&amp;(T23-INDEX('1 Matériel'!$F$6:$F$29,U23)+INDEX('1 Matériel'!$E$6:$E$29,U23))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U23)&amp;")","")))</f>
+        <f>IF(T23=0,"",IF(V23=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U23)),INDEX('1 Matériel'!$C$6:$C$29,U23)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U23)&gt;1,"  ("&amp;(T23-INDEX('1 Matériel'!$F$6:$F$29,U23)+INDEX('1 Matériel'!$E$6:$E$29,U23))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U23)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E23" s="29" t="n"/>
@@ -2088,34 +1897,28 @@
       <c r="J23" s="30" t="n"/>
       <c r="K23" s="27" t="n"/>
       <c r="L23" s="30" t="n"/>
-      <c r="M23" s="31" t="n"/>
-      <c r="N23" s="30" t="n"/>
-      <c r="O23" s="30" t="n"/>
-      <c r="P23" s="30" t="n"/>
-      <c r="Q23" s="31" t="n"/>
-      <c r="R23" s="30" t="n"/>
-      <c r="T23" s="32">
-        <f>IF(9&lt;=SUM('1 Matériel'!$E$6:$E$29),9,"")</f>
-        <v/>
-      </c>
-      <c r="U23" s="32">
-        <f>IF(T23="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T23)+1)</f>
-        <v/>
-      </c>
-      <c r="V23" s="32">
+      <c r="T23" s="31">
+        <f>IF(9&lt;=SUM('1 Matériel'!$E$6:$E$29),9,0)</f>
+        <v/>
+      </c>
+      <c r="U23" s="31">
+        <f>IF(T23=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T23)+1)</f>
+        <v/>
+      </c>
+      <c r="V23" s="31">
         <f>IF(U23="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U23)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="27" customHeight="1">
+    <row r="24" hidden="1" ht="27" customHeight="1">
       <c r="A24" s="7">
-        <f>IF(OR(T24="",V24=1),"",T24-COUNTIF(V$15:V24,1))</f>
+        <f>IF(OR(T24=0,V24=1),"",T24-COUNTIF(V$15:V24,1))</f>
         <v/>
       </c>
       <c r="B24" s="27" t="n"/>
       <c r="C24" s="27" t="n"/>
       <c r="D24" s="28">
-        <f>IF(T24="","",IF(V24=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U24)),INDEX('1 Matériel'!$C$6:$C$29,U24)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U24)&gt;1,"  ("&amp;(T24-INDEX('1 Matériel'!$F$6:$F$29,U24)+INDEX('1 Matériel'!$E$6:$E$29,U24))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U24)&amp;")","")))</f>
+        <f>IF(T24=0,"",IF(V24=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U24)),INDEX('1 Matériel'!$C$6:$C$29,U24)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U24)&gt;1,"  ("&amp;(T24-INDEX('1 Matériel'!$F$6:$F$29,U24)+INDEX('1 Matériel'!$E$6:$E$29,U24))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U24)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E24" s="29" t="n"/>
@@ -2126,34 +1929,28 @@
       <c r="J24" s="30" t="n"/>
       <c r="K24" s="27" t="n"/>
       <c r="L24" s="30" t="n"/>
-      <c r="M24" s="31" t="n"/>
-      <c r="N24" s="30" t="n"/>
-      <c r="O24" s="30" t="n"/>
-      <c r="P24" s="30" t="n"/>
-      <c r="Q24" s="31" t="n"/>
-      <c r="R24" s="30" t="n"/>
-      <c r="T24" s="32">
-        <f>IF(10&lt;=SUM('1 Matériel'!$E$6:$E$29),10,"")</f>
-        <v/>
-      </c>
-      <c r="U24" s="32">
-        <f>IF(T24="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T24)+1)</f>
-        <v/>
-      </c>
-      <c r="V24" s="32">
+      <c r="T24" s="31">
+        <f>IF(10&lt;=SUM('1 Matériel'!$E$6:$E$29),10,0)</f>
+        <v/>
+      </c>
+      <c r="U24" s="31">
+        <f>IF(T24=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T24)+1)</f>
+        <v/>
+      </c>
+      <c r="V24" s="31">
         <f>IF(U24="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U24)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="25" ht="27" customHeight="1">
+    <row r="25" hidden="1" ht="27" customHeight="1">
       <c r="A25" s="7">
-        <f>IF(OR(T25="",V25=1),"",T25-COUNTIF(V$15:V25,1))</f>
+        <f>IF(OR(T25=0,V25=1),"",T25-COUNTIF(V$15:V25,1))</f>
         <v/>
       </c>
       <c r="B25" s="27" t="n"/>
       <c r="C25" s="27" t="n"/>
       <c r="D25" s="28">
-        <f>IF(T25="","",IF(V25=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U25)),INDEX('1 Matériel'!$C$6:$C$29,U25)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U25)&gt;1,"  ("&amp;(T25-INDEX('1 Matériel'!$F$6:$F$29,U25)+INDEX('1 Matériel'!$E$6:$E$29,U25))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U25)&amp;")","")))</f>
+        <f>IF(T25=0,"",IF(V25=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U25)),INDEX('1 Matériel'!$C$6:$C$29,U25)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U25)&gt;1,"  ("&amp;(T25-INDEX('1 Matériel'!$F$6:$F$29,U25)+INDEX('1 Matériel'!$E$6:$E$29,U25))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U25)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E25" s="29" t="n"/>
@@ -2164,34 +1961,28 @@
       <c r="J25" s="30" t="n"/>
       <c r="K25" s="27" t="n"/>
       <c r="L25" s="30" t="n"/>
-      <c r="M25" s="31" t="n"/>
-      <c r="N25" s="30" t="n"/>
-      <c r="O25" s="30" t="n"/>
-      <c r="P25" s="30" t="n"/>
-      <c r="Q25" s="31" t="n"/>
-      <c r="R25" s="30" t="n"/>
-      <c r="T25" s="32">
-        <f>IF(11&lt;=SUM('1 Matériel'!$E$6:$E$29),11,"")</f>
-        <v/>
-      </c>
-      <c r="U25" s="32">
-        <f>IF(T25="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T25)+1)</f>
-        <v/>
-      </c>
-      <c r="V25" s="32">
+      <c r="T25" s="31">
+        <f>IF(11&lt;=SUM('1 Matériel'!$E$6:$E$29),11,0)</f>
+        <v/>
+      </c>
+      <c r="U25" s="31">
+        <f>IF(T25=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T25)+1)</f>
+        <v/>
+      </c>
+      <c r="V25" s="31">
         <f>IF(U25="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U25)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="26" ht="27" customHeight="1">
+    <row r="26" hidden="1" ht="27" customHeight="1">
       <c r="A26" s="7">
-        <f>IF(OR(T26="",V26=1),"",T26-COUNTIF(V$15:V26,1))</f>
+        <f>IF(OR(T26=0,V26=1),"",T26-COUNTIF(V$15:V26,1))</f>
         <v/>
       </c>
       <c r="B26" s="27" t="n"/>
       <c r="C26" s="27" t="n"/>
       <c r="D26" s="28">
-        <f>IF(T26="","",IF(V26=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U26)),INDEX('1 Matériel'!$C$6:$C$29,U26)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U26)&gt;1,"  ("&amp;(T26-INDEX('1 Matériel'!$F$6:$F$29,U26)+INDEX('1 Matériel'!$E$6:$E$29,U26))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U26)&amp;")","")))</f>
+        <f>IF(T26=0,"",IF(V26=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U26)),INDEX('1 Matériel'!$C$6:$C$29,U26)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U26)&gt;1,"  ("&amp;(T26-INDEX('1 Matériel'!$F$6:$F$29,U26)+INDEX('1 Matériel'!$E$6:$E$29,U26))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U26)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E26" s="29" t="n"/>
@@ -2202,34 +1993,28 @@
       <c r="J26" s="30" t="n"/>
       <c r="K26" s="27" t="n"/>
       <c r="L26" s="30" t="n"/>
-      <c r="M26" s="31" t="n"/>
-      <c r="N26" s="30" t="n"/>
-      <c r="O26" s="30" t="n"/>
-      <c r="P26" s="30" t="n"/>
-      <c r="Q26" s="31" t="n"/>
-      <c r="R26" s="30" t="n"/>
-      <c r="T26" s="32">
-        <f>IF(12&lt;=SUM('1 Matériel'!$E$6:$E$29),12,"")</f>
-        <v/>
-      </c>
-      <c r="U26" s="32">
-        <f>IF(T26="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T26)+1)</f>
-        <v/>
-      </c>
-      <c r="V26" s="32">
+      <c r="T26" s="31">
+        <f>IF(12&lt;=SUM('1 Matériel'!$E$6:$E$29),12,0)</f>
+        <v/>
+      </c>
+      <c r="U26" s="31">
+        <f>IF(T26=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T26)+1)</f>
+        <v/>
+      </c>
+      <c r="V26" s="31">
         <f>IF(U26="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U26)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="27" customHeight="1">
+    <row r="27" hidden="1" ht="27" customHeight="1">
       <c r="A27" s="7">
-        <f>IF(OR(T27="",V27=1),"",T27-COUNTIF(V$15:V27,1))</f>
+        <f>IF(OR(T27=0,V27=1),"",T27-COUNTIF(V$15:V27,1))</f>
         <v/>
       </c>
       <c r="B27" s="27" t="n"/>
       <c r="C27" s="27" t="n"/>
       <c r="D27" s="28">
-        <f>IF(T27="","",IF(V27=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U27)),INDEX('1 Matériel'!$C$6:$C$29,U27)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U27)&gt;1,"  ("&amp;(T27-INDEX('1 Matériel'!$F$6:$F$29,U27)+INDEX('1 Matériel'!$E$6:$E$29,U27))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U27)&amp;")","")))</f>
+        <f>IF(T27=0,"",IF(V27=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U27)),INDEX('1 Matériel'!$C$6:$C$29,U27)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U27)&gt;1,"  ("&amp;(T27-INDEX('1 Matériel'!$F$6:$F$29,U27)+INDEX('1 Matériel'!$E$6:$E$29,U27))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U27)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E27" s="29" t="n"/>
@@ -2240,34 +2025,28 @@
       <c r="J27" s="30" t="n"/>
       <c r="K27" s="27" t="n"/>
       <c r="L27" s="30" t="n"/>
-      <c r="M27" s="31" t="n"/>
-      <c r="N27" s="30" t="n"/>
-      <c r="O27" s="30" t="n"/>
-      <c r="P27" s="30" t="n"/>
-      <c r="Q27" s="31" t="n"/>
-      <c r="R27" s="30" t="n"/>
-      <c r="T27" s="32">
-        <f>IF(13&lt;=SUM('1 Matériel'!$E$6:$E$29),13,"")</f>
-        <v/>
-      </c>
-      <c r="U27" s="32">
-        <f>IF(T27="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T27)+1)</f>
-        <v/>
-      </c>
-      <c r="V27" s="32">
+      <c r="T27" s="31">
+        <f>IF(13&lt;=SUM('1 Matériel'!$E$6:$E$29),13,0)</f>
+        <v/>
+      </c>
+      <c r="U27" s="31">
+        <f>IF(T27=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T27)+1)</f>
+        <v/>
+      </c>
+      <c r="V27" s="31">
         <f>IF(U27="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U27)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="27" customHeight="1">
+    <row r="28" hidden="1" ht="27" customHeight="1">
       <c r="A28" s="7">
-        <f>IF(OR(T28="",V28=1),"",T28-COUNTIF(V$15:V28,1))</f>
+        <f>IF(OR(T28=0,V28=1),"",T28-COUNTIF(V$15:V28,1))</f>
         <v/>
       </c>
       <c r="B28" s="27" t="n"/>
       <c r="C28" s="27" t="n"/>
       <c r="D28" s="28">
-        <f>IF(T28="","",IF(V28=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U28)),INDEX('1 Matériel'!$C$6:$C$29,U28)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U28)&gt;1,"  ("&amp;(T28-INDEX('1 Matériel'!$F$6:$F$29,U28)+INDEX('1 Matériel'!$E$6:$E$29,U28))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U28)&amp;")","")))</f>
+        <f>IF(T28=0,"",IF(V28=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U28)),INDEX('1 Matériel'!$C$6:$C$29,U28)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U28)&gt;1,"  ("&amp;(T28-INDEX('1 Matériel'!$F$6:$F$29,U28)+INDEX('1 Matériel'!$E$6:$E$29,U28))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U28)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E28" s="29" t="n"/>
@@ -2278,34 +2057,28 @@
       <c r="J28" s="30" t="n"/>
       <c r="K28" s="27" t="n"/>
       <c r="L28" s="30" t="n"/>
-      <c r="M28" s="31" t="n"/>
-      <c r="N28" s="30" t="n"/>
-      <c r="O28" s="30" t="n"/>
-      <c r="P28" s="30" t="n"/>
-      <c r="Q28" s="31" t="n"/>
-      <c r="R28" s="30" t="n"/>
-      <c r="T28" s="32">
-        <f>IF(14&lt;=SUM('1 Matériel'!$E$6:$E$29),14,"")</f>
-        <v/>
-      </c>
-      <c r="U28" s="32">
-        <f>IF(T28="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T28)+1)</f>
-        <v/>
-      </c>
-      <c r="V28" s="32">
+      <c r="T28" s="31">
+        <f>IF(14&lt;=SUM('1 Matériel'!$E$6:$E$29),14,0)</f>
+        <v/>
+      </c>
+      <c r="U28" s="31">
+        <f>IF(T28=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T28)+1)</f>
+        <v/>
+      </c>
+      <c r="V28" s="31">
         <f>IF(U28="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U28)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="29" ht="27" customHeight="1">
+    <row r="29" hidden="1" ht="27" customHeight="1">
       <c r="A29" s="7">
-        <f>IF(OR(T29="",V29=1),"",T29-COUNTIF(V$15:V29,1))</f>
+        <f>IF(OR(T29=0,V29=1),"",T29-COUNTIF(V$15:V29,1))</f>
         <v/>
       </c>
       <c r="B29" s="27" t="n"/>
       <c r="C29" s="27" t="n"/>
       <c r="D29" s="28">
-        <f>IF(T29="","",IF(V29=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U29)),INDEX('1 Matériel'!$C$6:$C$29,U29)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U29)&gt;1,"  ("&amp;(T29-INDEX('1 Matériel'!$F$6:$F$29,U29)+INDEX('1 Matériel'!$E$6:$E$29,U29))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U29)&amp;")","")))</f>
+        <f>IF(T29=0,"",IF(V29=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U29)),INDEX('1 Matériel'!$C$6:$C$29,U29)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U29)&gt;1,"  ("&amp;(T29-INDEX('1 Matériel'!$F$6:$F$29,U29)+INDEX('1 Matériel'!$E$6:$E$29,U29))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U29)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E29" s="29" t="n"/>
@@ -2316,34 +2089,28 @@
       <c r="J29" s="30" t="n"/>
       <c r="K29" s="27" t="n"/>
       <c r="L29" s="30" t="n"/>
-      <c r="M29" s="31" t="n"/>
-      <c r="N29" s="30" t="n"/>
-      <c r="O29" s="30" t="n"/>
-      <c r="P29" s="30" t="n"/>
-      <c r="Q29" s="31" t="n"/>
-      <c r="R29" s="30" t="n"/>
-      <c r="T29" s="32">
-        <f>IF(15&lt;=SUM('1 Matériel'!$E$6:$E$29),15,"")</f>
-        <v/>
-      </c>
-      <c r="U29" s="32">
-        <f>IF(T29="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T29)+1)</f>
-        <v/>
-      </c>
-      <c r="V29" s="32">
+      <c r="T29" s="31">
+        <f>IF(15&lt;=SUM('1 Matériel'!$E$6:$E$29),15,0)</f>
+        <v/>
+      </c>
+      <c r="U29" s="31">
+        <f>IF(T29=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T29)+1)</f>
+        <v/>
+      </c>
+      <c r="V29" s="31">
         <f>IF(U29="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U29)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="30" ht="27" customHeight="1">
+    <row r="30" hidden="1" ht="27" customHeight="1">
       <c r="A30" s="7">
-        <f>IF(OR(T30="",V30=1),"",T30-COUNTIF(V$15:V30,1))</f>
+        <f>IF(OR(T30=0,V30=1),"",T30-COUNTIF(V$15:V30,1))</f>
         <v/>
       </c>
       <c r="B30" s="27" t="n"/>
       <c r="C30" s="27" t="n"/>
       <c r="D30" s="28">
-        <f>IF(T30="","",IF(V30=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U30)),INDEX('1 Matériel'!$C$6:$C$29,U30)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U30)&gt;1,"  ("&amp;(T30-INDEX('1 Matériel'!$F$6:$F$29,U30)+INDEX('1 Matériel'!$E$6:$E$29,U30))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U30)&amp;")","")))</f>
+        <f>IF(T30=0,"",IF(V30=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U30)),INDEX('1 Matériel'!$C$6:$C$29,U30)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U30)&gt;1,"  ("&amp;(T30-INDEX('1 Matériel'!$F$6:$F$29,U30)+INDEX('1 Matériel'!$E$6:$E$29,U30))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U30)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E30" s="29" t="n"/>
@@ -2354,34 +2121,28 @@
       <c r="J30" s="30" t="n"/>
       <c r="K30" s="27" t="n"/>
       <c r="L30" s="30" t="n"/>
-      <c r="M30" s="31" t="n"/>
-      <c r="N30" s="30" t="n"/>
-      <c r="O30" s="30" t="n"/>
-      <c r="P30" s="30" t="n"/>
-      <c r="Q30" s="31" t="n"/>
-      <c r="R30" s="30" t="n"/>
-      <c r="T30" s="32">
-        <f>IF(16&lt;=SUM('1 Matériel'!$E$6:$E$29),16,"")</f>
-        <v/>
-      </c>
-      <c r="U30" s="32">
-        <f>IF(T30="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T30)+1)</f>
-        <v/>
-      </c>
-      <c r="V30" s="32">
+      <c r="T30" s="31">
+        <f>IF(16&lt;=SUM('1 Matériel'!$E$6:$E$29),16,0)</f>
+        <v/>
+      </c>
+      <c r="U30" s="31">
+        <f>IF(T30=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T30)+1)</f>
+        <v/>
+      </c>
+      <c r="V30" s="31">
         <f>IF(U30="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U30)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="31" ht="27" customHeight="1">
+    <row r="31" hidden="1" ht="27" customHeight="1">
       <c r="A31" s="7">
-        <f>IF(OR(T31="",V31=1),"",T31-COUNTIF(V$15:V31,1))</f>
+        <f>IF(OR(T31=0,V31=1),"",T31-COUNTIF(V$15:V31,1))</f>
         <v/>
       </c>
       <c r="B31" s="27" t="n"/>
       <c r="C31" s="27" t="n"/>
       <c r="D31" s="28">
-        <f>IF(T31="","",IF(V31=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U31)),INDEX('1 Matériel'!$C$6:$C$29,U31)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U31)&gt;1,"  ("&amp;(T31-INDEX('1 Matériel'!$F$6:$F$29,U31)+INDEX('1 Matériel'!$E$6:$E$29,U31))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U31)&amp;")","")))</f>
+        <f>IF(T31=0,"",IF(V31=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U31)),INDEX('1 Matériel'!$C$6:$C$29,U31)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U31)&gt;1,"  ("&amp;(T31-INDEX('1 Matériel'!$F$6:$F$29,U31)+INDEX('1 Matériel'!$E$6:$E$29,U31))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U31)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E31" s="29" t="n"/>
@@ -2392,34 +2153,28 @@
       <c r="J31" s="30" t="n"/>
       <c r="K31" s="27" t="n"/>
       <c r="L31" s="30" t="n"/>
-      <c r="M31" s="31" t="n"/>
-      <c r="N31" s="30" t="n"/>
-      <c r="O31" s="30" t="n"/>
-      <c r="P31" s="30" t="n"/>
-      <c r="Q31" s="31" t="n"/>
-      <c r="R31" s="30" t="n"/>
-      <c r="T31" s="32">
-        <f>IF(17&lt;=SUM('1 Matériel'!$E$6:$E$29),17,"")</f>
-        <v/>
-      </c>
-      <c r="U31" s="32">
-        <f>IF(T31="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T31)+1)</f>
-        <v/>
-      </c>
-      <c r="V31" s="32">
+      <c r="T31" s="31">
+        <f>IF(17&lt;=SUM('1 Matériel'!$E$6:$E$29),17,0)</f>
+        <v/>
+      </c>
+      <c r="U31" s="31">
+        <f>IF(T31=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T31)+1)</f>
+        <v/>
+      </c>
+      <c r="V31" s="31">
         <f>IF(U31="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U31)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="32" ht="27" customHeight="1">
+    <row r="32" hidden="1" ht="27" customHeight="1">
       <c r="A32" s="7">
-        <f>IF(OR(T32="",V32=1),"",T32-COUNTIF(V$15:V32,1))</f>
+        <f>IF(OR(T32=0,V32=1),"",T32-COUNTIF(V$15:V32,1))</f>
         <v/>
       </c>
       <c r="B32" s="27" t="n"/>
       <c r="C32" s="27" t="n"/>
       <c r="D32" s="28">
-        <f>IF(T32="","",IF(V32=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U32)),INDEX('1 Matériel'!$C$6:$C$29,U32)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U32)&gt;1,"  ("&amp;(T32-INDEX('1 Matériel'!$F$6:$F$29,U32)+INDEX('1 Matériel'!$E$6:$E$29,U32))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U32)&amp;")","")))</f>
+        <f>IF(T32=0,"",IF(V32=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U32)),INDEX('1 Matériel'!$C$6:$C$29,U32)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U32)&gt;1,"  ("&amp;(T32-INDEX('1 Matériel'!$F$6:$F$29,U32)+INDEX('1 Matériel'!$E$6:$E$29,U32))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U32)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E32" s="29" t="n"/>
@@ -2430,34 +2185,28 @@
       <c r="J32" s="30" t="n"/>
       <c r="K32" s="27" t="n"/>
       <c r="L32" s="30" t="n"/>
-      <c r="M32" s="31" t="n"/>
-      <c r="N32" s="30" t="n"/>
-      <c r="O32" s="30" t="n"/>
-      <c r="P32" s="30" t="n"/>
-      <c r="Q32" s="31" t="n"/>
-      <c r="R32" s="30" t="n"/>
-      <c r="T32" s="32">
-        <f>IF(18&lt;=SUM('1 Matériel'!$E$6:$E$29),18,"")</f>
-        <v/>
-      </c>
-      <c r="U32" s="32">
-        <f>IF(T32="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T32)+1)</f>
-        <v/>
-      </c>
-      <c r="V32" s="32">
+      <c r="T32" s="31">
+        <f>IF(18&lt;=SUM('1 Matériel'!$E$6:$E$29),18,0)</f>
+        <v/>
+      </c>
+      <c r="U32" s="31">
+        <f>IF(T32=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T32)+1)</f>
+        <v/>
+      </c>
+      <c r="V32" s="31">
         <f>IF(U32="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U32)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="33" ht="27" customHeight="1">
+    <row r="33" hidden="1" ht="27" customHeight="1">
       <c r="A33" s="7">
-        <f>IF(OR(T33="",V33=1),"",T33-COUNTIF(V$15:V33,1))</f>
+        <f>IF(OR(T33=0,V33=1),"",T33-COUNTIF(V$15:V33,1))</f>
         <v/>
       </c>
       <c r="B33" s="27" t="n"/>
       <c r="C33" s="27" t="n"/>
       <c r="D33" s="28">
-        <f>IF(T33="","",IF(V33=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U33)),INDEX('1 Matériel'!$C$6:$C$29,U33)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U33)&gt;1,"  ("&amp;(T33-INDEX('1 Matériel'!$F$6:$F$29,U33)+INDEX('1 Matériel'!$E$6:$E$29,U33))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U33)&amp;")","")))</f>
+        <f>IF(T33=0,"",IF(V33=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U33)),INDEX('1 Matériel'!$C$6:$C$29,U33)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U33)&gt;1,"  ("&amp;(T33-INDEX('1 Matériel'!$F$6:$F$29,U33)+INDEX('1 Matériel'!$E$6:$E$29,U33))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U33)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E33" s="29" t="n"/>
@@ -2468,34 +2217,28 @@
       <c r="J33" s="30" t="n"/>
       <c r="K33" s="27" t="n"/>
       <c r="L33" s="30" t="n"/>
-      <c r="M33" s="31" t="n"/>
-      <c r="N33" s="30" t="n"/>
-      <c r="O33" s="30" t="n"/>
-      <c r="P33" s="30" t="n"/>
-      <c r="Q33" s="31" t="n"/>
-      <c r="R33" s="30" t="n"/>
-      <c r="T33" s="32">
-        <f>IF(19&lt;=SUM('1 Matériel'!$E$6:$E$29),19,"")</f>
-        <v/>
-      </c>
-      <c r="U33" s="32">
-        <f>IF(T33="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T33)+1)</f>
-        <v/>
-      </c>
-      <c r="V33" s="32">
+      <c r="T33" s="31">
+        <f>IF(19&lt;=SUM('1 Matériel'!$E$6:$E$29),19,0)</f>
+        <v/>
+      </c>
+      <c r="U33" s="31">
+        <f>IF(T33=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T33)+1)</f>
+        <v/>
+      </c>
+      <c r="V33" s="31">
         <f>IF(U33="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U33)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="34" ht="27" customHeight="1">
+    <row r="34" hidden="1" ht="27" customHeight="1">
       <c r="A34" s="7">
-        <f>IF(OR(T34="",V34=1),"",T34-COUNTIF(V$15:V34,1))</f>
+        <f>IF(OR(T34=0,V34=1),"",T34-COUNTIF(V$15:V34,1))</f>
         <v/>
       </c>
       <c r="B34" s="27" t="n"/>
       <c r="C34" s="27" t="n"/>
       <c r="D34" s="28">
-        <f>IF(T34="","",IF(V34=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U34)),INDEX('1 Matériel'!$C$6:$C$29,U34)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U34)&gt;1,"  ("&amp;(T34-INDEX('1 Matériel'!$F$6:$F$29,U34)+INDEX('1 Matériel'!$E$6:$E$29,U34))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U34)&amp;")","")))</f>
+        <f>IF(T34=0,"",IF(V34=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U34)),INDEX('1 Matériel'!$C$6:$C$29,U34)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U34)&gt;1,"  ("&amp;(T34-INDEX('1 Matériel'!$F$6:$F$29,U34)+INDEX('1 Matériel'!$E$6:$E$29,U34))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U34)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E34" s="29" t="n"/>
@@ -2506,34 +2249,28 @@
       <c r="J34" s="30" t="n"/>
       <c r="K34" s="27" t="n"/>
       <c r="L34" s="30" t="n"/>
-      <c r="M34" s="31" t="n"/>
-      <c r="N34" s="30" t="n"/>
-      <c r="O34" s="30" t="n"/>
-      <c r="P34" s="30" t="n"/>
-      <c r="Q34" s="31" t="n"/>
-      <c r="R34" s="30" t="n"/>
-      <c r="T34" s="32">
-        <f>IF(20&lt;=SUM('1 Matériel'!$E$6:$E$29),20,"")</f>
-        <v/>
-      </c>
-      <c r="U34" s="32">
-        <f>IF(T34="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T34)+1)</f>
-        <v/>
-      </c>
-      <c r="V34" s="32">
+      <c r="T34" s="31">
+        <f>IF(20&lt;=SUM('1 Matériel'!$E$6:$E$29),20,0)</f>
+        <v/>
+      </c>
+      <c r="U34" s="31">
+        <f>IF(T34=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T34)+1)</f>
+        <v/>
+      </c>
+      <c r="V34" s="31">
         <f>IF(U34="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U34)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="35" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="35" hidden="1" ht="27" customHeight="1">
       <c r="A35" s="7">
-        <f>IF(OR(T35="",V35=1),"",T35-COUNTIF(V$15:V35,1))</f>
+        <f>IF(OR(T35=0,V35=1),"",T35-COUNTIF(V$15:V35,1))</f>
         <v/>
       </c>
       <c r="B35" s="27" t="n"/>
       <c r="C35" s="27" t="n"/>
       <c r="D35" s="28">
-        <f>IF(T35="","",IF(V35=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U35)),INDEX('1 Matériel'!$C$6:$C$29,U35)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U35)&gt;1,"  ("&amp;(T35-INDEX('1 Matériel'!$F$6:$F$29,U35)+INDEX('1 Matériel'!$E$6:$E$29,U35))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U35)&amp;")","")))</f>
+        <f>IF(T35=0,"",IF(V35=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U35)),INDEX('1 Matériel'!$C$6:$C$29,U35)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U35)&gt;1,"  ("&amp;(T35-INDEX('1 Matériel'!$F$6:$F$29,U35)+INDEX('1 Matériel'!$E$6:$E$29,U35))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U35)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E35" s="29" t="n"/>
@@ -2544,34 +2281,28 @@
       <c r="J35" s="30" t="n"/>
       <c r="K35" s="27" t="n"/>
       <c r="L35" s="30" t="n"/>
-      <c r="M35" s="31" t="n"/>
-      <c r="N35" s="30" t="n"/>
-      <c r="O35" s="30" t="n"/>
-      <c r="P35" s="30" t="n"/>
-      <c r="Q35" s="31" t="n"/>
-      <c r="R35" s="30" t="n"/>
-      <c r="T35" s="32">
-        <f>IF(21&lt;=SUM('1 Matériel'!$E$6:$E$29),21,"")</f>
-        <v/>
-      </c>
-      <c r="U35" s="32">
-        <f>IF(T35="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T35)+1)</f>
-        <v/>
-      </c>
-      <c r="V35" s="32">
+      <c r="T35" s="31">
+        <f>IF(21&lt;=SUM('1 Matériel'!$E$6:$E$29),21,0)</f>
+        <v/>
+      </c>
+      <c r="U35" s="31">
+        <f>IF(T35=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T35)+1)</f>
+        <v/>
+      </c>
+      <c r="V35" s="31">
         <f>IF(U35="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U35)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="36" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="36" hidden="1" ht="27" customHeight="1">
       <c r="A36" s="7">
-        <f>IF(OR(T36="",V36=1),"",T36-COUNTIF(V$15:V36,1))</f>
+        <f>IF(OR(T36=0,V36=1),"",T36-COUNTIF(V$15:V36,1))</f>
         <v/>
       </c>
       <c r="B36" s="27" t="n"/>
       <c r="C36" s="27" t="n"/>
       <c r="D36" s="28">
-        <f>IF(T36="","",IF(V36=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U36)),INDEX('1 Matériel'!$C$6:$C$29,U36)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U36)&gt;1,"  ("&amp;(T36-INDEX('1 Matériel'!$F$6:$F$29,U36)+INDEX('1 Matériel'!$E$6:$E$29,U36))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U36)&amp;")","")))</f>
+        <f>IF(T36=0,"",IF(V36=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U36)),INDEX('1 Matériel'!$C$6:$C$29,U36)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U36)&gt;1,"  ("&amp;(T36-INDEX('1 Matériel'!$F$6:$F$29,U36)+INDEX('1 Matériel'!$E$6:$E$29,U36))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U36)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E36" s="29" t="n"/>
@@ -2582,34 +2313,28 @@
       <c r="J36" s="30" t="n"/>
       <c r="K36" s="27" t="n"/>
       <c r="L36" s="30" t="n"/>
-      <c r="M36" s="31" t="n"/>
-      <c r="N36" s="30" t="n"/>
-      <c r="O36" s="30" t="n"/>
-      <c r="P36" s="30" t="n"/>
-      <c r="Q36" s="31" t="n"/>
-      <c r="R36" s="30" t="n"/>
-      <c r="T36" s="32">
-        <f>IF(22&lt;=SUM('1 Matériel'!$E$6:$E$29),22,"")</f>
-        <v/>
-      </c>
-      <c r="U36" s="32">
-        <f>IF(T36="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T36)+1)</f>
-        <v/>
-      </c>
-      <c r="V36" s="32">
+      <c r="T36" s="31">
+        <f>IF(22&lt;=SUM('1 Matériel'!$E$6:$E$29),22,0)</f>
+        <v/>
+      </c>
+      <c r="U36" s="31">
+        <f>IF(T36=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T36)+1)</f>
+        <v/>
+      </c>
+      <c r="V36" s="31">
         <f>IF(U36="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U36)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="37" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="37" hidden="1" ht="27" customHeight="1">
       <c r="A37" s="7">
-        <f>IF(OR(T37="",V37=1),"",T37-COUNTIF(V$15:V37,1))</f>
+        <f>IF(OR(T37=0,V37=1),"",T37-COUNTIF(V$15:V37,1))</f>
         <v/>
       </c>
       <c r="B37" s="27" t="n"/>
       <c r="C37" s="27" t="n"/>
       <c r="D37" s="28">
-        <f>IF(T37="","",IF(V37=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U37)),INDEX('1 Matériel'!$C$6:$C$29,U37)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U37)&gt;1,"  ("&amp;(T37-INDEX('1 Matériel'!$F$6:$F$29,U37)+INDEX('1 Matériel'!$E$6:$E$29,U37))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U37)&amp;")","")))</f>
+        <f>IF(T37=0,"",IF(V37=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U37)),INDEX('1 Matériel'!$C$6:$C$29,U37)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U37)&gt;1,"  ("&amp;(T37-INDEX('1 Matériel'!$F$6:$F$29,U37)+INDEX('1 Matériel'!$E$6:$E$29,U37))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U37)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E37" s="29" t="n"/>
@@ -2620,34 +2345,28 @@
       <c r="J37" s="30" t="n"/>
       <c r="K37" s="27" t="n"/>
       <c r="L37" s="30" t="n"/>
-      <c r="M37" s="31" t="n"/>
-      <c r="N37" s="30" t="n"/>
-      <c r="O37" s="30" t="n"/>
-      <c r="P37" s="30" t="n"/>
-      <c r="Q37" s="31" t="n"/>
-      <c r="R37" s="30" t="n"/>
-      <c r="T37" s="32">
-        <f>IF(23&lt;=SUM('1 Matériel'!$E$6:$E$29),23,"")</f>
-        <v/>
-      </c>
-      <c r="U37" s="32">
-        <f>IF(T37="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T37)+1)</f>
-        <v/>
-      </c>
-      <c r="V37" s="32">
+      <c r="T37" s="31">
+        <f>IF(23&lt;=SUM('1 Matériel'!$E$6:$E$29),23,0)</f>
+        <v/>
+      </c>
+      <c r="U37" s="31">
+        <f>IF(T37=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T37)+1)</f>
+        <v/>
+      </c>
+      <c r="V37" s="31">
         <f>IF(U37="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U37)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="38" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="38" hidden="1" ht="27" customHeight="1">
       <c r="A38" s="7">
-        <f>IF(OR(T38="",V38=1),"",T38-COUNTIF(V$15:V38,1))</f>
+        <f>IF(OR(T38=0,V38=1),"",T38-COUNTIF(V$15:V38,1))</f>
         <v/>
       </c>
       <c r="B38" s="27" t="n"/>
       <c r="C38" s="27" t="n"/>
       <c r="D38" s="28">
-        <f>IF(T38="","",IF(V38=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U38)),INDEX('1 Matériel'!$C$6:$C$29,U38)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U38)&gt;1,"  ("&amp;(T38-INDEX('1 Matériel'!$F$6:$F$29,U38)+INDEX('1 Matériel'!$E$6:$E$29,U38))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U38)&amp;")","")))</f>
+        <f>IF(T38=0,"",IF(V38=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U38)),INDEX('1 Matériel'!$C$6:$C$29,U38)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U38)&gt;1,"  ("&amp;(T38-INDEX('1 Matériel'!$F$6:$F$29,U38)+INDEX('1 Matériel'!$E$6:$E$29,U38))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U38)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E38" s="29" t="n"/>
@@ -2658,34 +2377,28 @@
       <c r="J38" s="30" t="n"/>
       <c r="K38" s="27" t="n"/>
       <c r="L38" s="30" t="n"/>
-      <c r="M38" s="31" t="n"/>
-      <c r="N38" s="30" t="n"/>
-      <c r="O38" s="30" t="n"/>
-      <c r="P38" s="30" t="n"/>
-      <c r="Q38" s="31" t="n"/>
-      <c r="R38" s="30" t="n"/>
-      <c r="T38" s="32">
-        <f>IF(24&lt;=SUM('1 Matériel'!$E$6:$E$29),24,"")</f>
-        <v/>
-      </c>
-      <c r="U38" s="32">
-        <f>IF(T38="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T38)+1)</f>
-        <v/>
-      </c>
-      <c r="V38" s="32">
+      <c r="T38" s="31">
+        <f>IF(24&lt;=SUM('1 Matériel'!$E$6:$E$29),24,0)</f>
+        <v/>
+      </c>
+      <c r="U38" s="31">
+        <f>IF(T38=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T38)+1)</f>
+        <v/>
+      </c>
+      <c r="V38" s="31">
         <f>IF(U38="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U38)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="39" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="39" hidden="1" ht="27" customHeight="1">
       <c r="A39" s="7">
-        <f>IF(OR(T39="",V39=1),"",T39-COUNTIF(V$15:V39,1))</f>
+        <f>IF(OR(T39=0,V39=1),"",T39-COUNTIF(V$15:V39,1))</f>
         <v/>
       </c>
       <c r="B39" s="27" t="n"/>
       <c r="C39" s="27" t="n"/>
       <c r="D39" s="28">
-        <f>IF(T39="","",IF(V39=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U39)),INDEX('1 Matériel'!$C$6:$C$29,U39)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U39)&gt;1,"  ("&amp;(T39-INDEX('1 Matériel'!$F$6:$F$29,U39)+INDEX('1 Matériel'!$E$6:$E$29,U39))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U39)&amp;")","")))</f>
+        <f>IF(T39=0,"",IF(V39=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U39)),INDEX('1 Matériel'!$C$6:$C$29,U39)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U39)&gt;1,"  ("&amp;(T39-INDEX('1 Matériel'!$F$6:$F$29,U39)+INDEX('1 Matériel'!$E$6:$E$29,U39))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U39)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E39" s="29" t="n"/>
@@ -2696,34 +2409,28 @@
       <c r="J39" s="30" t="n"/>
       <c r="K39" s="27" t="n"/>
       <c r="L39" s="30" t="n"/>
-      <c r="M39" s="31" t="n"/>
-      <c r="N39" s="30" t="n"/>
-      <c r="O39" s="30" t="n"/>
-      <c r="P39" s="30" t="n"/>
-      <c r="Q39" s="31" t="n"/>
-      <c r="R39" s="30" t="n"/>
-      <c r="T39" s="32">
-        <f>IF(25&lt;=SUM('1 Matériel'!$E$6:$E$29),25,"")</f>
-        <v/>
-      </c>
-      <c r="U39" s="32">
-        <f>IF(T39="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T39)+1)</f>
-        <v/>
-      </c>
-      <c r="V39" s="32">
+      <c r="T39" s="31">
+        <f>IF(25&lt;=SUM('1 Matériel'!$E$6:$E$29),25,0)</f>
+        <v/>
+      </c>
+      <c r="U39" s="31">
+        <f>IF(T39=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T39)+1)</f>
+        <v/>
+      </c>
+      <c r="V39" s="31">
         <f>IF(U39="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U39)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="40" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="40" hidden="1" ht="27" customHeight="1">
       <c r="A40" s="7">
-        <f>IF(OR(T40="",V40=1),"",T40-COUNTIF(V$15:V40,1))</f>
+        <f>IF(OR(T40=0,V40=1),"",T40-COUNTIF(V$15:V40,1))</f>
         <v/>
       </c>
       <c r="B40" s="27" t="n"/>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="28">
-        <f>IF(T40="","",IF(V40=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U40)),INDEX('1 Matériel'!$C$6:$C$29,U40)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U40)&gt;1,"  ("&amp;(T40-INDEX('1 Matériel'!$F$6:$F$29,U40)+INDEX('1 Matériel'!$E$6:$E$29,U40))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U40)&amp;")","")))</f>
+        <f>IF(T40=0,"",IF(V40=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U40)),INDEX('1 Matériel'!$C$6:$C$29,U40)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U40)&gt;1,"  ("&amp;(T40-INDEX('1 Matériel'!$F$6:$F$29,U40)+INDEX('1 Matériel'!$E$6:$E$29,U40))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U40)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E40" s="29" t="n"/>
@@ -2734,34 +2441,28 @@
       <c r="J40" s="30" t="n"/>
       <c r="K40" s="27" t="n"/>
       <c r="L40" s="30" t="n"/>
-      <c r="M40" s="31" t="n"/>
-      <c r="N40" s="30" t="n"/>
-      <c r="O40" s="30" t="n"/>
-      <c r="P40" s="30" t="n"/>
-      <c r="Q40" s="31" t="n"/>
-      <c r="R40" s="30" t="n"/>
-      <c r="T40" s="32">
-        <f>IF(26&lt;=SUM('1 Matériel'!$E$6:$E$29),26,"")</f>
-        <v/>
-      </c>
-      <c r="U40" s="32">
-        <f>IF(T40="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T40)+1)</f>
-        <v/>
-      </c>
-      <c r="V40" s="32">
+      <c r="T40" s="31">
+        <f>IF(26&lt;=SUM('1 Matériel'!$E$6:$E$29),26,0)</f>
+        <v/>
+      </c>
+      <c r="U40" s="31">
+        <f>IF(T40=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T40)+1)</f>
+        <v/>
+      </c>
+      <c r="V40" s="31">
         <f>IF(U40="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U40)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="41" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="41" hidden="1" ht="27" customHeight="1">
       <c r="A41" s="7">
-        <f>IF(OR(T41="",V41=1),"",T41-COUNTIF(V$15:V41,1))</f>
+        <f>IF(OR(T41=0,V41=1),"",T41-COUNTIF(V$15:V41,1))</f>
         <v/>
       </c>
       <c r="B41" s="27" t="n"/>
       <c r="C41" s="27" t="n"/>
       <c r="D41" s="28">
-        <f>IF(T41="","",IF(V41=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U41)),INDEX('1 Matériel'!$C$6:$C$29,U41)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U41)&gt;1,"  ("&amp;(T41-INDEX('1 Matériel'!$F$6:$F$29,U41)+INDEX('1 Matériel'!$E$6:$E$29,U41))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U41)&amp;")","")))</f>
+        <f>IF(T41=0,"",IF(V41=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U41)),INDEX('1 Matériel'!$C$6:$C$29,U41)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U41)&gt;1,"  ("&amp;(T41-INDEX('1 Matériel'!$F$6:$F$29,U41)+INDEX('1 Matériel'!$E$6:$E$29,U41))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U41)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E41" s="29" t="n"/>
@@ -2772,34 +2473,28 @@
       <c r="J41" s="30" t="n"/>
       <c r="K41" s="27" t="n"/>
       <c r="L41" s="30" t="n"/>
-      <c r="M41" s="31" t="n"/>
-      <c r="N41" s="30" t="n"/>
-      <c r="O41" s="30" t="n"/>
-      <c r="P41" s="30" t="n"/>
-      <c r="Q41" s="31" t="n"/>
-      <c r="R41" s="30" t="n"/>
-      <c r="T41" s="32">
-        <f>IF(27&lt;=SUM('1 Matériel'!$E$6:$E$29),27,"")</f>
-        <v/>
-      </c>
-      <c r="U41" s="32">
-        <f>IF(T41="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T41)+1)</f>
-        <v/>
-      </c>
-      <c r="V41" s="32">
+      <c r="T41" s="31">
+        <f>IF(27&lt;=SUM('1 Matériel'!$E$6:$E$29),27,0)</f>
+        <v/>
+      </c>
+      <c r="U41" s="31">
+        <f>IF(T41=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T41)+1)</f>
+        <v/>
+      </c>
+      <c r="V41" s="31">
         <f>IF(U41="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U41)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="42" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="42" hidden="1" ht="27" customHeight="1">
       <c r="A42" s="7">
-        <f>IF(OR(T42="",V42=1),"",T42-COUNTIF(V$15:V42,1))</f>
+        <f>IF(OR(T42=0,V42=1),"",T42-COUNTIF(V$15:V42,1))</f>
         <v/>
       </c>
       <c r="B42" s="27" t="n"/>
       <c r="C42" s="27" t="n"/>
       <c r="D42" s="28">
-        <f>IF(T42="","",IF(V42=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U42)),INDEX('1 Matériel'!$C$6:$C$29,U42)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U42)&gt;1,"  ("&amp;(T42-INDEX('1 Matériel'!$F$6:$F$29,U42)+INDEX('1 Matériel'!$E$6:$E$29,U42))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U42)&amp;")","")))</f>
+        <f>IF(T42=0,"",IF(V42=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U42)),INDEX('1 Matériel'!$C$6:$C$29,U42)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U42)&gt;1,"  ("&amp;(T42-INDEX('1 Matériel'!$F$6:$F$29,U42)+INDEX('1 Matériel'!$E$6:$E$29,U42))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U42)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E42" s="29" t="n"/>
@@ -2810,34 +2505,28 @@
       <c r="J42" s="30" t="n"/>
       <c r="K42" s="27" t="n"/>
       <c r="L42" s="30" t="n"/>
-      <c r="M42" s="31" t="n"/>
-      <c r="N42" s="30" t="n"/>
-      <c r="O42" s="30" t="n"/>
-      <c r="P42" s="30" t="n"/>
-      <c r="Q42" s="31" t="n"/>
-      <c r="R42" s="30" t="n"/>
-      <c r="T42" s="32">
-        <f>IF(28&lt;=SUM('1 Matériel'!$E$6:$E$29),28,"")</f>
-        <v/>
-      </c>
-      <c r="U42" s="32">
-        <f>IF(T42="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T42)+1)</f>
-        <v/>
-      </c>
-      <c r="V42" s="32">
+      <c r="T42" s="31">
+        <f>IF(28&lt;=SUM('1 Matériel'!$E$6:$E$29),28,0)</f>
+        <v/>
+      </c>
+      <c r="U42" s="31">
+        <f>IF(T42=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T42)+1)</f>
+        <v/>
+      </c>
+      <c r="V42" s="31">
         <f>IF(U42="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U42)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="43" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="43" hidden="1" ht="27" customHeight="1">
       <c r="A43" s="7">
-        <f>IF(OR(T43="",V43=1),"",T43-COUNTIF(V$15:V43,1))</f>
+        <f>IF(OR(T43=0,V43=1),"",T43-COUNTIF(V$15:V43,1))</f>
         <v/>
       </c>
       <c r="B43" s="27" t="n"/>
       <c r="C43" s="27" t="n"/>
       <c r="D43" s="28">
-        <f>IF(T43="","",IF(V43=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U43)),INDEX('1 Matériel'!$C$6:$C$29,U43)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U43)&gt;1,"  ("&amp;(T43-INDEX('1 Matériel'!$F$6:$F$29,U43)+INDEX('1 Matériel'!$E$6:$E$29,U43))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U43)&amp;")","")))</f>
+        <f>IF(T43=0,"",IF(V43=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U43)),INDEX('1 Matériel'!$C$6:$C$29,U43)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U43)&gt;1,"  ("&amp;(T43-INDEX('1 Matériel'!$F$6:$F$29,U43)+INDEX('1 Matériel'!$E$6:$E$29,U43))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U43)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E43" s="29" t="n"/>
@@ -2848,34 +2537,28 @@
       <c r="J43" s="30" t="n"/>
       <c r="K43" s="27" t="n"/>
       <c r="L43" s="30" t="n"/>
-      <c r="M43" s="31" t="n"/>
-      <c r="N43" s="30" t="n"/>
-      <c r="O43" s="30" t="n"/>
-      <c r="P43" s="30" t="n"/>
-      <c r="Q43" s="31" t="n"/>
-      <c r="R43" s="30" t="n"/>
-      <c r="T43" s="32">
-        <f>IF(29&lt;=SUM('1 Matériel'!$E$6:$E$29),29,"")</f>
-        <v/>
-      </c>
-      <c r="U43" s="32">
-        <f>IF(T43="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T43)+1)</f>
-        <v/>
-      </c>
-      <c r="V43" s="32">
+      <c r="T43" s="31">
+        <f>IF(29&lt;=SUM('1 Matériel'!$E$6:$E$29),29,0)</f>
+        <v/>
+      </c>
+      <c r="U43" s="31">
+        <f>IF(T43=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T43)+1)</f>
+        <v/>
+      </c>
+      <c r="V43" s="31">
         <f>IF(U43="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U43)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="44" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="44" hidden="1" ht="27" customHeight="1">
       <c r="A44" s="7">
-        <f>IF(OR(T44="",V44=1),"",T44-COUNTIF(V$15:V44,1))</f>
+        <f>IF(OR(T44=0,V44=1),"",T44-COUNTIF(V$15:V44,1))</f>
         <v/>
       </c>
       <c r="B44" s="27" t="n"/>
       <c r="C44" s="27" t="n"/>
       <c r="D44" s="28">
-        <f>IF(T44="","",IF(V44=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U44)),INDEX('1 Matériel'!$C$6:$C$29,U44)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U44)&gt;1,"  ("&amp;(T44-INDEX('1 Matériel'!$F$6:$F$29,U44)+INDEX('1 Matériel'!$E$6:$E$29,U44))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U44)&amp;")","")))</f>
+        <f>IF(T44=0,"",IF(V44=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U44)),INDEX('1 Matériel'!$C$6:$C$29,U44)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U44)&gt;1,"  ("&amp;(T44-INDEX('1 Matériel'!$F$6:$F$29,U44)+INDEX('1 Matériel'!$E$6:$E$29,U44))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U44)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E44" s="29" t="n"/>
@@ -2886,34 +2569,28 @@
       <c r="J44" s="30" t="n"/>
       <c r="K44" s="27" t="n"/>
       <c r="L44" s="30" t="n"/>
-      <c r="M44" s="31" t="n"/>
-      <c r="N44" s="30" t="n"/>
-      <c r="O44" s="30" t="n"/>
-      <c r="P44" s="30" t="n"/>
-      <c r="Q44" s="31" t="n"/>
-      <c r="R44" s="30" t="n"/>
-      <c r="T44" s="32">
-        <f>IF(30&lt;=SUM('1 Matériel'!$E$6:$E$29),30,"")</f>
-        <v/>
-      </c>
-      <c r="U44" s="32">
-        <f>IF(T44="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T44)+1)</f>
-        <v/>
-      </c>
-      <c r="V44" s="32">
+      <c r="T44" s="31">
+        <f>IF(30&lt;=SUM('1 Matériel'!$E$6:$E$29),30,0)</f>
+        <v/>
+      </c>
+      <c r="U44" s="31">
+        <f>IF(T44=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T44)+1)</f>
+        <v/>
+      </c>
+      <c r="V44" s="31">
         <f>IF(U44="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U44)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="45" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="45" hidden="1" ht="27" customHeight="1">
       <c r="A45" s="7">
-        <f>IF(OR(T45="",V45=1),"",T45-COUNTIF(V$15:V45,1))</f>
+        <f>IF(OR(T45=0,V45=1),"",T45-COUNTIF(V$15:V45,1))</f>
         <v/>
       </c>
       <c r="B45" s="27" t="n"/>
       <c r="C45" s="27" t="n"/>
       <c r="D45" s="28">
-        <f>IF(T45="","",IF(V45=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U45)),INDEX('1 Matériel'!$C$6:$C$29,U45)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U45)&gt;1,"  ("&amp;(T45-INDEX('1 Matériel'!$F$6:$F$29,U45)+INDEX('1 Matériel'!$E$6:$E$29,U45))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U45)&amp;")","")))</f>
+        <f>IF(T45=0,"",IF(V45=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U45)),INDEX('1 Matériel'!$C$6:$C$29,U45)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U45)&gt;1,"  ("&amp;(T45-INDEX('1 Matériel'!$F$6:$F$29,U45)+INDEX('1 Matériel'!$E$6:$E$29,U45))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U45)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E45" s="29" t="n"/>
@@ -2924,34 +2601,28 @@
       <c r="J45" s="30" t="n"/>
       <c r="K45" s="27" t="n"/>
       <c r="L45" s="30" t="n"/>
-      <c r="M45" s="31" t="n"/>
-      <c r="N45" s="30" t="n"/>
-      <c r="O45" s="30" t="n"/>
-      <c r="P45" s="30" t="n"/>
-      <c r="Q45" s="31" t="n"/>
-      <c r="R45" s="30" t="n"/>
-      <c r="T45" s="32">
-        <f>IF(31&lt;=SUM('1 Matériel'!$E$6:$E$29),31,"")</f>
-        <v/>
-      </c>
-      <c r="U45" s="32">
-        <f>IF(T45="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T45)+1)</f>
-        <v/>
-      </c>
-      <c r="V45" s="32">
+      <c r="T45" s="31">
+        <f>IF(31&lt;=SUM('1 Matériel'!$E$6:$E$29),31,0)</f>
+        <v/>
+      </c>
+      <c r="U45" s="31">
+        <f>IF(T45=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T45)+1)</f>
+        <v/>
+      </c>
+      <c r="V45" s="31">
         <f>IF(U45="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U45)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="46" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="46" hidden="1" ht="27" customHeight="1">
       <c r="A46" s="7">
-        <f>IF(OR(T46="",V46=1),"",T46-COUNTIF(V$15:V46,1))</f>
+        <f>IF(OR(T46=0,V46=1),"",T46-COUNTIF(V$15:V46,1))</f>
         <v/>
       </c>
       <c r="B46" s="27" t="n"/>
       <c r="C46" s="27" t="n"/>
       <c r="D46" s="28">
-        <f>IF(T46="","",IF(V46=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U46)),INDEX('1 Matériel'!$C$6:$C$29,U46)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U46)&gt;1,"  ("&amp;(T46-INDEX('1 Matériel'!$F$6:$F$29,U46)+INDEX('1 Matériel'!$E$6:$E$29,U46))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U46)&amp;")","")))</f>
+        <f>IF(T46=0,"",IF(V46=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U46)),INDEX('1 Matériel'!$C$6:$C$29,U46)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U46)&gt;1,"  ("&amp;(T46-INDEX('1 Matériel'!$F$6:$F$29,U46)+INDEX('1 Matériel'!$E$6:$E$29,U46))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U46)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E46" s="29" t="n"/>
@@ -2962,34 +2633,28 @@
       <c r="J46" s="30" t="n"/>
       <c r="K46" s="27" t="n"/>
       <c r="L46" s="30" t="n"/>
-      <c r="M46" s="31" t="n"/>
-      <c r="N46" s="30" t="n"/>
-      <c r="O46" s="30" t="n"/>
-      <c r="P46" s="30" t="n"/>
-      <c r="Q46" s="31" t="n"/>
-      <c r="R46" s="30" t="n"/>
-      <c r="T46" s="32">
-        <f>IF(32&lt;=SUM('1 Matériel'!$E$6:$E$29),32,"")</f>
-        <v/>
-      </c>
-      <c r="U46" s="32">
-        <f>IF(T46="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T46)+1)</f>
-        <v/>
-      </c>
-      <c r="V46" s="32">
+      <c r="T46" s="31">
+        <f>IF(32&lt;=SUM('1 Matériel'!$E$6:$E$29),32,0)</f>
+        <v/>
+      </c>
+      <c r="U46" s="31">
+        <f>IF(T46=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T46)+1)</f>
+        <v/>
+      </c>
+      <c r="V46" s="31">
         <f>IF(U46="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U46)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="47" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="47" hidden="1" ht="27" customHeight="1">
       <c r="A47" s="7">
-        <f>IF(OR(T47="",V47=1),"",T47-COUNTIF(V$15:V47,1))</f>
+        <f>IF(OR(T47=0,V47=1),"",T47-COUNTIF(V$15:V47,1))</f>
         <v/>
       </c>
       <c r="B47" s="27" t="n"/>
       <c r="C47" s="27" t="n"/>
       <c r="D47" s="28">
-        <f>IF(T47="","",IF(V47=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U47)),INDEX('1 Matériel'!$C$6:$C$29,U47)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U47)&gt;1,"  ("&amp;(T47-INDEX('1 Matériel'!$F$6:$F$29,U47)+INDEX('1 Matériel'!$E$6:$E$29,U47))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U47)&amp;")","")))</f>
+        <f>IF(T47=0,"",IF(V47=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U47)),INDEX('1 Matériel'!$C$6:$C$29,U47)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U47)&gt;1,"  ("&amp;(T47-INDEX('1 Matériel'!$F$6:$F$29,U47)+INDEX('1 Matériel'!$E$6:$E$29,U47))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U47)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E47" s="29" t="n"/>
@@ -3000,34 +2665,28 @@
       <c r="J47" s="30" t="n"/>
       <c r="K47" s="27" t="n"/>
       <c r="L47" s="30" t="n"/>
-      <c r="M47" s="31" t="n"/>
-      <c r="N47" s="30" t="n"/>
-      <c r="O47" s="30" t="n"/>
-      <c r="P47" s="30" t="n"/>
-      <c r="Q47" s="31" t="n"/>
-      <c r="R47" s="30" t="n"/>
-      <c r="T47" s="32">
-        <f>IF(33&lt;=SUM('1 Matériel'!$E$6:$E$29),33,"")</f>
-        <v/>
-      </c>
-      <c r="U47" s="32">
-        <f>IF(T47="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T47)+1)</f>
-        <v/>
-      </c>
-      <c r="V47" s="32">
+      <c r="T47" s="31">
+        <f>IF(33&lt;=SUM('1 Matériel'!$E$6:$E$29),33,0)</f>
+        <v/>
+      </c>
+      <c r="U47" s="31">
+        <f>IF(T47=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T47)+1)</f>
+        <v/>
+      </c>
+      <c r="V47" s="31">
         <f>IF(U47="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U47)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="48" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="48" hidden="1" ht="27" customHeight="1">
       <c r="A48" s="7">
-        <f>IF(OR(T48="",V48=1),"",T48-COUNTIF(V$15:V48,1))</f>
+        <f>IF(OR(T48=0,V48=1),"",T48-COUNTIF(V$15:V48,1))</f>
         <v/>
       </c>
       <c r="B48" s="27" t="n"/>
       <c r="C48" s="27" t="n"/>
       <c r="D48" s="28">
-        <f>IF(T48="","",IF(V48=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U48)),INDEX('1 Matériel'!$C$6:$C$29,U48)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U48)&gt;1,"  ("&amp;(T48-INDEX('1 Matériel'!$F$6:$F$29,U48)+INDEX('1 Matériel'!$E$6:$E$29,U48))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U48)&amp;")","")))</f>
+        <f>IF(T48=0,"",IF(V48=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U48)),INDEX('1 Matériel'!$C$6:$C$29,U48)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U48)&gt;1,"  ("&amp;(T48-INDEX('1 Matériel'!$F$6:$F$29,U48)+INDEX('1 Matériel'!$E$6:$E$29,U48))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U48)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E48" s="29" t="n"/>
@@ -3038,34 +2697,28 @@
       <c r="J48" s="30" t="n"/>
       <c r="K48" s="27" t="n"/>
       <c r="L48" s="30" t="n"/>
-      <c r="M48" s="31" t="n"/>
-      <c r="N48" s="30" t="n"/>
-      <c r="O48" s="30" t="n"/>
-      <c r="P48" s="30" t="n"/>
-      <c r="Q48" s="31" t="n"/>
-      <c r="R48" s="30" t="n"/>
-      <c r="T48" s="32">
-        <f>IF(34&lt;=SUM('1 Matériel'!$E$6:$E$29),34,"")</f>
-        <v/>
-      </c>
-      <c r="U48" s="32">
-        <f>IF(T48="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T48)+1)</f>
-        <v/>
-      </c>
-      <c r="V48" s="32">
+      <c r="T48" s="31">
+        <f>IF(34&lt;=SUM('1 Matériel'!$E$6:$E$29),34,0)</f>
+        <v/>
+      </c>
+      <c r="U48" s="31">
+        <f>IF(T48=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T48)+1)</f>
+        <v/>
+      </c>
+      <c r="V48" s="31">
         <f>IF(U48="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U48)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="49" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="49" hidden="1" ht="27" customHeight="1">
       <c r="A49" s="7">
-        <f>IF(OR(T49="",V49=1),"",T49-COUNTIF(V$15:V49,1))</f>
+        <f>IF(OR(T49=0,V49=1),"",T49-COUNTIF(V$15:V49,1))</f>
         <v/>
       </c>
       <c r="B49" s="27" t="n"/>
       <c r="C49" s="27" t="n"/>
       <c r="D49" s="28">
-        <f>IF(T49="","",IF(V49=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U49)),INDEX('1 Matériel'!$C$6:$C$29,U49)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U49)&gt;1,"  ("&amp;(T49-INDEX('1 Matériel'!$F$6:$F$29,U49)+INDEX('1 Matériel'!$E$6:$E$29,U49))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U49)&amp;")","")))</f>
+        <f>IF(T49=0,"",IF(V49=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U49)),INDEX('1 Matériel'!$C$6:$C$29,U49)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U49)&gt;1,"  ("&amp;(T49-INDEX('1 Matériel'!$F$6:$F$29,U49)+INDEX('1 Matériel'!$E$6:$E$29,U49))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U49)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E49" s="29" t="n"/>
@@ -3076,34 +2729,28 @@
       <c r="J49" s="30" t="n"/>
       <c r="K49" s="27" t="n"/>
       <c r="L49" s="30" t="n"/>
-      <c r="M49" s="31" t="n"/>
-      <c r="N49" s="30" t="n"/>
-      <c r="O49" s="30" t="n"/>
-      <c r="P49" s="30" t="n"/>
-      <c r="Q49" s="31" t="n"/>
-      <c r="R49" s="30" t="n"/>
-      <c r="T49" s="32">
-        <f>IF(35&lt;=SUM('1 Matériel'!$E$6:$E$29),35,"")</f>
-        <v/>
-      </c>
-      <c r="U49" s="32">
-        <f>IF(T49="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T49)+1)</f>
-        <v/>
-      </c>
-      <c r="V49" s="32">
+      <c r="T49" s="31">
+        <f>IF(35&lt;=SUM('1 Matériel'!$E$6:$E$29),35,0)</f>
+        <v/>
+      </c>
+      <c r="U49" s="31">
+        <f>IF(T49=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T49)+1)</f>
+        <v/>
+      </c>
+      <c r="V49" s="31">
         <f>IF(U49="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U49)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="50" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="50" hidden="1" ht="27" customHeight="1">
       <c r="A50" s="7">
-        <f>IF(OR(T50="",V50=1),"",T50-COUNTIF(V$15:V50,1))</f>
+        <f>IF(OR(T50=0,V50=1),"",T50-COUNTIF(V$15:V50,1))</f>
         <v/>
       </c>
       <c r="B50" s="27" t="n"/>
       <c r="C50" s="27" t="n"/>
       <c r="D50" s="28">
-        <f>IF(T50="","",IF(V50=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U50)),INDEX('1 Matériel'!$C$6:$C$29,U50)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U50)&gt;1,"  ("&amp;(T50-INDEX('1 Matériel'!$F$6:$F$29,U50)+INDEX('1 Matériel'!$E$6:$E$29,U50))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U50)&amp;")","")))</f>
+        <f>IF(T50=0,"",IF(V50=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U50)),INDEX('1 Matériel'!$C$6:$C$29,U50)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U50)&gt;1,"  ("&amp;(T50-INDEX('1 Matériel'!$F$6:$F$29,U50)+INDEX('1 Matériel'!$E$6:$E$29,U50))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U50)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E50" s="29" t="n"/>
@@ -3114,34 +2761,28 @@
       <c r="J50" s="30" t="n"/>
       <c r="K50" s="27" t="n"/>
       <c r="L50" s="30" t="n"/>
-      <c r="M50" s="31" t="n"/>
-      <c r="N50" s="30" t="n"/>
-      <c r="O50" s="30" t="n"/>
-      <c r="P50" s="30" t="n"/>
-      <c r="Q50" s="31" t="n"/>
-      <c r="R50" s="30" t="n"/>
-      <c r="T50" s="32">
-        <f>IF(36&lt;=SUM('1 Matériel'!$E$6:$E$29),36,"")</f>
-        <v/>
-      </c>
-      <c r="U50" s="32">
-        <f>IF(T50="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T50)+1)</f>
-        <v/>
-      </c>
-      <c r="V50" s="32">
+      <c r="T50" s="31">
+        <f>IF(36&lt;=SUM('1 Matériel'!$E$6:$E$29),36,0)</f>
+        <v/>
+      </c>
+      <c r="U50" s="31">
+        <f>IF(T50=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T50)+1)</f>
+        <v/>
+      </c>
+      <c r="V50" s="31">
         <f>IF(U50="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U50)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="51" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="51" hidden="1" ht="27" customHeight="1">
       <c r="A51" s="7">
-        <f>IF(OR(T51="",V51=1),"",T51-COUNTIF(V$15:V51,1))</f>
+        <f>IF(OR(T51=0,V51=1),"",T51-COUNTIF(V$15:V51,1))</f>
         <v/>
       </c>
       <c r="B51" s="27" t="n"/>
       <c r="C51" s="27" t="n"/>
       <c r="D51" s="28">
-        <f>IF(T51="","",IF(V51=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U51)),INDEX('1 Matériel'!$C$6:$C$29,U51)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U51)&gt;1,"  ("&amp;(T51-INDEX('1 Matériel'!$F$6:$F$29,U51)+INDEX('1 Matériel'!$E$6:$E$29,U51))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U51)&amp;")","")))</f>
+        <f>IF(T51=0,"",IF(V51=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U51)),INDEX('1 Matériel'!$C$6:$C$29,U51)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U51)&gt;1,"  ("&amp;(T51-INDEX('1 Matériel'!$F$6:$F$29,U51)+INDEX('1 Matériel'!$E$6:$E$29,U51))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U51)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E51" s="29" t="n"/>
@@ -3152,34 +2793,28 @@
       <c r="J51" s="30" t="n"/>
       <c r="K51" s="27" t="n"/>
       <c r="L51" s="30" t="n"/>
-      <c r="M51" s="31" t="n"/>
-      <c r="N51" s="30" t="n"/>
-      <c r="O51" s="30" t="n"/>
-      <c r="P51" s="30" t="n"/>
-      <c r="Q51" s="31" t="n"/>
-      <c r="R51" s="30" t="n"/>
-      <c r="T51" s="32">
-        <f>IF(37&lt;=SUM('1 Matériel'!$E$6:$E$29),37,"")</f>
-        <v/>
-      </c>
-      <c r="U51" s="32">
-        <f>IF(T51="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T51)+1)</f>
-        <v/>
-      </c>
-      <c r="V51" s="32">
+      <c r="T51" s="31">
+        <f>IF(37&lt;=SUM('1 Matériel'!$E$6:$E$29),37,0)</f>
+        <v/>
+      </c>
+      <c r="U51" s="31">
+        <f>IF(T51=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T51)+1)</f>
+        <v/>
+      </c>
+      <c r="V51" s="31">
         <f>IF(U51="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U51)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="52" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="52" hidden="1" ht="27" customHeight="1">
       <c r="A52" s="7">
-        <f>IF(OR(T52="",V52=1),"",T52-COUNTIF(V$15:V52,1))</f>
+        <f>IF(OR(T52=0,V52=1),"",T52-COUNTIF(V$15:V52,1))</f>
         <v/>
       </c>
       <c r="B52" s="27" t="n"/>
       <c r="C52" s="27" t="n"/>
       <c r="D52" s="28">
-        <f>IF(T52="","",IF(V52=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U52)),INDEX('1 Matériel'!$C$6:$C$29,U52)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U52)&gt;1,"  ("&amp;(T52-INDEX('1 Matériel'!$F$6:$F$29,U52)+INDEX('1 Matériel'!$E$6:$E$29,U52))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U52)&amp;")","")))</f>
+        <f>IF(T52=0,"",IF(V52=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U52)),INDEX('1 Matériel'!$C$6:$C$29,U52)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U52)&gt;1,"  ("&amp;(T52-INDEX('1 Matériel'!$F$6:$F$29,U52)+INDEX('1 Matériel'!$E$6:$E$29,U52))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U52)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E52" s="29" t="n"/>
@@ -3190,34 +2825,28 @@
       <c r="J52" s="30" t="n"/>
       <c r="K52" s="27" t="n"/>
       <c r="L52" s="30" t="n"/>
-      <c r="M52" s="31" t="n"/>
-      <c r="N52" s="30" t="n"/>
-      <c r="O52" s="30" t="n"/>
-      <c r="P52" s="30" t="n"/>
-      <c r="Q52" s="31" t="n"/>
-      <c r="R52" s="30" t="n"/>
-      <c r="T52" s="32">
-        <f>IF(38&lt;=SUM('1 Matériel'!$E$6:$E$29),38,"")</f>
-        <v/>
-      </c>
-      <c r="U52" s="32">
-        <f>IF(T52="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T52)+1)</f>
-        <v/>
-      </c>
-      <c r="V52" s="32">
+      <c r="T52" s="31">
+        <f>IF(38&lt;=SUM('1 Matériel'!$E$6:$E$29),38,0)</f>
+        <v/>
+      </c>
+      <c r="U52" s="31">
+        <f>IF(T52=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T52)+1)</f>
+        <v/>
+      </c>
+      <c r="V52" s="31">
         <f>IF(U52="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U52)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="53" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="53" hidden="1" ht="27" customHeight="1">
       <c r="A53" s="7">
-        <f>IF(OR(T53="",V53=1),"",T53-COUNTIF(V$15:V53,1))</f>
+        <f>IF(OR(T53=0,V53=1),"",T53-COUNTIF(V$15:V53,1))</f>
         <v/>
       </c>
       <c r="B53" s="27" t="n"/>
       <c r="C53" s="27" t="n"/>
       <c r="D53" s="28">
-        <f>IF(T53="","",IF(V53=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U53)),INDEX('1 Matériel'!$C$6:$C$29,U53)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U53)&gt;1,"  ("&amp;(T53-INDEX('1 Matériel'!$F$6:$F$29,U53)+INDEX('1 Matériel'!$E$6:$E$29,U53))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U53)&amp;")","")))</f>
+        <f>IF(T53=0,"",IF(V53=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U53)),INDEX('1 Matériel'!$C$6:$C$29,U53)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U53)&gt;1,"  ("&amp;(T53-INDEX('1 Matériel'!$F$6:$F$29,U53)+INDEX('1 Matériel'!$E$6:$E$29,U53))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U53)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E53" s="29" t="n"/>
@@ -3228,34 +2857,28 @@
       <c r="J53" s="30" t="n"/>
       <c r="K53" s="27" t="n"/>
       <c r="L53" s="30" t="n"/>
-      <c r="M53" s="31" t="n"/>
-      <c r="N53" s="30" t="n"/>
-      <c r="O53" s="30" t="n"/>
-      <c r="P53" s="30" t="n"/>
-      <c r="Q53" s="31" t="n"/>
-      <c r="R53" s="30" t="n"/>
-      <c r="T53" s="32">
-        <f>IF(39&lt;=SUM('1 Matériel'!$E$6:$E$29),39,"")</f>
-        <v/>
-      </c>
-      <c r="U53" s="32">
-        <f>IF(T53="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T53)+1)</f>
-        <v/>
-      </c>
-      <c r="V53" s="32">
+      <c r="T53" s="31">
+        <f>IF(39&lt;=SUM('1 Matériel'!$E$6:$E$29),39,0)</f>
+        <v/>
+      </c>
+      <c r="U53" s="31">
+        <f>IF(T53=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T53)+1)</f>
+        <v/>
+      </c>
+      <c r="V53" s="31">
         <f>IF(U53="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U53)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="54" hidden="1" outlineLevel="1" ht="27" customHeight="1">
+    <row r="54" hidden="1" ht="27" customHeight="1">
       <c r="A54" s="7">
-        <f>IF(OR(T54="",V54=1),"",T54-COUNTIF(V$15:V54,1))</f>
+        <f>IF(OR(T54=0,V54=1),"",T54-COUNTIF(V$15:V54,1))</f>
         <v/>
       </c>
       <c r="B54" s="27" t="n"/>
       <c r="C54" s="27" t="n"/>
       <c r="D54" s="28">
-        <f>IF(T54="","",IF(V54=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U54)),INDEX('1 Matériel'!$C$6:$C$29,U54)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U54)&gt;1,"  ("&amp;(T54-INDEX('1 Matériel'!$F$6:$F$29,U54)+INDEX('1 Matériel'!$E$6:$E$29,U54))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U54)&amp;")","")))</f>
+        <f>IF(T54=0,"",IF(V54=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U54)),INDEX('1 Matériel'!$C$6:$C$29,U54)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U54)&gt;1,"  ("&amp;(T54-INDEX('1 Matériel'!$F$6:$F$29,U54)+INDEX('1 Matériel'!$E$6:$E$29,U54))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U54)&amp;")","")))</f>
         <v/>
       </c>
       <c r="E54" s="29" t="n"/>
@@ -3266,31 +2889,21 @@
       <c r="J54" s="30" t="n"/>
       <c r="K54" s="27" t="n"/>
       <c r="L54" s="30" t="n"/>
-      <c r="M54" s="31" t="n"/>
-      <c r="N54" s="30" t="n"/>
-      <c r="O54" s="30" t="n"/>
-      <c r="P54" s="30" t="n"/>
-      <c r="Q54" s="31" t="n"/>
-      <c r="R54" s="30" t="n"/>
-      <c r="T54" s="32">
-        <f>IF(40&lt;=SUM('1 Matériel'!$E$6:$E$29),40,"")</f>
-        <v/>
-      </c>
-      <c r="U54" s="32">
-        <f>IF(T54="","",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T54)+1)</f>
-        <v/>
-      </c>
-      <c r="V54" s="32">
+      <c r="T54" s="31">
+        <f>IF(40&lt;=SUM('1 Matériel'!$E$6:$E$29),40,0)</f>
+        <v/>
+      </c>
+      <c r="U54" s="31">
+        <f>IF(T54=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T54)+1)</f>
+        <v/>
+      </c>
+      <c r="V54" s="31">
         <f>IF(U54="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U54)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="33">
-        <f>IF(SUM('1 Matériel'!$E$6:$E$29)&gt;20,"⚠  "&amp;(SUM('1 Matériel'!$E$6:$E$29)-20)&amp;" ligne(s) au-delà de la ligne 20 sont masquées : cliquer sur le [+] dans la marge gauche pour les afficher.","")</f>
-        <v/>
-      </c>
-    </row>
+    <row r="55" ht="18" customHeight="1"/>
+    <row r="56" ht="18" customHeight="1"/>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="22" t="inlineStr">
         <is>
@@ -3308,23 +2921,17 @@
       <c r="J57" s="1" t="n"/>
       <c r="K57" s="1" t="n"/>
       <c r="L57" s="1" t="n"/>
-      <c r="M57" s="1" t="n"/>
-      <c r="N57" s="1" t="n"/>
-      <c r="O57" s="1" t="n"/>
-      <c r="P57" s="1" t="n"/>
-      <c r="Q57" s="1" t="n"/>
-      <c r="R57" s="1" t="n"/>
-    </row>
-    <row r="58" ht="22" customHeight="1">
+    </row>
+    <row r="58" ht="26" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
           <t>Colis</t>
         </is>
       </c>
-      <c r="B58" s="34" t="n"/>
+      <c r="B58" s="32" t="n"/>
       <c r="C58" s="25" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Type de colisage</t>
         </is>
       </c>
       <c r="D58" s="25" t="inlineStr">
@@ -3334,27 +2941,32 @@
       </c>
       <c r="E58" s="25" t="inlineStr">
         <is>
-          <t>L (cm)</t>
+          <t>Longueur
+(cm)</t>
         </is>
       </c>
       <c r="F58" s="25" t="inlineStr">
         <is>
-          <t>l (cm)</t>
+          <t>Largeur
+(cm)</t>
         </is>
       </c>
       <c r="G58" s="25" t="inlineStr">
         <is>
-          <t>h (cm)</t>
+          <t>Hauteur
+(cm)</t>
         </is>
       </c>
       <c r="H58" s="25" t="inlineStr">
         <is>
-          <t>Poids (kg)</t>
+          <t>Poids
+(kg)</t>
         </is>
       </c>
       <c r="I58" s="25" t="inlineStr">
         <is>
-          <t>Volume (m³)</t>
+          <t>Volume
+(m³)</t>
         </is>
       </c>
       <c r="J58" s="25" t="inlineStr">
@@ -3362,472 +2974,400 @@
           <t>Remarques</t>
         </is>
       </c>
-      <c r="K58" s="34" t="n"/>
+      <c r="K58" s="32" t="n"/>
     </row>
     <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="35" t="inlineStr">
+      <c r="A59" s="33" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B59" s="36" t="n"/>
-      <c r="C59" s="37" t="n"/>
-      <c r="D59" s="38">
-        <f t="array" ref="D59">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A59,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E59" s="39" t="n"/>
-      <c r="F59" s="39" t="n"/>
-      <c r="G59" s="39" t="n"/>
-      <c r="H59" s="40" t="n"/>
-      <c r="I59" s="41">
+      <c r="B59" s="34" t="n"/>
+      <c r="C59" s="35" t="n"/>
+      <c r="D59" s="36">
+        <f t="array" ref="D59">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A59,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E59" s="37" t="n"/>
+      <c r="F59" s="37" t="n"/>
+      <c r="G59" s="37" t="n"/>
+      <c r="H59" s="38" t="n"/>
+      <c r="I59" s="39">
         <f>IF(COUNT(E59:G59)=3,E59*F59*G59/1000000,"")</f>
         <v/>
       </c>
-      <c r="J59" s="42" t="n"/>
-      <c r="K59" s="36" t="n"/>
+      <c r="J59" s="40" t="n"/>
+      <c r="K59" s="34" t="n"/>
     </row>
     <row r="60" ht="22" customHeight="1">
-      <c r="A60" s="35" t="inlineStr">
+      <c r="A60" s="33" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B60" s="36" t="n"/>
-      <c r="C60" s="37" t="n"/>
-      <c r="D60" s="38">
-        <f t="array" ref="D60">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A60,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E60" s="39" t="n"/>
-      <c r="F60" s="39" t="n"/>
-      <c r="G60" s="39" t="n"/>
-      <c r="H60" s="40" t="n"/>
-      <c r="I60" s="41">
+      <c r="B60" s="34" t="n"/>
+      <c r="C60" s="35" t="n"/>
+      <c r="D60" s="36">
+        <f t="array" ref="D60">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A60,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E60" s="37" t="n"/>
+      <c r="F60" s="37" t="n"/>
+      <c r="G60" s="37" t="n"/>
+      <c r="H60" s="38" t="n"/>
+      <c r="I60" s="39">
         <f>IF(COUNT(E60:G60)=3,E60*F60*G60/1000000,"")</f>
         <v/>
       </c>
-      <c r="J60" s="42" t="n"/>
-      <c r="K60" s="36" t="n"/>
+      <c r="J60" s="40" t="n"/>
+      <c r="K60" s="34" t="n"/>
     </row>
     <row r="61" ht="22" customHeight="1">
-      <c r="A61" s="35" t="inlineStr">
+      <c r="A61" s="33" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B61" s="36" t="n"/>
-      <c r="C61" s="37" t="n"/>
-      <c r="D61" s="38">
-        <f t="array" ref="D61">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A61,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E61" s="39" t="n"/>
-      <c r="F61" s="39" t="n"/>
-      <c r="G61" s="39" t="n"/>
-      <c r="H61" s="40" t="n"/>
-      <c r="I61" s="41">
+      <c r="B61" s="34" t="n"/>
+      <c r="C61" s="35" t="n"/>
+      <c r="D61" s="36">
+        <f t="array" ref="D61">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A61,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E61" s="37" t="n"/>
+      <c r="F61" s="37" t="n"/>
+      <c r="G61" s="37" t="n"/>
+      <c r="H61" s="38" t="n"/>
+      <c r="I61" s="39">
         <f>IF(COUNT(E61:G61)=3,E61*F61*G61/1000000,"")</f>
         <v/>
       </c>
-      <c r="J61" s="42" t="n"/>
-      <c r="K61" s="36" t="n"/>
+      <c r="J61" s="40" t="n"/>
+      <c r="K61" s="34" t="n"/>
     </row>
     <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="35" t="inlineStr">
+      <c r="A62" s="33" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="B62" s="36" t="n"/>
-      <c r="C62" s="37" t="n"/>
-      <c r="D62" s="38">
-        <f t="array" ref="D62">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A62,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E62" s="39" t="n"/>
-      <c r="F62" s="39" t="n"/>
-      <c r="G62" s="39" t="n"/>
-      <c r="H62" s="40" t="n"/>
-      <c r="I62" s="41">
+      <c r="B62" s="34" t="n"/>
+      <c r="C62" s="35" t="n"/>
+      <c r="D62" s="36">
+        <f t="array" ref="D62">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A62,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E62" s="37" t="n"/>
+      <c r="F62" s="37" t="n"/>
+      <c r="G62" s="37" t="n"/>
+      <c r="H62" s="38" t="n"/>
+      <c r="I62" s="39">
         <f>IF(COUNT(E62:G62)=3,E62*F62*G62/1000000,"")</f>
         <v/>
       </c>
-      <c r="J62" s="42" t="n"/>
-      <c r="K62" s="36" t="n"/>
+      <c r="J62" s="40" t="n"/>
+      <c r="K62" s="34" t="n"/>
     </row>
     <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="35" t="inlineStr">
+      <c r="A63" s="33" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="B63" s="36" t="n"/>
-      <c r="C63" s="37" t="n"/>
-      <c r="D63" s="38">
-        <f t="array" ref="D63">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A63,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E63" s="39" t="n"/>
-      <c r="F63" s="39" t="n"/>
-      <c r="G63" s="39" t="n"/>
-      <c r="H63" s="40" t="n"/>
-      <c r="I63" s="41">
+      <c r="B63" s="34" t="n"/>
+      <c r="C63" s="35" t="n"/>
+      <c r="D63" s="36">
+        <f t="array" ref="D63">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A63,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E63" s="37" t="n"/>
+      <c r="F63" s="37" t="n"/>
+      <c r="G63" s="37" t="n"/>
+      <c r="H63" s="38" t="n"/>
+      <c r="I63" s="39">
         <f>IF(COUNT(E63:G63)=3,E63*F63*G63/1000000,"")</f>
         <v/>
       </c>
-      <c r="J63" s="42" t="n"/>
-      <c r="K63" s="36" t="n"/>
+      <c r="J63" s="40" t="n"/>
+      <c r="K63" s="34" t="n"/>
     </row>
     <row r="64" ht="22" customHeight="1">
-      <c r="A64" s="35" t="inlineStr">
+      <c r="A64" s="33" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="B64" s="36" t="n"/>
-      <c r="C64" s="37" t="n"/>
-      <c r="D64" s="38">
-        <f t="array" ref="D64">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A64,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E64" s="39" t="n"/>
-      <c r="F64" s="39" t="n"/>
-      <c r="G64" s="39" t="n"/>
-      <c r="H64" s="40" t="n"/>
-      <c r="I64" s="41">
+      <c r="B64" s="34" t="n"/>
+      <c r="C64" s="35" t="n"/>
+      <c r="D64" s="36">
+        <f t="array" ref="D64">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A64,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E64" s="37" t="n"/>
+      <c r="F64" s="37" t="n"/>
+      <c r="G64" s="37" t="n"/>
+      <c r="H64" s="38" t="n"/>
+      <c r="I64" s="39">
         <f>IF(COUNT(E64:G64)=3,E64*F64*G64/1000000,"")</f>
         <v/>
       </c>
-      <c r="J64" s="42" t="n"/>
-      <c r="K64" s="36" t="n"/>
+      <c r="J64" s="40" t="n"/>
+      <c r="K64" s="34" t="n"/>
     </row>
     <row r="65" ht="22" customHeight="1">
-      <c r="A65" s="35" t="inlineStr">
+      <c r="A65" s="33" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="B65" s="36" t="n"/>
-      <c r="C65" s="37" t="n"/>
-      <c r="D65" s="38">
-        <f t="array" ref="D65">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A65,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E65" s="39" t="n"/>
-      <c r="F65" s="39" t="n"/>
-      <c r="G65" s="39" t="n"/>
-      <c r="H65" s="40" t="n"/>
-      <c r="I65" s="41">
+      <c r="B65" s="34" t="n"/>
+      <c r="C65" s="35" t="n"/>
+      <c r="D65" s="36">
+        <f t="array" ref="D65">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A65,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E65" s="37" t="n"/>
+      <c r="F65" s="37" t="n"/>
+      <c r="G65" s="37" t="n"/>
+      <c r="H65" s="38" t="n"/>
+      <c r="I65" s="39">
         <f>IF(COUNT(E65:G65)=3,E65*F65*G65/1000000,"")</f>
         <v/>
       </c>
-      <c r="J65" s="42" t="n"/>
-      <c r="K65" s="36" t="n"/>
+      <c r="J65" s="40" t="n"/>
+      <c r="K65" s="34" t="n"/>
     </row>
     <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="35" t="inlineStr">
+      <c r="A66" s="33" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="B66" s="36" t="n"/>
-      <c r="C66" s="37" t="n"/>
-      <c r="D66" s="38">
-        <f t="array" ref="D66">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A66,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E66" s="39" t="n"/>
-      <c r="F66" s="39" t="n"/>
-      <c r="G66" s="39" t="n"/>
-      <c r="H66" s="40" t="n"/>
-      <c r="I66" s="41">
+      <c r="B66" s="34" t="n"/>
+      <c r="C66" s="35" t="n"/>
+      <c r="D66" s="36">
+        <f t="array" ref="D66">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A66,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E66" s="37" t="n"/>
+      <c r="F66" s="37" t="n"/>
+      <c r="G66" s="37" t="n"/>
+      <c r="H66" s="38" t="n"/>
+      <c r="I66" s="39">
         <f>IF(COUNT(E66:G66)=3,E66*F66*G66/1000000,"")</f>
         <v/>
       </c>
-      <c r="J66" s="42" t="n"/>
-      <c r="K66" s="36" t="n"/>
+      <c r="J66" s="40" t="n"/>
+      <c r="K66" s="34" t="n"/>
     </row>
     <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="35" t="inlineStr">
+      <c r="A67" s="33" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
-      <c r="B67" s="36" t="n"/>
-      <c r="C67" s="37" t="n"/>
-      <c r="D67" s="38">
-        <f t="array" ref="D67">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A67,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E67" s="39" t="n"/>
-      <c r="F67" s="39" t="n"/>
-      <c r="G67" s="39" t="n"/>
-      <c r="H67" s="40" t="n"/>
-      <c r="I67" s="41">
+      <c r="B67" s="34" t="n"/>
+      <c r="C67" s="35" t="n"/>
+      <c r="D67" s="36">
+        <f t="array" ref="D67">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A67,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E67" s="37" t="n"/>
+      <c r="F67" s="37" t="n"/>
+      <c r="G67" s="37" t="n"/>
+      <c r="H67" s="38" t="n"/>
+      <c r="I67" s="39">
         <f>IF(COUNT(E67:G67)=3,E67*F67*G67/1000000,"")</f>
         <v/>
       </c>
-      <c r="J67" s="42" t="n"/>
-      <c r="K67" s="36" t="n"/>
+      <c r="J67" s="40" t="n"/>
+      <c r="K67" s="34" t="n"/>
     </row>
     <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="35" t="inlineStr">
+      <c r="A68" s="33" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="B68" s="36" t="n"/>
-      <c r="C68" s="37" t="n"/>
-      <c r="D68" s="38">
-        <f t="array" ref="D68">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A68,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E68" s="39" t="n"/>
-      <c r="F68" s="39" t="n"/>
-      <c r="G68" s="39" t="n"/>
-      <c r="H68" s="40" t="n"/>
-      <c r="I68" s="41">
+      <c r="B68" s="34" t="n"/>
+      <c r="C68" s="35" t="n"/>
+      <c r="D68" s="36">
+        <f t="array" ref="D68">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A68,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E68" s="37" t="n"/>
+      <c r="F68" s="37" t="n"/>
+      <c r="G68" s="37" t="n"/>
+      <c r="H68" s="38" t="n"/>
+      <c r="I68" s="39">
         <f>IF(COUNT(E68:G68)=3,E68*F68*G68/1000000,"")</f>
         <v/>
       </c>
-      <c r="J68" s="42" t="n"/>
-      <c r="K68" s="36" t="n"/>
+      <c r="J68" s="40" t="n"/>
+      <c r="K68" s="34" t="n"/>
     </row>
     <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="35" t="inlineStr">
+      <c r="A69" s="33" t="inlineStr">
         <is>
           <t>Vrac</t>
         </is>
       </c>
-      <c r="B69" s="36" t="n"/>
-      <c r="C69" s="43" t="inlineStr">
+      <c r="B69" s="34" t="n"/>
+      <c r="C69" s="41" t="inlineStr">
         <is>
           <t>Vrac</t>
         </is>
       </c>
-      <c r="D69" s="38">
-        <f t="array" ref="D69">_xlfn.TEXTJOIN(", ",TRUE,IF($O$15:$O$54=$A69,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E69" s="36" t="n"/>
-      <c r="F69" s="36" t="n"/>
-      <c r="G69" s="36" t="n"/>
-      <c r="H69" s="40" t="n"/>
-      <c r="I69" s="36" t="n"/>
-      <c r="J69" s="36" t="n"/>
-      <c r="K69" s="36" t="n"/>
+      <c r="D69" s="36">
+        <f t="array" ref="D69">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A69,$A$15:$A$54,""))</f>
+        <v/>
+      </c>
+      <c r="E69" s="34" t="n"/>
+      <c r="F69" s="34" t="n"/>
+      <c r="G69" s="34" t="n"/>
+      <c r="H69" s="38" t="n"/>
+      <c r="I69" s="34" t="n"/>
+      <c r="J69" s="34" t="n"/>
+      <c r="K69" s="34" t="n"/>
     </row>
     <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="44">
+      <c r="A70" s="42">
         <f>"TOTAL  ·  "&amp;COUNTA(C59:C68)&amp;" colis  ·  "&amp;COUNT($A$15:$A$54)&amp;" outil(s)"</f>
         <v/>
       </c>
-      <c r="B70" s="45" t="n"/>
-      <c r="C70" s="45" t="n"/>
-      <c r="D70" s="45" t="n"/>
-      <c r="E70" s="45" t="n"/>
-      <c r="F70" s="45" t="n"/>
-      <c r="G70" s="45" t="n"/>
-      <c r="H70" s="46">
+      <c r="B70" s="43" t="n"/>
+      <c r="C70" s="43" t="n"/>
+      <c r="D70" s="43" t="n"/>
+      <c r="E70" s="43" t="n"/>
+      <c r="F70" s="43" t="n"/>
+      <c r="G70" s="43" t="n"/>
+      <c r="H70" s="44">
         <f>SUM(H59:H69)</f>
         <v/>
       </c>
-      <c r="I70" s="47">
+      <c r="I70" s="45">
         <f>SUM(I59:I68)</f>
         <v/>
       </c>
-      <c r="J70" s="48" t="n"/>
-      <c r="K70" s="48" t="n"/>
-    </row>
-    <row r="72" ht="16" customHeight="1">
-      <c r="A72" s="49" t="inlineStr">
-        <is>
-          <t>PRÉPARÉ PAR · Nom, date, signature</t>
-        </is>
-      </c>
-      <c r="B72" s="50" t="n"/>
-      <c r="C72" s="50" t="n"/>
-      <c r="D72" s="51" t="n"/>
-      <c r="E72" s="49" t="inlineStr">
-        <is>
-          <t>CONTRÔLÉ PAR (superviseur) · Nom, date, signature</t>
-        </is>
-      </c>
-      <c r="F72" s="50" t="n"/>
-      <c r="G72" s="50" t="n"/>
-      <c r="H72" s="50" t="n"/>
-      <c r="I72" s="50" t="n"/>
-      <c r="J72" s="50" t="n"/>
-      <c r="K72" s="51" t="n"/>
-      <c r="L72" s="49" t="inlineStr">
-        <is>
-          <t>COLISAGE VÉRIFIÉ PAR · Nom, date</t>
-        </is>
-      </c>
-      <c r="M72" s="50" t="n"/>
-      <c r="N72" s="50" t="n"/>
-      <c r="O72" s="50" t="n"/>
-      <c r="P72" s="50" t="n"/>
-      <c r="Q72" s="50" t="n"/>
-      <c r="R72" s="51" t="n"/>
-    </row>
-    <row r="73" ht="16" customHeight="1">
-      <c r="A73" s="52" t="n"/>
-      <c r="B73" s="53" t="n"/>
-      <c r="C73" s="53" t="n"/>
-      <c r="D73" s="54" t="n"/>
-      <c r="E73" s="52" t="n"/>
-      <c r="F73" s="53" t="n"/>
-      <c r="G73" s="53" t="n"/>
-      <c r="H73" s="53" t="n"/>
-      <c r="I73" s="53" t="n"/>
-      <c r="J73" s="53" t="n"/>
-      <c r="K73" s="54" t="n"/>
-      <c r="L73" s="52" t="n"/>
-      <c r="M73" s="53" t="n"/>
-      <c r="N73" s="53" t="n"/>
-      <c r="O73" s="53" t="n"/>
-      <c r="P73" s="53" t="n"/>
-      <c r="Q73" s="53" t="n"/>
-      <c r="R73" s="54" t="n"/>
-    </row>
-    <row r="74" ht="16" customHeight="1">
-      <c r="A74" s="52" t="n"/>
-      <c r="B74" s="53" t="n"/>
-      <c r="C74" s="53" t="n"/>
-      <c r="D74" s="54" t="n"/>
-      <c r="E74" s="52" t="n"/>
-      <c r="F74" s="53" t="n"/>
-      <c r="G74" s="53" t="n"/>
-      <c r="H74" s="53" t="n"/>
-      <c r="I74" s="53" t="n"/>
-      <c r="J74" s="53" t="n"/>
-      <c r="K74" s="54" t="n"/>
-      <c r="L74" s="52" t="n"/>
-      <c r="M74" s="53" t="n"/>
-      <c r="N74" s="53" t="n"/>
-      <c r="O74" s="53" t="n"/>
-      <c r="P74" s="53" t="n"/>
-      <c r="Q74" s="53" t="n"/>
-      <c r="R74" s="54" t="n"/>
-    </row>
-    <row r="75" ht="16" customHeight="1">
-      <c r="A75" s="55" t="n"/>
-      <c r="B75" s="36" t="n"/>
-      <c r="C75" s="36" t="n"/>
-      <c r="D75" s="56" t="n"/>
-      <c r="E75" s="55" t="n"/>
-      <c r="F75" s="36" t="n"/>
-      <c r="G75" s="36" t="n"/>
-      <c r="H75" s="36" t="n"/>
-      <c r="I75" s="36" t="n"/>
-      <c r="J75" s="36" t="n"/>
-      <c r="K75" s="56" t="n"/>
-      <c r="L75" s="55" t="n"/>
-      <c r="M75" s="36" t="n"/>
-      <c r="N75" s="36" t="n"/>
-      <c r="O75" s="36" t="n"/>
-      <c r="P75" s="36" t="n"/>
-      <c r="Q75" s="36" t="n"/>
-      <c r="R75" s="56" t="n"/>
+      <c r="J70" s="46" t="n"/>
+      <c r="K70" s="46" t="n"/>
+    </row>
+    <row r="72" ht="26" customHeight="1">
+      <c r="A72" s="47" t="inlineStr">
+        <is>
+          <t>NOMBRE DE SERRAGES EFFECTUÉS</t>
+        </is>
+      </c>
+      <c r="B72" s="34" t="n"/>
+      <c r="C72" s="34" t="n"/>
+      <c r="D72" s="34" t="n"/>
+      <c r="E72" s="37" t="n"/>
+      <c r="F72" s="40" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="59">
+  <autoFilter ref="A14:V54">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="12" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="13" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="14" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="15" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="16" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="17" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="18" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="19" hiddenButton="1" showButton="0">
+      <customFilters>
+        <customFilter val="0" operator="greaterThan"/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="20" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="21" hiddenButton="1" showButton="0"/>
+  </autoFilter>
+  <mergeCells count="56">
+    <mergeCell ref="J6:L6"/>
     <mergeCell ref="J64:K64"/>
     <mergeCell ref="A64:B64"/>
     <mergeCell ref="A59:B59"/>
-    <mergeCell ref="J67:K67"/>
+    <mergeCell ref="G6:I6"/>
     <mergeCell ref="A60:B60"/>
     <mergeCell ref="A67:B67"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="L9:R9"/>
+    <mergeCell ref="J67:K67"/>
+    <mergeCell ref="A72:D72"/>
     <mergeCell ref="J59:K59"/>
-    <mergeCell ref="L6:R6"/>
     <mergeCell ref="D7:F7"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="A61:B61"/>
-    <mergeCell ref="G8:K8"/>
     <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A12:L12"/>
     <mergeCell ref="J60:K60"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A57:L57"/>
     <mergeCell ref="A69:B69"/>
+    <mergeCell ref="F1:L1"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="J68:K68"/>
-    <mergeCell ref="A55:R55"/>
-    <mergeCell ref="G7:K7"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A57:R57"/>
+    <mergeCell ref="G5:I5"/>
     <mergeCell ref="A65:B65"/>
-    <mergeCell ref="F1:R1"/>
     <mergeCell ref="A8:C8"/>
-    <mergeCell ref="G10:K10"/>
+    <mergeCell ref="E10:I10"/>
     <mergeCell ref="E13:I13"/>
-    <mergeCell ref="P13:R13"/>
     <mergeCell ref="A66:B66"/>
-    <mergeCell ref="L7:R7"/>
     <mergeCell ref="J65:K65"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="E9:I9"/>
     <mergeCell ref="D5:F5"/>
-    <mergeCell ref="L13:O13"/>
     <mergeCell ref="A70:G70"/>
-    <mergeCell ref="A9:F9"/>
     <mergeCell ref="J63:K63"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="A72:D75"/>
+    <mergeCell ref="J8:L8"/>
     <mergeCell ref="J66:K66"/>
-    <mergeCell ref="L72:R75"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A62:B62"/>
-    <mergeCell ref="L5:R5"/>
-    <mergeCell ref="L8:R8"/>
-    <mergeCell ref="A11:R11"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="A68:B68"/>
     <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="E72:F72"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
     <mergeCell ref="J62:K62"/>
-    <mergeCell ref="F2:R2"/>
-    <mergeCell ref="E72:K75"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="G8:I8"/>
     <mergeCell ref="J61:K61"/>
-    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="J9:L9"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="L10:R10"/>
-    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="A58:B58"/>
   </mergeCells>
-  <conditionalFormatting sqref="A15:R54">
+  <conditionalFormatting sqref="A15:L54">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
       <formula>$V15=1</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="2">
-      <formula>$T15&lt;&gt;""</formula>
+      <formula>$T15&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L15:L54">
-    <cfRule type="expression" priority="3" dxfId="3">
-      <formula>AND($V15=0,$L15="Oui")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="17">
+  <dataValidations count="13">
     <dataValidation sqref="I15:I54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$Q$2:$Q$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="L15:L54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$P$2:$P$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="O15:O54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$K$2:$K$12</formula1>
     </dataValidation>
     <dataValidation sqref="J15:J54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$G$2:$G$12</formula1>
     </dataValidation>
-    <dataValidation sqref="P15:P54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$G$2:$G$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="N15:N54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$A$2:$A$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="R15:R54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$A$2:$A$12</formula1>
+    <dataValidation sqref="L15:L54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
+      <formula1>=Listes!$K$2:$K$12</formula1>
     </dataValidation>
     <dataValidation sqref="C59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$J$2:$J$12</formula1>
@@ -3860,7 +3400,7 @@
       <formula1>=Listes!$J$2:$J$12</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
@@ -3870,9 +3410,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="56" min="0" max="16383" man="1"/>
-  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -3903,366 +3440,366 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="57" t="inlineStr">
+      <c r="A1" s="48" t="inlineStr">
         <is>
           <t>Contact Enedril</t>
         </is>
       </c>
-      <c r="B1" s="57" t="inlineStr">
+      <c r="B1" s="48" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="D1" s="57" t="inlineStr">
+      <c r="D1" s="48" t="inlineStr">
         <is>
           <t>Incoterm</t>
         </is>
       </c>
-      <c r="E1" s="57" t="inlineStr">
+      <c r="E1" s="48" t="inlineStr">
         <is>
           <t>Validité</t>
         </is>
       </c>
-      <c r="F1" s="57" t="inlineStr">
+      <c r="F1" s="48" t="inlineStr">
         <is>
           <t>Règlement</t>
         </is>
       </c>
-      <c r="G1" s="57" t="inlineStr">
+      <c r="G1" s="48" t="inlineStr">
         <is>
           <t>Oui / Non</t>
         </is>
       </c>
-      <c r="H1" s="58" t="n">
+      <c r="H1" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="J1" s="57" t="inlineStr">
+      <c r="J1" s="48" t="inlineStr">
         <is>
           <t>Support de colisage</t>
         </is>
       </c>
-      <c r="K1" s="57" t="inlineStr">
+      <c r="K1" s="48" t="inlineStr">
         <is>
           <t>N° de colis</t>
         </is>
       </c>
-      <c r="L1" s="57" t="inlineStr">
+      <c r="L1" s="48" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="M1" s="57" t="inlineStr">
+      <c r="M1" s="48" t="inlineStr">
         <is>
           <t>Mode transport</t>
         </is>
       </c>
-      <c r="N1" s="57" t="inlineStr">
+      <c r="N1" s="48" t="inlineStr">
         <is>
           <t>Mode forfait</t>
         </is>
       </c>
-      <c r="P1" s="57" t="inlineStr">
+      <c r="P1" s="48" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="Q1" s="57" t="inlineStr">
+      <c r="Q1" s="48" t="inlineStr">
         <is>
           <t>Test / Taille</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="59" t="inlineStr">
+      <c r="A2" s="50" t="inlineStr">
         <is>
           <t>Fabien JACQUOT</t>
         </is>
       </c>
-      <c r="B2" s="59" t="inlineStr">
+      <c r="B2" s="50" t="inlineStr">
         <is>
           <t>fjacquot@enedril.fr</t>
         </is>
       </c>
-      <c r="D2" s="59" t="inlineStr">
+      <c r="D2" s="50" t="inlineStr">
         <is>
           <t>EXW Lons</t>
         </is>
       </c>
-      <c r="E2" s="59" t="inlineStr">
+      <c r="E2" s="50" t="inlineStr">
         <is>
           <t>15 jours / 15 days</t>
         </is>
       </c>
-      <c r="F2" s="59" t="inlineStr">
+      <c r="F2" s="50" t="inlineStr">
         <is>
           <t>30 jours date de facture / 30 days invoice date</t>
         </is>
       </c>
-      <c r="G2" s="59" t="inlineStr">
+      <c r="G2" s="50" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="H2" s="60" t="inlineStr">
+      <c r="H2" s="51" t="inlineStr">
         <is>
           <t>← langue du devis : 1 = français, 2 = anglais</t>
         </is>
       </c>
-      <c r="J2" s="59" t="inlineStr">
+      <c r="J2" s="50" t="inlineStr">
         <is>
           <t>Palette</t>
         </is>
       </c>
-      <c r="K2" s="59" t="inlineStr">
+      <c r="K2" s="50" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L2" s="59" t="inlineStr">
+      <c r="L2" s="50" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="M2" s="59" t="inlineStr">
+      <c r="M2" s="50" t="inlineStr">
         <is>
           <t>Coût réel +15 %</t>
         </is>
       </c>
-      <c r="N2" s="59" t="inlineStr">
+      <c r="N2" s="50" t="inlineStr">
         <is>
           <t>Forfait calculé (S + O + UC)</t>
         </is>
       </c>
-      <c r="P2" s="59" t="inlineStr">
+      <c r="P2" s="50" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="Q2" s="59" t="inlineStr">
+      <c r="Q2" s="50" t="inlineStr">
         <is>
           <t>Taille OK</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="50" t="inlineStr">
         <is>
           <t>Alexis ESTINES</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="50" t="inlineStr">
         <is>
           <t>aestines@enedril.fr</t>
         </is>
       </c>
-      <c r="D3" s="59" t="inlineStr">
+      <c r="D3" s="50" t="inlineStr">
         <is>
           <t>FCA Lons</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr">
+      <c r="E3" s="50" t="inlineStr">
         <is>
           <t>30 jours / 30 days</t>
         </is>
       </c>
-      <c r="F3" s="59" t="inlineStr">
+      <c r="F3" s="50" t="inlineStr">
         <is>
           <t>30 jours fin de mois / 30 days end of month</t>
         </is>
       </c>
-      <c r="G3" s="59" t="inlineStr">
+      <c r="G3" s="50" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="J3" s="59" t="inlineStr">
+      <c r="J3" s="50" t="inlineStr">
         <is>
           <t>Fishing basket</t>
         </is>
       </c>
-      <c r="K3" s="59" t="inlineStr">
+      <c r="K3" s="50" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="L3" s="59" t="inlineStr">
+      <c r="L3" s="50" t="inlineStr">
         <is>
           <t>€/jour</t>
         </is>
       </c>
-      <c r="M3" s="59" t="inlineStr">
+      <c r="M3" s="50" t="inlineStr">
         <is>
           <t>Forfait</t>
         </is>
       </c>
-      <c r="N3" s="59" t="inlineStr">
+      <c r="N3" s="50" t="inlineStr">
         <is>
           <t>Forfait global</t>
         </is>
       </c>
-      <c r="P3" s="59" t="inlineStr">
+      <c r="P3" s="50" t="inlineStr">
         <is>
           <t>En cours</t>
         </is>
       </c>
-      <c r="Q3" s="59" t="inlineStr">
+      <c r="Q3" s="50" t="inlineStr">
         <is>
           <t>Test OK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Paul HYNDERICK</t>
         </is>
       </c>
-      <c r="B4" s="59" t="inlineStr">
+      <c r="B4" s="50" t="inlineStr">
         <is>
           <t>phynderick@enedril.fr</t>
         </is>
       </c>
-      <c r="D4" s="59" t="inlineStr">
+      <c r="D4" s="50" t="inlineStr">
         <is>
           <t>DAP</t>
         </is>
       </c>
-      <c r="E4" s="59" t="inlineStr">
+      <c r="E4" s="50" t="inlineStr">
         <is>
           <t>60 jours / 60 days</t>
         </is>
       </c>
-      <c r="F4" s="59" t="inlineStr">
+      <c r="F4" s="50" t="inlineStr">
         <is>
           <t>45 jours fin de mois / 45 days end of month</t>
         </is>
       </c>
-      <c r="J4" s="59" t="inlineStr">
+      <c r="J4" s="50" t="inlineStr">
         <is>
           <t>Caisse</t>
         </is>
       </c>
-      <c r="K4" s="59" t="inlineStr">
+      <c r="K4" s="50" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="L4" s="59" t="inlineStr">
+      <c r="L4" s="50" t="inlineStr">
         <is>
           <t>€/jour/pers</t>
         </is>
       </c>
-      <c r="N4" s="59" t="inlineStr">
+      <c r="N4" s="50" t="inlineStr">
         <is>
           <t>Forfait par jour</t>
         </is>
       </c>
-      <c r="Q4" s="59" t="inlineStr">
+      <c r="Q4" s="50" t="inlineStr">
         <is>
           <t>Taille + test OK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="50" t="inlineStr">
         <is>
           <t>Céline CARDONA</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="50" t="inlineStr">
         <is>
           <t>ccardona@enedril.fr</t>
         </is>
       </c>
-      <c r="D5" s="59" t="inlineStr">
+      <c r="D5" s="50" t="inlineStr">
         <is>
           <t>DDP</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr">
+      <c r="E5" s="50" t="inlineStr">
         <is>
           <t>90 jours / 90 days</t>
         </is>
       </c>
-      <c r="F5" s="59" t="inlineStr">
+      <c r="F5" s="50" t="inlineStr">
         <is>
           <t>À la commande / Upon order</t>
         </is>
       </c>
-      <c r="J5" s="59" t="inlineStr">
+      <c r="J5" s="50" t="inlineStr">
         <is>
           <t>Vrac</t>
         </is>
       </c>
-      <c r="K5" s="59" t="inlineStr">
+      <c r="K5" s="50" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="L5" s="59" t="inlineStr">
+      <c r="L5" s="50" t="inlineStr">
         <is>
           <t>€/pers</t>
         </is>
       </c>
-      <c r="Q5" s="59" t="inlineStr">
+      <c r="Q5" s="50" t="inlineStr">
         <is>
           <t>À contrôler</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="50" t="inlineStr">
         <is>
           <t>Koen MONDELAERS</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="50" t="inlineStr">
         <is>
           <t>kmondelaers@enedril.fr</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="50" t="inlineStr">
         <is>
           <t>FOB</t>
         </is>
       </c>
-      <c r="K6" s="59" t="inlineStr">
+      <c r="K6" s="50" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="L6" s="59" t="inlineStr">
+      <c r="L6" s="50" t="inlineStr">
         <is>
           <t>€/unité</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr">
         <is>
           <t>Luigi LIBERATORE</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>lliberatore@enedril.fr</t>
         </is>
       </c>
-      <c r="K7" s="59" t="inlineStr">
+      <c r="K7" s="50" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="K8" s="59" t="inlineStr">
+      <c r="K8" s="50" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="K9" s="59" t="inlineStr">
+      <c r="K9" s="50" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
@@ -4274,21 +3811,21 @@
           <t>Pour ajouter un contact, une validité, etc. : écrire à la suite dans la colonne (les listes déroulantes lisent les 12 premières lignes).</t>
         </is>
       </c>
-      <c r="K10" s="59" t="inlineStr">
+      <c r="K10" s="50" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="K11" s="59" t="inlineStr">
+      <c r="K11" s="50" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="K12" s="59" t="inlineStr">
+      <c r="K12" s="50" t="inlineStr">
         <is>
           <t>Vrac</t>
         </is>

</xml_diff>

<commit_message>
Tool list : colisage compacté sur une page
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Tool_List_Enedril_2027.xlsx
+++ b/devis_2027/Tool_List_Enedril_2027.xlsx
@@ -2976,7 +2976,7 @@
       </c>
       <c r="K58" s="32" t="n"/>
     </row>
-    <row r="59" ht="22" customHeight="1">
+    <row r="59" ht="17" customHeight="1">
       <c r="A59" s="33" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2999,7 +2999,7 @@
       <c r="J59" s="40" t="n"/>
       <c r="K59" s="34" t="n"/>
     </row>
-    <row r="60" ht="22" customHeight="1">
+    <row r="60" ht="17" customHeight="1">
       <c r="A60" s="33" t="inlineStr">
         <is>
           <t>P2</t>
@@ -3022,7 +3022,7 @@
       <c r="J60" s="40" t="n"/>
       <c r="K60" s="34" t="n"/>
     </row>
-    <row r="61" ht="22" customHeight="1">
+    <row r="61" ht="17" customHeight="1">
       <c r="A61" s="33" t="inlineStr">
         <is>
           <t>P3</t>
@@ -3045,7 +3045,7 @@
       <c r="J61" s="40" t="n"/>
       <c r="K61" s="34" t="n"/>
     </row>
-    <row r="62" ht="22" customHeight="1">
+    <row r="62" ht="17" customHeight="1">
       <c r="A62" s="33" t="inlineStr">
         <is>
           <t>P4</t>
@@ -3068,7 +3068,7 @@
       <c r="J62" s="40" t="n"/>
       <c r="K62" s="34" t="n"/>
     </row>
-    <row r="63" ht="22" customHeight="1">
+    <row r="63" ht="17" customHeight="1">
       <c r="A63" s="33" t="inlineStr">
         <is>
           <t>P5</t>
@@ -3091,7 +3091,7 @@
       <c r="J63" s="40" t="n"/>
       <c r="K63" s="34" t="n"/>
     </row>
-    <row r="64" ht="22" customHeight="1">
+    <row r="64" ht="17" customHeight="1">
       <c r="A64" s="33" t="inlineStr">
         <is>
           <t>P6</t>
@@ -3114,7 +3114,7 @@
       <c r="J64" s="40" t="n"/>
       <c r="K64" s="34" t="n"/>
     </row>
-    <row r="65" ht="22" customHeight="1">
+    <row r="65" ht="17" customHeight="1">
       <c r="A65" s="33" t="inlineStr">
         <is>
           <t>P7</t>
@@ -3137,7 +3137,7 @@
       <c r="J65" s="40" t="n"/>
       <c r="K65" s="34" t="n"/>
     </row>
-    <row r="66" ht="22" customHeight="1">
+    <row r="66" ht="17" customHeight="1">
       <c r="A66" s="33" t="inlineStr">
         <is>
           <t>P8</t>
@@ -3160,7 +3160,7 @@
       <c r="J66" s="40" t="n"/>
       <c r="K66" s="34" t="n"/>
     </row>
-    <row r="67" ht="22" customHeight="1">
+    <row r="67" ht="17" customHeight="1">
       <c r="A67" s="33" t="inlineStr">
         <is>
           <t>P9</t>
@@ -3183,7 +3183,7 @@
       <c r="J67" s="40" t="n"/>
       <c r="K67" s="34" t="n"/>
     </row>
-    <row r="68" ht="22" customHeight="1">
+    <row r="68" ht="17" customHeight="1">
       <c r="A68" s="33" t="inlineStr">
         <is>
           <t>P10</t>
@@ -3206,7 +3206,7 @@
       <c r="J68" s="40" t="n"/>
       <c r="K68" s="34" t="n"/>
     </row>
-    <row r="69" ht="22" customHeight="1">
+    <row r="69" ht="17" customHeight="1">
       <c r="A69" s="33" t="inlineStr">
         <is>
           <t>Vrac</t>
@@ -3230,7 +3230,7 @@
       <c r="J69" s="34" t="n"/>
       <c r="K69" s="34" t="n"/>
     </row>
-    <row r="70" ht="22" customHeight="1">
+    <row r="70" ht="20" customHeight="1">
       <c r="A70" s="42">
         <f>"TOTAL  ·  "&amp;COUNTA(C59:C68)&amp;" colis  ·  "&amp;COUNT($A$15:$A$54)&amp;" outil(s)"</f>
         <v/>
@@ -3252,7 +3252,7 @@
       <c r="J70" s="46" t="n"/>
       <c r="K70" s="46" t="n"/>
     </row>
-    <row r="72" ht="26" customHeight="1">
+    <row r="72" ht="22" customHeight="1">
       <c r="A72" s="47" t="inlineStr">
         <is>
           <t>NOMBRE DE SERRAGES EFFECTUÉS</t>

</xml_diff>

<commit_message>
Tool list : texte plus gros, sans n° de série ni stock ni colis par item, serrages au-dessus du colisage global
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Tool_List_Enedril_2027.xlsx
+++ b/devis_2027/Tool_List_Enedril_2027.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Tool List'!$A$14:$V$54</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'2 Tool List'!$A$1:$L$72</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'2 Tool List'!$A$1:$I$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="#,##0.0 &quot;kg&quot;"/>
     <numFmt numFmtId="169" formatCode="0.000 &quot;m³&quot;"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,42 +102,42 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="17"/>
+      <sz val="20"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="009FD8F5"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0051647A"/>
-      <sz val="7.5"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000A4FA0"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00E2231A"/>
       <sz val="10.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00E2231A"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="8.5"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0008203F"/>
-      <sz val="8"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -151,30 +151,60 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0051647A"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="000B1B2E"/>
-      <sz val="9.5"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="000A4FA0"/>
-      <sz val="9.5"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00E2231A"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0008203F"/>
-      <sz val="10"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="0051647A"/>
-      <sz val="9.5"/>
+      <b val="1"/>
+      <color rgb="000A4FA0"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0008203F"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000B1B2E"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000A4FA0"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="8">
@@ -236,23 +266,19 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00D5DEE8"/>
+        <color rgb="00B7DDF2"/>
       </bottom>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
-        <color rgb="0000AEEF"/>
+        <color rgb="00D5DEE8"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -307,6 +333,9 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -318,62 +347,66 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="26" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -505,7 +538,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1333500" cy="304800"/>
+    <ext cx="1428750" cy="323850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1335,43 +1368,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V72"/>
+  <dimension ref="A1:V67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5.5" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>LISTE DE MATÉRIEL</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="1" t="n"/>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="16">
-        <f>"N° "&amp;G8&amp;IF(G6="","","   ·   "&amp;G6)</f>
+      <c r="E2" s="16">
+        <f>"N° "&amp;D8&amp;IF(D6="","","   ·   "&amp;D6)</f>
         <v/>
       </c>
     </row>
@@ -1385,1884 +1413,1572 @@
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4" ht="8" customHeight="1"/>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>CLIENT</t>
         </is>
       </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>PUITS / CHANTIER</t>
+        </is>
+      </c>
       <c r="D5" s="17" t="inlineStr">
         <is>
-          <t>PUITS / CHANTIER</t>
-        </is>
-      </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
           <t>DOSSIER N° · RIG</t>
         </is>
       </c>
-      <c r="J5" s="17" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>DESTINATION</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="21" customHeight="1">
+    <row r="6" ht="26" customHeight="1">
       <c r="A6" s="18" t="n"/>
       <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
+      <c r="C6" s="18" t="n"/>
       <c r="D6" s="18" t="n"/>
       <c r="E6" s="19" t="n"/>
       <c r="F6" s="19" t="n"/>
-      <c r="G6" s="18" t="n"/>
-      <c r="H6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
+      <c r="H6" s="18" t="n"/>
       <c r="I6" s="19" t="n"/>
-      <c r="J6" s="18" t="n"/>
-      <c r="K6" s="19" t="n"/>
-      <c r="L6" s="19" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+    </row>
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>DATE DE DÉPART</t>
         </is>
       </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>FAITE LE</t>
+        </is>
+      </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>FAITE LE</t>
-        </is>
-      </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
           <t>N° DE LISTE</t>
         </is>
       </c>
-      <c r="J7" s="17" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>PRÉPARÉE PAR</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="21" customHeight="1">
+    <row r="8" ht="26" customHeight="1">
       <c r="A8" s="20" t="n"/>
       <c r="B8" s="19" t="n"/>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="20" t="n"/>
+      <c r="C8" s="20" t="n"/>
+      <c r="D8" s="18" t="n"/>
       <c r="E8" s="19" t="n"/>
       <c r="F8" s="19" t="n"/>
-      <c r="G8" s="18" t="n"/>
-      <c r="H8" s="19" t="n"/>
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="18" t="n"/>
       <c r="I8" s="19" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="19" t="n"/>
-      <c r="L8" s="19" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+    </row>
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>DESCRIPTION GÉNÉRALE</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>COLISAGE</t>
         </is>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>VALIDÉE PAR</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="21" customHeight="1">
+    <row r="10" ht="26" customHeight="1">
       <c r="A10" s="18" t="n"/>
       <c r="B10" s="19" t="n"/>
       <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>A communiquer dès que possible</t>
         </is>
       </c>
+      <c r="E10" s="19" t="n"/>
       <c r="F10" s="19" t="n"/>
       <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
+      <c r="H10" s="18" t="n"/>
       <c r="I10" s="19" t="n"/>
-      <c r="J10" s="18" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="19" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Toute modification par rapport à la liste ci-dessous doit être évitée, et impérativement signalée si pas le choix.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="14" customHeight="1">
-      <c r="A12" s="21">
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="22">
         <f>IF(SUBTOTAL(103,A15:A54)&lt;MIN(SUM('1 Matériel'!$E$6:$E$29),40),"⚠  Appuyer sur Ctrl + Alt + L pour afficher toutes les lignes de la liste.","")</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>ÉQUIPEMENT</t>
         </is>
       </c>
       <c r="B13" s="1" t="n"/>
       <c r="C13" s="1" t="n"/>
-      <c r="D13" s="1" t="n"/>
-      <c r="E13" s="23" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>RELEVÉS (pouces)</t>
         </is>
       </c>
-      <c r="F13" s="24" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="24" t="n"/>
-      <c r="I13" s="24" t="n"/>
-      <c r="J13" s="22" t="inlineStr">
-        <is>
-          <t>STOCK ET REMARQUES</t>
-        </is>
-      </c>
-      <c r="K13" s="1" t="n"/>
-      <c r="L13" s="23" t="inlineStr">
-        <is>
-          <t>COLIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>REMARQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B14" s="25" t="inlineStr">
-        <is>
-          <t>Référence
-(PL)</t>
-        </is>
-      </c>
-      <c r="C14" s="25" t="inlineStr">
-        <is>
-          <t>N° de série</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Référence / N° de série
+(à écrire)</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E14" s="25" t="inlineStr">
+      <c r="D14" s="26" t="inlineStr">
         <is>
           <t>OD</t>
         </is>
       </c>
-      <c r="F14" s="25" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="G14" s="25" t="inlineStr">
+      <c r="F14" s="26" t="inlineStr">
         <is>
           <t>Ouverture
 blades</t>
         </is>
       </c>
-      <c r="H14" s="25" t="inlineStr">
+      <c r="G14" s="26" t="inlineStr">
         <is>
           <t>Ouverture max
 couteaux</t>
         </is>
       </c>
-      <c r="I14" s="25" t="inlineStr">
+      <c r="H14" s="26" t="inlineStr">
         <is>
           <t>Taille / test
 confirmé</t>
         </is>
       </c>
-      <c r="J14" s="25" t="inlineStr">
-        <is>
-          <t>Stock
-@CC</t>
-        </is>
-      </c>
-      <c r="K14" s="25" t="inlineStr">
+      <c r="I14" s="26" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
       </c>
-      <c r="L14" s="25" t="inlineStr">
-        <is>
-          <t>N° colis</t>
-        </is>
-      </c>
-      <c r="T14" s="26" t="inlineStr">
+      <c r="T14" s="27" t="inlineStr">
         <is>
           <t>ligne</t>
         </is>
       </c>
-      <c r="U14" s="26" t="inlineStr">
+      <c r="U14" s="27" t="inlineStr">
         <is>
           <t>réf.</t>
         </is>
       </c>
-      <c r="V14" s="26" t="inlineStr">
+      <c r="V14" s="27" t="inlineStr">
         <is>
           <t>bannière</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="27" customHeight="1">
-      <c r="A15" s="7">
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="28">
         <f>IF(OR(T15=0,V15=1),"",T15-COUNTIF(V$15:V15,1))</f>
         <v/>
       </c>
-      <c r="B15" s="27" t="n"/>
-      <c r="C15" s="27" t="n"/>
-      <c r="D15" s="28">
+      <c r="B15" s="29" t="n"/>
+      <c r="C15" s="30">
         <f>IF(T15=0,"",IF(V15=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U15)),INDEX('1 Matériel'!$C$6:$C$29,U15)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U15)&gt;1,"  ("&amp;(T15-INDEX('1 Matériel'!$F$6:$F$29,U15)+INDEX('1 Matériel'!$E$6:$E$29,U15))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U15)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E15" s="29" t="n"/>
-      <c r="F15" s="29" t="n"/>
-      <c r="G15" s="29" t="n"/>
-      <c r="H15" s="29" t="n"/>
-      <c r="I15" s="30" t="n"/>
-      <c r="J15" s="30" t="n"/>
-      <c r="K15" s="27" t="n"/>
-      <c r="L15" s="30" t="n"/>
-      <c r="T15" s="31">
+      <c r="D15" s="31" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="31" t="n"/>
+      <c r="H15" s="32" t="n"/>
+      <c r="I15" s="29" t="n"/>
+      <c r="T15" s="33">
         <f>IF(1&lt;=SUM('1 Matériel'!$E$6:$E$29),1,0)</f>
         <v/>
       </c>
-      <c r="U15" s="31">
+      <c r="U15" s="33">
         <f>IF(T15=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T15)+1)</f>
         <v/>
       </c>
-      <c r="V15" s="31">
+      <c r="V15" s="33">
         <f>IF(U15="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U15)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="7">
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="28">
         <f>IF(OR(T16=0,V16=1),"",T16-COUNTIF(V$15:V16,1))</f>
         <v/>
       </c>
-      <c r="B16" s="27" t="n"/>
-      <c r="C16" s="27" t="n"/>
-      <c r="D16" s="28">
+      <c r="B16" s="29" t="n"/>
+      <c r="C16" s="30">
         <f>IF(T16=0,"",IF(V16=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U16)),INDEX('1 Matériel'!$C$6:$C$29,U16)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U16)&gt;1,"  ("&amp;(T16-INDEX('1 Matériel'!$F$6:$F$29,U16)+INDEX('1 Matériel'!$E$6:$E$29,U16))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U16)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E16" s="29" t="n"/>
-      <c r="F16" s="29" t="n"/>
-      <c r="G16" s="29" t="n"/>
-      <c r="H16" s="29" t="n"/>
-      <c r="I16" s="30" t="n"/>
-      <c r="J16" s="30" t="n"/>
-      <c r="K16" s="27" t="n"/>
-      <c r="L16" s="30" t="n"/>
-      <c r="T16" s="31">
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
+      <c r="H16" s="32" t="n"/>
+      <c r="I16" s="29" t="n"/>
+      <c r="T16" s="33">
         <f>IF(2&lt;=SUM('1 Matériel'!$E$6:$E$29),2,0)</f>
         <v/>
       </c>
-      <c r="U16" s="31">
+      <c r="U16" s="33">
         <f>IF(T16=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T16)+1)</f>
         <v/>
       </c>
-      <c r="V16" s="31">
+      <c r="V16" s="33">
         <f>IF(U16="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U16)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="7">
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="28">
         <f>IF(OR(T17=0,V17=1),"",T17-COUNTIF(V$15:V17,1))</f>
         <v/>
       </c>
-      <c r="B17" s="27" t="n"/>
-      <c r="C17" s="27" t="n"/>
-      <c r="D17" s="28">
+      <c r="B17" s="29" t="n"/>
+      <c r="C17" s="30">
         <f>IF(T17=0,"",IF(V17=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U17)),INDEX('1 Matériel'!$C$6:$C$29,U17)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U17)&gt;1,"  ("&amp;(T17-INDEX('1 Matériel'!$F$6:$F$29,U17)+INDEX('1 Matériel'!$E$6:$E$29,U17))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U17)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E17" s="29" t="n"/>
-      <c r="F17" s="29" t="n"/>
-      <c r="G17" s="29" t="n"/>
-      <c r="H17" s="29" t="n"/>
-      <c r="I17" s="30" t="n"/>
-      <c r="J17" s="30" t="n"/>
-      <c r="K17" s="27" t="n"/>
-      <c r="L17" s="30" t="n"/>
-      <c r="T17" s="31">
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="32" t="n"/>
+      <c r="I17" s="29" t="n"/>
+      <c r="T17" s="33">
         <f>IF(3&lt;=SUM('1 Matériel'!$E$6:$E$29),3,0)</f>
         <v/>
       </c>
-      <c r="U17" s="31">
+      <c r="U17" s="33">
         <f>IF(T17=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T17)+1)</f>
         <v/>
       </c>
-      <c r="V17" s="31">
+      <c r="V17" s="33">
         <f>IF(U17="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U17)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="7">
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="28">
         <f>IF(OR(T18=0,V18=1),"",T18-COUNTIF(V$15:V18,1))</f>
         <v/>
       </c>
-      <c r="B18" s="27" t="n"/>
-      <c r="C18" s="27" t="n"/>
-      <c r="D18" s="28">
+      <c r="B18" s="29" t="n"/>
+      <c r="C18" s="30">
         <f>IF(T18=0,"",IF(V18=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U18)),INDEX('1 Matériel'!$C$6:$C$29,U18)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U18)&gt;1,"  ("&amp;(T18-INDEX('1 Matériel'!$F$6:$F$29,U18)+INDEX('1 Matériel'!$E$6:$E$29,U18))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U18)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E18" s="29" t="n"/>
-      <c r="F18" s="29" t="n"/>
-      <c r="G18" s="29" t="n"/>
-      <c r="H18" s="29" t="n"/>
-      <c r="I18" s="30" t="n"/>
-      <c r="J18" s="30" t="n"/>
-      <c r="K18" s="27" t="n"/>
-      <c r="L18" s="30" t="n"/>
-      <c r="T18" s="31">
+      <c r="D18" s="31" t="n"/>
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="31" t="n"/>
+      <c r="G18" s="31" t="n"/>
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="29" t="n"/>
+      <c r="T18" s="33">
         <f>IF(4&lt;=SUM('1 Matériel'!$E$6:$E$29),4,0)</f>
         <v/>
       </c>
-      <c r="U18" s="31">
+      <c r="U18" s="33">
         <f>IF(T18=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T18)+1)</f>
         <v/>
       </c>
-      <c r="V18" s="31">
+      <c r="V18" s="33">
         <f>IF(U18="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U18)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="7">
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="28">
         <f>IF(OR(T19=0,V19=1),"",T19-COUNTIF(V$15:V19,1))</f>
         <v/>
       </c>
-      <c r="B19" s="27" t="n"/>
-      <c r="C19" s="27" t="n"/>
-      <c r="D19" s="28">
+      <c r="B19" s="29" t="n"/>
+      <c r="C19" s="30">
         <f>IF(T19=0,"",IF(V19=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U19)),INDEX('1 Matériel'!$C$6:$C$29,U19)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U19)&gt;1,"  ("&amp;(T19-INDEX('1 Matériel'!$F$6:$F$29,U19)+INDEX('1 Matériel'!$E$6:$E$29,U19))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U19)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E19" s="29" t="n"/>
-      <c r="F19" s="29" t="n"/>
-      <c r="G19" s="29" t="n"/>
-      <c r="H19" s="29" t="n"/>
-      <c r="I19" s="30" t="n"/>
-      <c r="J19" s="30" t="n"/>
-      <c r="K19" s="27" t="n"/>
-      <c r="L19" s="30" t="n"/>
-      <c r="T19" s="31">
+      <c r="D19" s="31" t="n"/>
+      <c r="E19" s="31" t="n"/>
+      <c r="F19" s="31" t="n"/>
+      <c r="G19" s="31" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="29" t="n"/>
+      <c r="T19" s="33">
         <f>IF(5&lt;=SUM('1 Matériel'!$E$6:$E$29),5,0)</f>
         <v/>
       </c>
-      <c r="U19" s="31">
+      <c r="U19" s="33">
         <f>IF(T19=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T19)+1)</f>
         <v/>
       </c>
-      <c r="V19" s="31">
+      <c r="V19" s="33">
         <f>IF(U19="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U19)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="20" hidden="1" ht="27" customHeight="1">
-      <c r="A20" s="7">
+    <row r="20" hidden="1" ht="40" customHeight="1">
+      <c r="A20" s="28">
         <f>IF(OR(T20=0,V20=1),"",T20-COUNTIF(V$15:V20,1))</f>
         <v/>
       </c>
-      <c r="B20" s="27" t="n"/>
-      <c r="C20" s="27" t="n"/>
-      <c r="D20" s="28">
+      <c r="B20" s="29" t="n"/>
+      <c r="C20" s="30">
         <f>IF(T20=0,"",IF(V20=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U20)),INDEX('1 Matériel'!$C$6:$C$29,U20)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U20)&gt;1,"  ("&amp;(T20-INDEX('1 Matériel'!$F$6:$F$29,U20)+INDEX('1 Matériel'!$E$6:$E$29,U20))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U20)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E20" s="29" t="n"/>
-      <c r="F20" s="29" t="n"/>
-      <c r="G20" s="29" t="n"/>
-      <c r="H20" s="29" t="n"/>
-      <c r="I20" s="30" t="n"/>
-      <c r="J20" s="30" t="n"/>
-      <c r="K20" s="27" t="n"/>
-      <c r="L20" s="30" t="n"/>
-      <c r="T20" s="31">
+      <c r="D20" s="31" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="31" t="n"/>
+      <c r="G20" s="31" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="29" t="n"/>
+      <c r="T20" s="33">
         <f>IF(6&lt;=SUM('1 Matériel'!$E$6:$E$29),6,0)</f>
         <v/>
       </c>
-      <c r="U20" s="31">
+      <c r="U20" s="33">
         <f>IF(T20=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T20)+1)</f>
         <v/>
       </c>
-      <c r="V20" s="31">
+      <c r="V20" s="33">
         <f>IF(U20="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U20)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="21" hidden="1" ht="27" customHeight="1">
-      <c r="A21" s="7">
+    <row r="21" hidden="1" ht="40" customHeight="1">
+      <c r="A21" s="28">
         <f>IF(OR(T21=0,V21=1),"",T21-COUNTIF(V$15:V21,1))</f>
         <v/>
       </c>
-      <c r="B21" s="27" t="n"/>
-      <c r="C21" s="27" t="n"/>
-      <c r="D21" s="28">
+      <c r="B21" s="29" t="n"/>
+      <c r="C21" s="30">
         <f>IF(T21=0,"",IF(V21=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U21)),INDEX('1 Matériel'!$C$6:$C$29,U21)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U21)&gt;1,"  ("&amp;(T21-INDEX('1 Matériel'!$F$6:$F$29,U21)+INDEX('1 Matériel'!$E$6:$E$29,U21))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U21)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E21" s="29" t="n"/>
-      <c r="F21" s="29" t="n"/>
-      <c r="G21" s="29" t="n"/>
-      <c r="H21" s="29" t="n"/>
-      <c r="I21" s="30" t="n"/>
-      <c r="J21" s="30" t="n"/>
-      <c r="K21" s="27" t="n"/>
-      <c r="L21" s="30" t="n"/>
-      <c r="T21" s="31">
+      <c r="D21" s="31" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="31" t="n"/>
+      <c r="G21" s="31" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="29" t="n"/>
+      <c r="T21" s="33">
         <f>IF(7&lt;=SUM('1 Matériel'!$E$6:$E$29),7,0)</f>
         <v/>
       </c>
-      <c r="U21" s="31">
+      <c r="U21" s="33">
         <f>IF(T21=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T21)+1)</f>
         <v/>
       </c>
-      <c r="V21" s="31">
+      <c r="V21" s="33">
         <f>IF(U21="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U21)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="22" hidden="1" ht="27" customHeight="1">
-      <c r="A22" s="7">
+    <row r="22" hidden="1" ht="40" customHeight="1">
+      <c r="A22" s="28">
         <f>IF(OR(T22=0,V22=1),"",T22-COUNTIF(V$15:V22,1))</f>
         <v/>
       </c>
-      <c r="B22" s="27" t="n"/>
-      <c r="C22" s="27" t="n"/>
-      <c r="D22" s="28">
+      <c r="B22" s="29" t="n"/>
+      <c r="C22" s="30">
         <f>IF(T22=0,"",IF(V22=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U22)),INDEX('1 Matériel'!$C$6:$C$29,U22)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U22)&gt;1,"  ("&amp;(T22-INDEX('1 Matériel'!$F$6:$F$29,U22)+INDEX('1 Matériel'!$E$6:$E$29,U22))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U22)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E22" s="29" t="n"/>
-      <c r="F22" s="29" t="n"/>
-      <c r="G22" s="29" t="n"/>
-      <c r="H22" s="29" t="n"/>
-      <c r="I22" s="30" t="n"/>
-      <c r="J22" s="30" t="n"/>
-      <c r="K22" s="27" t="n"/>
-      <c r="L22" s="30" t="n"/>
-      <c r="T22" s="31">
+      <c r="D22" s="31" t="n"/>
+      <c r="E22" s="31" t="n"/>
+      <c r="F22" s="31" t="n"/>
+      <c r="G22" s="31" t="n"/>
+      <c r="H22" s="32" t="n"/>
+      <c r="I22" s="29" t="n"/>
+      <c r="T22" s="33">
         <f>IF(8&lt;=SUM('1 Matériel'!$E$6:$E$29),8,0)</f>
         <v/>
       </c>
-      <c r="U22" s="31">
+      <c r="U22" s="33">
         <f>IF(T22=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T22)+1)</f>
         <v/>
       </c>
-      <c r="V22" s="31">
+      <c r="V22" s="33">
         <f>IF(U22="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U22)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="23" hidden="1" ht="27" customHeight="1">
-      <c r="A23" s="7">
+    <row r="23" hidden="1" ht="40" customHeight="1">
+      <c r="A23" s="28">
         <f>IF(OR(T23=0,V23=1),"",T23-COUNTIF(V$15:V23,1))</f>
         <v/>
       </c>
-      <c r="B23" s="27" t="n"/>
-      <c r="C23" s="27" t="n"/>
-      <c r="D23" s="28">
+      <c r="B23" s="29" t="n"/>
+      <c r="C23" s="30">
         <f>IF(T23=0,"",IF(V23=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U23)),INDEX('1 Matériel'!$C$6:$C$29,U23)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U23)&gt;1,"  ("&amp;(T23-INDEX('1 Matériel'!$F$6:$F$29,U23)+INDEX('1 Matériel'!$E$6:$E$29,U23))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U23)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E23" s="29" t="n"/>
-      <c r="F23" s="29" t="n"/>
-      <c r="G23" s="29" t="n"/>
-      <c r="H23" s="29" t="n"/>
-      <c r="I23" s="30" t="n"/>
-      <c r="J23" s="30" t="n"/>
-      <c r="K23" s="27" t="n"/>
-      <c r="L23" s="30" t="n"/>
-      <c r="T23" s="31">
+      <c r="D23" s="31" t="n"/>
+      <c r="E23" s="31" t="n"/>
+      <c r="F23" s="31" t="n"/>
+      <c r="G23" s="31" t="n"/>
+      <c r="H23" s="32" t="n"/>
+      <c r="I23" s="29" t="n"/>
+      <c r="T23" s="33">
         <f>IF(9&lt;=SUM('1 Matériel'!$E$6:$E$29),9,0)</f>
         <v/>
       </c>
-      <c r="U23" s="31">
+      <c r="U23" s="33">
         <f>IF(T23=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T23)+1)</f>
         <v/>
       </c>
-      <c r="V23" s="31">
+      <c r="V23" s="33">
         <f>IF(U23="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U23)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="24" hidden="1" ht="27" customHeight="1">
-      <c r="A24" s="7">
+    <row r="24" hidden="1" ht="40" customHeight="1">
+      <c r="A24" s="28">
         <f>IF(OR(T24=0,V24=1),"",T24-COUNTIF(V$15:V24,1))</f>
         <v/>
       </c>
-      <c r="B24" s="27" t="n"/>
-      <c r="C24" s="27" t="n"/>
-      <c r="D24" s="28">
+      <c r="B24" s="29" t="n"/>
+      <c r="C24" s="30">
         <f>IF(T24=0,"",IF(V24=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U24)),INDEX('1 Matériel'!$C$6:$C$29,U24)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U24)&gt;1,"  ("&amp;(T24-INDEX('1 Matériel'!$F$6:$F$29,U24)+INDEX('1 Matériel'!$E$6:$E$29,U24))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U24)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E24" s="29" t="n"/>
-      <c r="F24" s="29" t="n"/>
-      <c r="G24" s="29" t="n"/>
-      <c r="H24" s="29" t="n"/>
-      <c r="I24" s="30" t="n"/>
-      <c r="J24" s="30" t="n"/>
-      <c r="K24" s="27" t="n"/>
-      <c r="L24" s="30" t="n"/>
-      <c r="T24" s="31">
+      <c r="D24" s="31" t="n"/>
+      <c r="E24" s="31" t="n"/>
+      <c r="F24" s="31" t="n"/>
+      <c r="G24" s="31" t="n"/>
+      <c r="H24" s="32" t="n"/>
+      <c r="I24" s="29" t="n"/>
+      <c r="T24" s="33">
         <f>IF(10&lt;=SUM('1 Matériel'!$E$6:$E$29),10,0)</f>
         <v/>
       </c>
-      <c r="U24" s="31">
+      <c r="U24" s="33">
         <f>IF(T24=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T24)+1)</f>
         <v/>
       </c>
-      <c r="V24" s="31">
+      <c r="V24" s="33">
         <f>IF(U24="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U24)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="25" hidden="1" ht="27" customHeight="1">
-      <c r="A25" s="7">
+    <row r="25" hidden="1" ht="40" customHeight="1">
+      <c r="A25" s="28">
         <f>IF(OR(T25=0,V25=1),"",T25-COUNTIF(V$15:V25,1))</f>
         <v/>
       </c>
-      <c r="B25" s="27" t="n"/>
-      <c r="C25" s="27" t="n"/>
-      <c r="D25" s="28">
+      <c r="B25" s="29" t="n"/>
+      <c r="C25" s="30">
         <f>IF(T25=0,"",IF(V25=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U25)),INDEX('1 Matériel'!$C$6:$C$29,U25)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U25)&gt;1,"  ("&amp;(T25-INDEX('1 Matériel'!$F$6:$F$29,U25)+INDEX('1 Matériel'!$E$6:$E$29,U25))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U25)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E25" s="29" t="n"/>
-      <c r="F25" s="29" t="n"/>
-      <c r="G25" s="29" t="n"/>
-      <c r="H25" s="29" t="n"/>
-      <c r="I25" s="30" t="n"/>
-      <c r="J25" s="30" t="n"/>
-      <c r="K25" s="27" t="n"/>
-      <c r="L25" s="30" t="n"/>
-      <c r="T25" s="31">
+      <c r="D25" s="31" t="n"/>
+      <c r="E25" s="31" t="n"/>
+      <c r="F25" s="31" t="n"/>
+      <c r="G25" s="31" t="n"/>
+      <c r="H25" s="32" t="n"/>
+      <c r="I25" s="29" t="n"/>
+      <c r="T25" s="33">
         <f>IF(11&lt;=SUM('1 Matériel'!$E$6:$E$29),11,0)</f>
         <v/>
       </c>
-      <c r="U25" s="31">
+      <c r="U25" s="33">
         <f>IF(T25=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T25)+1)</f>
         <v/>
       </c>
-      <c r="V25" s="31">
+      <c r="V25" s="33">
         <f>IF(U25="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U25)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="26" hidden="1" ht="27" customHeight="1">
-      <c r="A26" s="7">
+    <row r="26" hidden="1" ht="40" customHeight="1">
+      <c r="A26" s="28">
         <f>IF(OR(T26=0,V26=1),"",T26-COUNTIF(V$15:V26,1))</f>
         <v/>
       </c>
-      <c r="B26" s="27" t="n"/>
-      <c r="C26" s="27" t="n"/>
-      <c r="D26" s="28">
+      <c r="B26" s="29" t="n"/>
+      <c r="C26" s="30">
         <f>IF(T26=0,"",IF(V26=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U26)),INDEX('1 Matériel'!$C$6:$C$29,U26)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U26)&gt;1,"  ("&amp;(T26-INDEX('1 Matériel'!$F$6:$F$29,U26)+INDEX('1 Matériel'!$E$6:$E$29,U26))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U26)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E26" s="29" t="n"/>
-      <c r="F26" s="29" t="n"/>
-      <c r="G26" s="29" t="n"/>
-      <c r="H26" s="29" t="n"/>
-      <c r="I26" s="30" t="n"/>
-      <c r="J26" s="30" t="n"/>
-      <c r="K26" s="27" t="n"/>
-      <c r="L26" s="30" t="n"/>
-      <c r="T26" s="31">
+      <c r="D26" s="31" t="n"/>
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="31" t="n"/>
+      <c r="G26" s="31" t="n"/>
+      <c r="H26" s="32" t="n"/>
+      <c r="I26" s="29" t="n"/>
+      <c r="T26" s="33">
         <f>IF(12&lt;=SUM('1 Matériel'!$E$6:$E$29),12,0)</f>
         <v/>
       </c>
-      <c r="U26" s="31">
+      <c r="U26" s="33">
         <f>IF(T26=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T26)+1)</f>
         <v/>
       </c>
-      <c r="V26" s="31">
+      <c r="V26" s="33">
         <f>IF(U26="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U26)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="27" hidden="1" ht="27" customHeight="1">
-      <c r="A27" s="7">
+    <row r="27" hidden="1" ht="40" customHeight="1">
+      <c r="A27" s="28">
         <f>IF(OR(T27=0,V27=1),"",T27-COUNTIF(V$15:V27,1))</f>
         <v/>
       </c>
-      <c r="B27" s="27" t="n"/>
-      <c r="C27" s="27" t="n"/>
-      <c r="D27" s="28">
+      <c r="B27" s="29" t="n"/>
+      <c r="C27" s="30">
         <f>IF(T27=0,"",IF(V27=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U27)),INDEX('1 Matériel'!$C$6:$C$29,U27)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U27)&gt;1,"  ("&amp;(T27-INDEX('1 Matériel'!$F$6:$F$29,U27)+INDEX('1 Matériel'!$E$6:$E$29,U27))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U27)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E27" s="29" t="n"/>
-      <c r="F27" s="29" t="n"/>
-      <c r="G27" s="29" t="n"/>
-      <c r="H27" s="29" t="n"/>
-      <c r="I27" s="30" t="n"/>
-      <c r="J27" s="30" t="n"/>
-      <c r="K27" s="27" t="n"/>
-      <c r="L27" s="30" t="n"/>
-      <c r="T27" s="31">
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="31" t="n"/>
+      <c r="G27" s="31" t="n"/>
+      <c r="H27" s="32" t="n"/>
+      <c r="I27" s="29" t="n"/>
+      <c r="T27" s="33">
         <f>IF(13&lt;=SUM('1 Matériel'!$E$6:$E$29),13,0)</f>
         <v/>
       </c>
-      <c r="U27" s="31">
+      <c r="U27" s="33">
         <f>IF(T27=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T27)+1)</f>
         <v/>
       </c>
-      <c r="V27" s="31">
+      <c r="V27" s="33">
         <f>IF(U27="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U27)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="28" hidden="1" ht="27" customHeight="1">
-      <c r="A28" s="7">
+    <row r="28" hidden="1" ht="40" customHeight="1">
+      <c r="A28" s="28">
         <f>IF(OR(T28=0,V28=1),"",T28-COUNTIF(V$15:V28,1))</f>
         <v/>
       </c>
-      <c r="B28" s="27" t="n"/>
-      <c r="C28" s="27" t="n"/>
-      <c r="D28" s="28">
+      <c r="B28" s="29" t="n"/>
+      <c r="C28" s="30">
         <f>IF(T28=0,"",IF(V28=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U28)),INDEX('1 Matériel'!$C$6:$C$29,U28)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U28)&gt;1,"  ("&amp;(T28-INDEX('1 Matériel'!$F$6:$F$29,U28)+INDEX('1 Matériel'!$E$6:$E$29,U28))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U28)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E28" s="29" t="n"/>
-      <c r="F28" s="29" t="n"/>
-      <c r="G28" s="29" t="n"/>
-      <c r="H28" s="29" t="n"/>
-      <c r="I28" s="30" t="n"/>
-      <c r="J28" s="30" t="n"/>
-      <c r="K28" s="27" t="n"/>
-      <c r="L28" s="30" t="n"/>
-      <c r="T28" s="31">
+      <c r="D28" s="31" t="n"/>
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="31" t="n"/>
+      <c r="G28" s="31" t="n"/>
+      <c r="H28" s="32" t="n"/>
+      <c r="I28" s="29" t="n"/>
+      <c r="T28" s="33">
         <f>IF(14&lt;=SUM('1 Matériel'!$E$6:$E$29),14,0)</f>
         <v/>
       </c>
-      <c r="U28" s="31">
+      <c r="U28" s="33">
         <f>IF(T28=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T28)+1)</f>
         <v/>
       </c>
-      <c r="V28" s="31">
+      <c r="V28" s="33">
         <f>IF(U28="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U28)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="29" hidden="1" ht="27" customHeight="1">
-      <c r="A29" s="7">
+    <row r="29" hidden="1" ht="40" customHeight="1">
+      <c r="A29" s="28">
         <f>IF(OR(T29=0,V29=1),"",T29-COUNTIF(V$15:V29,1))</f>
         <v/>
       </c>
-      <c r="B29" s="27" t="n"/>
-      <c r="C29" s="27" t="n"/>
-      <c r="D29" s="28">
+      <c r="B29" s="29" t="n"/>
+      <c r="C29" s="30">
         <f>IF(T29=0,"",IF(V29=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U29)),INDEX('1 Matériel'!$C$6:$C$29,U29)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U29)&gt;1,"  ("&amp;(T29-INDEX('1 Matériel'!$F$6:$F$29,U29)+INDEX('1 Matériel'!$E$6:$E$29,U29))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U29)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E29" s="29" t="n"/>
-      <c r="F29" s="29" t="n"/>
-      <c r="G29" s="29" t="n"/>
-      <c r="H29" s="29" t="n"/>
-      <c r="I29" s="30" t="n"/>
-      <c r="J29" s="30" t="n"/>
-      <c r="K29" s="27" t="n"/>
-      <c r="L29" s="30" t="n"/>
-      <c r="T29" s="31">
+      <c r="D29" s="31" t="n"/>
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="31" t="n"/>
+      <c r="G29" s="31" t="n"/>
+      <c r="H29" s="32" t="n"/>
+      <c r="I29" s="29" t="n"/>
+      <c r="T29" s="33">
         <f>IF(15&lt;=SUM('1 Matériel'!$E$6:$E$29),15,0)</f>
         <v/>
       </c>
-      <c r="U29" s="31">
+      <c r="U29" s="33">
         <f>IF(T29=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T29)+1)</f>
         <v/>
       </c>
-      <c r="V29" s="31">
+      <c r="V29" s="33">
         <f>IF(U29="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U29)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="30" hidden="1" ht="27" customHeight="1">
-      <c r="A30" s="7">
+    <row r="30" hidden="1" ht="40" customHeight="1">
+      <c r="A30" s="28">
         <f>IF(OR(T30=0,V30=1),"",T30-COUNTIF(V$15:V30,1))</f>
         <v/>
       </c>
-      <c r="B30" s="27" t="n"/>
-      <c r="C30" s="27" t="n"/>
-      <c r="D30" s="28">
+      <c r="B30" s="29" t="n"/>
+      <c r="C30" s="30">
         <f>IF(T30=0,"",IF(V30=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U30)),INDEX('1 Matériel'!$C$6:$C$29,U30)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U30)&gt;1,"  ("&amp;(T30-INDEX('1 Matériel'!$F$6:$F$29,U30)+INDEX('1 Matériel'!$E$6:$E$29,U30))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U30)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E30" s="29" t="n"/>
-      <c r="F30" s="29" t="n"/>
-      <c r="G30" s="29" t="n"/>
-      <c r="H30" s="29" t="n"/>
-      <c r="I30" s="30" t="n"/>
-      <c r="J30" s="30" t="n"/>
-      <c r="K30" s="27" t="n"/>
-      <c r="L30" s="30" t="n"/>
-      <c r="T30" s="31">
+      <c r="D30" s="31" t="n"/>
+      <c r="E30" s="31" t="n"/>
+      <c r="F30" s="31" t="n"/>
+      <c r="G30" s="31" t="n"/>
+      <c r="H30" s="32" t="n"/>
+      <c r="I30" s="29" t="n"/>
+      <c r="T30" s="33">
         <f>IF(16&lt;=SUM('1 Matériel'!$E$6:$E$29),16,0)</f>
         <v/>
       </c>
-      <c r="U30" s="31">
+      <c r="U30" s="33">
         <f>IF(T30=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T30)+1)</f>
         <v/>
       </c>
-      <c r="V30" s="31">
+      <c r="V30" s="33">
         <f>IF(U30="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U30)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="31" hidden="1" ht="27" customHeight="1">
-      <c r="A31" s="7">
+    <row r="31" hidden="1" ht="40" customHeight="1">
+      <c r="A31" s="28">
         <f>IF(OR(T31=0,V31=1),"",T31-COUNTIF(V$15:V31,1))</f>
         <v/>
       </c>
-      <c r="B31" s="27" t="n"/>
-      <c r="C31" s="27" t="n"/>
-      <c r="D31" s="28">
+      <c r="B31" s="29" t="n"/>
+      <c r="C31" s="30">
         <f>IF(T31=0,"",IF(V31=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U31)),INDEX('1 Matériel'!$C$6:$C$29,U31)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U31)&gt;1,"  ("&amp;(T31-INDEX('1 Matériel'!$F$6:$F$29,U31)+INDEX('1 Matériel'!$E$6:$E$29,U31))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U31)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E31" s="29" t="n"/>
-      <c r="F31" s="29" t="n"/>
-      <c r="G31" s="29" t="n"/>
-      <c r="H31" s="29" t="n"/>
-      <c r="I31" s="30" t="n"/>
-      <c r="J31" s="30" t="n"/>
-      <c r="K31" s="27" t="n"/>
-      <c r="L31" s="30" t="n"/>
-      <c r="T31" s="31">
+      <c r="D31" s="31" t="n"/>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="31" t="n"/>
+      <c r="G31" s="31" t="n"/>
+      <c r="H31" s="32" t="n"/>
+      <c r="I31" s="29" t="n"/>
+      <c r="T31" s="33">
         <f>IF(17&lt;=SUM('1 Matériel'!$E$6:$E$29),17,0)</f>
         <v/>
       </c>
-      <c r="U31" s="31">
+      <c r="U31" s="33">
         <f>IF(T31=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T31)+1)</f>
         <v/>
       </c>
-      <c r="V31" s="31">
+      <c r="V31" s="33">
         <f>IF(U31="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U31)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="32" hidden="1" ht="27" customHeight="1">
-      <c r="A32" s="7">
+    <row r="32" hidden="1" ht="40" customHeight="1">
+      <c r="A32" s="28">
         <f>IF(OR(T32=0,V32=1),"",T32-COUNTIF(V$15:V32,1))</f>
         <v/>
       </c>
-      <c r="B32" s="27" t="n"/>
-      <c r="C32" s="27" t="n"/>
-      <c r="D32" s="28">
+      <c r="B32" s="29" t="n"/>
+      <c r="C32" s="30">
         <f>IF(T32=0,"",IF(V32=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U32)),INDEX('1 Matériel'!$C$6:$C$29,U32)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U32)&gt;1,"  ("&amp;(T32-INDEX('1 Matériel'!$F$6:$F$29,U32)+INDEX('1 Matériel'!$E$6:$E$29,U32))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U32)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E32" s="29" t="n"/>
-      <c r="F32" s="29" t="n"/>
-      <c r="G32" s="29" t="n"/>
-      <c r="H32" s="29" t="n"/>
-      <c r="I32" s="30" t="n"/>
-      <c r="J32" s="30" t="n"/>
-      <c r="K32" s="27" t="n"/>
-      <c r="L32" s="30" t="n"/>
-      <c r="T32" s="31">
+      <c r="D32" s="31" t="n"/>
+      <c r="E32" s="31" t="n"/>
+      <c r="F32" s="31" t="n"/>
+      <c r="G32" s="31" t="n"/>
+      <c r="H32" s="32" t="n"/>
+      <c r="I32" s="29" t="n"/>
+      <c r="T32" s="33">
         <f>IF(18&lt;=SUM('1 Matériel'!$E$6:$E$29),18,0)</f>
         <v/>
       </c>
-      <c r="U32" s="31">
+      <c r="U32" s="33">
         <f>IF(T32=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T32)+1)</f>
         <v/>
       </c>
-      <c r="V32" s="31">
+      <c r="V32" s="33">
         <f>IF(U32="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U32)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="33" hidden="1" ht="27" customHeight="1">
-      <c r="A33" s="7">
+    <row r="33" hidden="1" ht="40" customHeight="1">
+      <c r="A33" s="28">
         <f>IF(OR(T33=0,V33=1),"",T33-COUNTIF(V$15:V33,1))</f>
         <v/>
       </c>
-      <c r="B33" s="27" t="n"/>
-      <c r="C33" s="27" t="n"/>
-      <c r="D33" s="28">
+      <c r="B33" s="29" t="n"/>
+      <c r="C33" s="30">
         <f>IF(T33=0,"",IF(V33=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U33)),INDEX('1 Matériel'!$C$6:$C$29,U33)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U33)&gt;1,"  ("&amp;(T33-INDEX('1 Matériel'!$F$6:$F$29,U33)+INDEX('1 Matériel'!$E$6:$E$29,U33))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U33)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E33" s="29" t="n"/>
-      <c r="F33" s="29" t="n"/>
-      <c r="G33" s="29" t="n"/>
-      <c r="H33" s="29" t="n"/>
-      <c r="I33" s="30" t="n"/>
-      <c r="J33" s="30" t="n"/>
-      <c r="K33" s="27" t="n"/>
-      <c r="L33" s="30" t="n"/>
-      <c r="T33" s="31">
+      <c r="D33" s="31" t="n"/>
+      <c r="E33" s="31" t="n"/>
+      <c r="F33" s="31" t="n"/>
+      <c r="G33" s="31" t="n"/>
+      <c r="H33" s="32" t="n"/>
+      <c r="I33" s="29" t="n"/>
+      <c r="T33" s="33">
         <f>IF(19&lt;=SUM('1 Matériel'!$E$6:$E$29),19,0)</f>
         <v/>
       </c>
-      <c r="U33" s="31">
+      <c r="U33" s="33">
         <f>IF(T33=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T33)+1)</f>
         <v/>
       </c>
-      <c r="V33" s="31">
+      <c r="V33" s="33">
         <f>IF(U33="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U33)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="34" hidden="1" ht="27" customHeight="1">
-      <c r="A34" s="7">
+    <row r="34" hidden="1" ht="40" customHeight="1">
+      <c r="A34" s="28">
         <f>IF(OR(T34=0,V34=1),"",T34-COUNTIF(V$15:V34,1))</f>
         <v/>
       </c>
-      <c r="B34" s="27" t="n"/>
-      <c r="C34" s="27" t="n"/>
-      <c r="D34" s="28">
+      <c r="B34" s="29" t="n"/>
+      <c r="C34" s="30">
         <f>IF(T34=0,"",IF(V34=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U34)),INDEX('1 Matériel'!$C$6:$C$29,U34)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U34)&gt;1,"  ("&amp;(T34-INDEX('1 Matériel'!$F$6:$F$29,U34)+INDEX('1 Matériel'!$E$6:$E$29,U34))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U34)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E34" s="29" t="n"/>
-      <c r="F34" s="29" t="n"/>
-      <c r="G34" s="29" t="n"/>
-      <c r="H34" s="29" t="n"/>
-      <c r="I34" s="30" t="n"/>
-      <c r="J34" s="30" t="n"/>
-      <c r="K34" s="27" t="n"/>
-      <c r="L34" s="30" t="n"/>
-      <c r="T34" s="31">
+      <c r="D34" s="31" t="n"/>
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="31" t="n"/>
+      <c r="G34" s="31" t="n"/>
+      <c r="H34" s="32" t="n"/>
+      <c r="I34" s="29" t="n"/>
+      <c r="T34" s="33">
         <f>IF(20&lt;=SUM('1 Matériel'!$E$6:$E$29),20,0)</f>
         <v/>
       </c>
-      <c r="U34" s="31">
+      <c r="U34" s="33">
         <f>IF(T34=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T34)+1)</f>
         <v/>
       </c>
-      <c r="V34" s="31">
+      <c r="V34" s="33">
         <f>IF(U34="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U34)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="35" hidden="1" ht="27" customHeight="1">
-      <c r="A35" s="7">
+    <row r="35" hidden="1" ht="40" customHeight="1">
+      <c r="A35" s="28">
         <f>IF(OR(T35=0,V35=1),"",T35-COUNTIF(V$15:V35,1))</f>
         <v/>
       </c>
-      <c r="B35" s="27" t="n"/>
-      <c r="C35" s="27" t="n"/>
-      <c r="D35" s="28">
+      <c r="B35" s="29" t="n"/>
+      <c r="C35" s="30">
         <f>IF(T35=0,"",IF(V35=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U35)),INDEX('1 Matériel'!$C$6:$C$29,U35)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U35)&gt;1,"  ("&amp;(T35-INDEX('1 Matériel'!$F$6:$F$29,U35)+INDEX('1 Matériel'!$E$6:$E$29,U35))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U35)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E35" s="29" t="n"/>
-      <c r="F35" s="29" t="n"/>
-      <c r="G35" s="29" t="n"/>
-      <c r="H35" s="29" t="n"/>
-      <c r="I35" s="30" t="n"/>
-      <c r="J35" s="30" t="n"/>
-      <c r="K35" s="27" t="n"/>
-      <c r="L35" s="30" t="n"/>
-      <c r="T35" s="31">
+      <c r="D35" s="31" t="n"/>
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="31" t="n"/>
+      <c r="G35" s="31" t="n"/>
+      <c r="H35" s="32" t="n"/>
+      <c r="I35" s="29" t="n"/>
+      <c r="T35" s="33">
         <f>IF(21&lt;=SUM('1 Matériel'!$E$6:$E$29),21,0)</f>
         <v/>
       </c>
-      <c r="U35" s="31">
+      <c r="U35" s="33">
         <f>IF(T35=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T35)+1)</f>
         <v/>
       </c>
-      <c r="V35" s="31">
+      <c r="V35" s="33">
         <f>IF(U35="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U35)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="36" hidden="1" ht="27" customHeight="1">
-      <c r="A36" s="7">
+    <row r="36" hidden="1" ht="40" customHeight="1">
+      <c r="A36" s="28">
         <f>IF(OR(T36=0,V36=1),"",T36-COUNTIF(V$15:V36,1))</f>
         <v/>
       </c>
-      <c r="B36" s="27" t="n"/>
-      <c r="C36" s="27" t="n"/>
-      <c r="D36" s="28">
+      <c r="B36" s="29" t="n"/>
+      <c r="C36" s="30">
         <f>IF(T36=0,"",IF(V36=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U36)),INDEX('1 Matériel'!$C$6:$C$29,U36)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U36)&gt;1,"  ("&amp;(T36-INDEX('1 Matériel'!$F$6:$F$29,U36)+INDEX('1 Matériel'!$E$6:$E$29,U36))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U36)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E36" s="29" t="n"/>
-      <c r="F36" s="29" t="n"/>
-      <c r="G36" s="29" t="n"/>
-      <c r="H36" s="29" t="n"/>
-      <c r="I36" s="30" t="n"/>
-      <c r="J36" s="30" t="n"/>
-      <c r="K36" s="27" t="n"/>
-      <c r="L36" s="30" t="n"/>
-      <c r="T36" s="31">
+      <c r="D36" s="31" t="n"/>
+      <c r="E36" s="31" t="n"/>
+      <c r="F36" s="31" t="n"/>
+      <c r="G36" s="31" t="n"/>
+      <c r="H36" s="32" t="n"/>
+      <c r="I36" s="29" t="n"/>
+      <c r="T36" s="33">
         <f>IF(22&lt;=SUM('1 Matériel'!$E$6:$E$29),22,0)</f>
         <v/>
       </c>
-      <c r="U36" s="31">
+      <c r="U36" s="33">
         <f>IF(T36=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T36)+1)</f>
         <v/>
       </c>
-      <c r="V36" s="31">
+      <c r="V36" s="33">
         <f>IF(U36="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U36)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="37" hidden="1" ht="27" customHeight="1">
-      <c r="A37" s="7">
+    <row r="37" hidden="1" ht="40" customHeight="1">
+      <c r="A37" s="28">
         <f>IF(OR(T37=0,V37=1),"",T37-COUNTIF(V$15:V37,1))</f>
         <v/>
       </c>
-      <c r="B37" s="27" t="n"/>
-      <c r="C37" s="27" t="n"/>
-      <c r="D37" s="28">
+      <c r="B37" s="29" t="n"/>
+      <c r="C37" s="30">
         <f>IF(T37=0,"",IF(V37=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U37)),INDEX('1 Matériel'!$C$6:$C$29,U37)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U37)&gt;1,"  ("&amp;(T37-INDEX('1 Matériel'!$F$6:$F$29,U37)+INDEX('1 Matériel'!$E$6:$E$29,U37))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U37)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E37" s="29" t="n"/>
-      <c r="F37" s="29" t="n"/>
-      <c r="G37" s="29" t="n"/>
-      <c r="H37" s="29" t="n"/>
-      <c r="I37" s="30" t="n"/>
-      <c r="J37" s="30" t="n"/>
-      <c r="K37" s="27" t="n"/>
-      <c r="L37" s="30" t="n"/>
-      <c r="T37" s="31">
+      <c r="D37" s="31" t="n"/>
+      <c r="E37" s="31" t="n"/>
+      <c r="F37" s="31" t="n"/>
+      <c r="G37" s="31" t="n"/>
+      <c r="H37" s="32" t="n"/>
+      <c r="I37" s="29" t="n"/>
+      <c r="T37" s="33">
         <f>IF(23&lt;=SUM('1 Matériel'!$E$6:$E$29),23,0)</f>
         <v/>
       </c>
-      <c r="U37" s="31">
+      <c r="U37" s="33">
         <f>IF(T37=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T37)+1)</f>
         <v/>
       </c>
-      <c r="V37" s="31">
+      <c r="V37" s="33">
         <f>IF(U37="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U37)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="38" hidden="1" ht="27" customHeight="1">
-      <c r="A38" s="7">
+    <row r="38" hidden="1" ht="40" customHeight="1">
+      <c r="A38" s="28">
         <f>IF(OR(T38=0,V38=1),"",T38-COUNTIF(V$15:V38,1))</f>
         <v/>
       </c>
-      <c r="B38" s="27" t="n"/>
-      <c r="C38" s="27" t="n"/>
-      <c r="D38" s="28">
+      <c r="B38" s="29" t="n"/>
+      <c r="C38" s="30">
         <f>IF(T38=0,"",IF(V38=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U38)),INDEX('1 Matériel'!$C$6:$C$29,U38)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U38)&gt;1,"  ("&amp;(T38-INDEX('1 Matériel'!$F$6:$F$29,U38)+INDEX('1 Matériel'!$E$6:$E$29,U38))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U38)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E38" s="29" t="n"/>
-      <c r="F38" s="29" t="n"/>
-      <c r="G38" s="29" t="n"/>
-      <c r="H38" s="29" t="n"/>
-      <c r="I38" s="30" t="n"/>
-      <c r="J38" s="30" t="n"/>
-      <c r="K38" s="27" t="n"/>
-      <c r="L38" s="30" t="n"/>
-      <c r="T38" s="31">
+      <c r="D38" s="31" t="n"/>
+      <c r="E38" s="31" t="n"/>
+      <c r="F38" s="31" t="n"/>
+      <c r="G38" s="31" t="n"/>
+      <c r="H38" s="32" t="n"/>
+      <c r="I38" s="29" t="n"/>
+      <c r="T38" s="33">
         <f>IF(24&lt;=SUM('1 Matériel'!$E$6:$E$29),24,0)</f>
         <v/>
       </c>
-      <c r="U38" s="31">
+      <c r="U38" s="33">
         <f>IF(T38=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T38)+1)</f>
         <v/>
       </c>
-      <c r="V38" s="31">
+      <c r="V38" s="33">
         <f>IF(U38="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U38)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="39" hidden="1" ht="27" customHeight="1">
-      <c r="A39" s="7">
+    <row r="39" hidden="1" ht="40" customHeight="1">
+      <c r="A39" s="28">
         <f>IF(OR(T39=0,V39=1),"",T39-COUNTIF(V$15:V39,1))</f>
         <v/>
       </c>
-      <c r="B39" s="27" t="n"/>
-      <c r="C39" s="27" t="n"/>
-      <c r="D39" s="28">
+      <c r="B39" s="29" t="n"/>
+      <c r="C39" s="30">
         <f>IF(T39=0,"",IF(V39=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U39)),INDEX('1 Matériel'!$C$6:$C$29,U39)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U39)&gt;1,"  ("&amp;(T39-INDEX('1 Matériel'!$F$6:$F$29,U39)+INDEX('1 Matériel'!$E$6:$E$29,U39))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U39)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E39" s="29" t="n"/>
-      <c r="F39" s="29" t="n"/>
-      <c r="G39" s="29" t="n"/>
-      <c r="H39" s="29" t="n"/>
-      <c r="I39" s="30" t="n"/>
-      <c r="J39" s="30" t="n"/>
-      <c r="K39" s="27" t="n"/>
-      <c r="L39" s="30" t="n"/>
-      <c r="T39" s="31">
+      <c r="D39" s="31" t="n"/>
+      <c r="E39" s="31" t="n"/>
+      <c r="F39" s="31" t="n"/>
+      <c r="G39" s="31" t="n"/>
+      <c r="H39" s="32" t="n"/>
+      <c r="I39" s="29" t="n"/>
+      <c r="T39" s="33">
         <f>IF(25&lt;=SUM('1 Matériel'!$E$6:$E$29),25,0)</f>
         <v/>
       </c>
-      <c r="U39" s="31">
+      <c r="U39" s="33">
         <f>IF(T39=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T39)+1)</f>
         <v/>
       </c>
-      <c r="V39" s="31">
+      <c r="V39" s="33">
         <f>IF(U39="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U39)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="40" hidden="1" ht="27" customHeight="1">
-      <c r="A40" s="7">
+    <row r="40" hidden="1" ht="40" customHeight="1">
+      <c r="A40" s="28">
         <f>IF(OR(T40=0,V40=1),"",T40-COUNTIF(V$15:V40,1))</f>
         <v/>
       </c>
-      <c r="B40" s="27" t="n"/>
-      <c r="C40" s="27" t="n"/>
-      <c r="D40" s="28">
+      <c r="B40" s="29" t="n"/>
+      <c r="C40" s="30">
         <f>IF(T40=0,"",IF(V40=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U40)),INDEX('1 Matériel'!$C$6:$C$29,U40)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U40)&gt;1,"  ("&amp;(T40-INDEX('1 Matériel'!$F$6:$F$29,U40)+INDEX('1 Matériel'!$E$6:$E$29,U40))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U40)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E40" s="29" t="n"/>
-      <c r="F40" s="29" t="n"/>
-      <c r="G40" s="29" t="n"/>
-      <c r="H40" s="29" t="n"/>
-      <c r="I40" s="30" t="n"/>
-      <c r="J40" s="30" t="n"/>
-      <c r="K40" s="27" t="n"/>
-      <c r="L40" s="30" t="n"/>
-      <c r="T40" s="31">
+      <c r="D40" s="31" t="n"/>
+      <c r="E40" s="31" t="n"/>
+      <c r="F40" s="31" t="n"/>
+      <c r="G40" s="31" t="n"/>
+      <c r="H40" s="32" t="n"/>
+      <c r="I40" s="29" t="n"/>
+      <c r="T40" s="33">
         <f>IF(26&lt;=SUM('1 Matériel'!$E$6:$E$29),26,0)</f>
         <v/>
       </c>
-      <c r="U40" s="31">
+      <c r="U40" s="33">
         <f>IF(T40=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T40)+1)</f>
         <v/>
       </c>
-      <c r="V40" s="31">
+      <c r="V40" s="33">
         <f>IF(U40="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U40)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="41" hidden="1" ht="27" customHeight="1">
-      <c r="A41" s="7">
+    <row r="41" hidden="1" ht="40" customHeight="1">
+      <c r="A41" s="28">
         <f>IF(OR(T41=0,V41=1),"",T41-COUNTIF(V$15:V41,1))</f>
         <v/>
       </c>
-      <c r="B41" s="27" t="n"/>
-      <c r="C41" s="27" t="n"/>
-      <c r="D41" s="28">
+      <c r="B41" s="29" t="n"/>
+      <c r="C41" s="30">
         <f>IF(T41=0,"",IF(V41=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U41)),INDEX('1 Matériel'!$C$6:$C$29,U41)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U41)&gt;1,"  ("&amp;(T41-INDEX('1 Matériel'!$F$6:$F$29,U41)+INDEX('1 Matériel'!$E$6:$E$29,U41))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U41)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E41" s="29" t="n"/>
-      <c r="F41" s="29" t="n"/>
-      <c r="G41" s="29" t="n"/>
-      <c r="H41" s="29" t="n"/>
-      <c r="I41" s="30" t="n"/>
-      <c r="J41" s="30" t="n"/>
-      <c r="K41" s="27" t="n"/>
-      <c r="L41" s="30" t="n"/>
-      <c r="T41" s="31">
+      <c r="D41" s="31" t="n"/>
+      <c r="E41" s="31" t="n"/>
+      <c r="F41" s="31" t="n"/>
+      <c r="G41" s="31" t="n"/>
+      <c r="H41" s="32" t="n"/>
+      <c r="I41" s="29" t="n"/>
+      <c r="T41" s="33">
         <f>IF(27&lt;=SUM('1 Matériel'!$E$6:$E$29),27,0)</f>
         <v/>
       </c>
-      <c r="U41" s="31">
+      <c r="U41" s="33">
         <f>IF(T41=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T41)+1)</f>
         <v/>
       </c>
-      <c r="V41" s="31">
+      <c r="V41" s="33">
         <f>IF(U41="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U41)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="42" hidden="1" ht="27" customHeight="1">
-      <c r="A42" s="7">
+    <row r="42" hidden="1" ht="40" customHeight="1">
+      <c r="A42" s="28">
         <f>IF(OR(T42=0,V42=1),"",T42-COUNTIF(V$15:V42,1))</f>
         <v/>
       </c>
-      <c r="B42" s="27" t="n"/>
-      <c r="C42" s="27" t="n"/>
-      <c r="D42" s="28">
+      <c r="B42" s="29" t="n"/>
+      <c r="C42" s="30">
         <f>IF(T42=0,"",IF(V42=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U42)),INDEX('1 Matériel'!$C$6:$C$29,U42)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U42)&gt;1,"  ("&amp;(T42-INDEX('1 Matériel'!$F$6:$F$29,U42)+INDEX('1 Matériel'!$E$6:$E$29,U42))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U42)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E42" s="29" t="n"/>
-      <c r="F42" s="29" t="n"/>
-      <c r="G42" s="29" t="n"/>
-      <c r="H42" s="29" t="n"/>
-      <c r="I42" s="30" t="n"/>
-      <c r="J42" s="30" t="n"/>
-      <c r="K42" s="27" t="n"/>
-      <c r="L42" s="30" t="n"/>
-      <c r="T42" s="31">
+      <c r="D42" s="31" t="n"/>
+      <c r="E42" s="31" t="n"/>
+      <c r="F42" s="31" t="n"/>
+      <c r="G42" s="31" t="n"/>
+      <c r="H42" s="32" t="n"/>
+      <c r="I42" s="29" t="n"/>
+      <c r="T42" s="33">
         <f>IF(28&lt;=SUM('1 Matériel'!$E$6:$E$29),28,0)</f>
         <v/>
       </c>
-      <c r="U42" s="31">
+      <c r="U42" s="33">
         <f>IF(T42=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T42)+1)</f>
         <v/>
       </c>
-      <c r="V42" s="31">
+      <c r="V42" s="33">
         <f>IF(U42="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U42)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="43" hidden="1" ht="27" customHeight="1">
-      <c r="A43" s="7">
+    <row r="43" hidden="1" ht="40" customHeight="1">
+      <c r="A43" s="28">
         <f>IF(OR(T43=0,V43=1),"",T43-COUNTIF(V$15:V43,1))</f>
         <v/>
       </c>
-      <c r="B43" s="27" t="n"/>
-      <c r="C43" s="27" t="n"/>
-      <c r="D43" s="28">
+      <c r="B43" s="29" t="n"/>
+      <c r="C43" s="30">
         <f>IF(T43=0,"",IF(V43=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U43)),INDEX('1 Matériel'!$C$6:$C$29,U43)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U43)&gt;1,"  ("&amp;(T43-INDEX('1 Matériel'!$F$6:$F$29,U43)+INDEX('1 Matériel'!$E$6:$E$29,U43))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U43)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E43" s="29" t="n"/>
-      <c r="F43" s="29" t="n"/>
-      <c r="G43" s="29" t="n"/>
-      <c r="H43" s="29" t="n"/>
-      <c r="I43" s="30" t="n"/>
-      <c r="J43" s="30" t="n"/>
-      <c r="K43" s="27" t="n"/>
-      <c r="L43" s="30" t="n"/>
-      <c r="T43" s="31">
+      <c r="D43" s="31" t="n"/>
+      <c r="E43" s="31" t="n"/>
+      <c r="F43" s="31" t="n"/>
+      <c r="G43" s="31" t="n"/>
+      <c r="H43" s="32" t="n"/>
+      <c r="I43" s="29" t="n"/>
+      <c r="T43" s="33">
         <f>IF(29&lt;=SUM('1 Matériel'!$E$6:$E$29),29,0)</f>
         <v/>
       </c>
-      <c r="U43" s="31">
+      <c r="U43" s="33">
         <f>IF(T43=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T43)+1)</f>
         <v/>
       </c>
-      <c r="V43" s="31">
+      <c r="V43" s="33">
         <f>IF(U43="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U43)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="44" hidden="1" ht="27" customHeight="1">
-      <c r="A44" s="7">
+    <row r="44" hidden="1" ht="40" customHeight="1">
+      <c r="A44" s="28">
         <f>IF(OR(T44=0,V44=1),"",T44-COUNTIF(V$15:V44,1))</f>
         <v/>
       </c>
-      <c r="B44" s="27" t="n"/>
-      <c r="C44" s="27" t="n"/>
-      <c r="D44" s="28">
+      <c r="B44" s="29" t="n"/>
+      <c r="C44" s="30">
         <f>IF(T44=0,"",IF(V44=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U44)),INDEX('1 Matériel'!$C$6:$C$29,U44)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U44)&gt;1,"  ("&amp;(T44-INDEX('1 Matériel'!$F$6:$F$29,U44)+INDEX('1 Matériel'!$E$6:$E$29,U44))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U44)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E44" s="29" t="n"/>
-      <c r="F44" s="29" t="n"/>
-      <c r="G44" s="29" t="n"/>
-      <c r="H44" s="29" t="n"/>
-      <c r="I44" s="30" t="n"/>
-      <c r="J44" s="30" t="n"/>
-      <c r="K44" s="27" t="n"/>
-      <c r="L44" s="30" t="n"/>
-      <c r="T44" s="31">
+      <c r="D44" s="31" t="n"/>
+      <c r="E44" s="31" t="n"/>
+      <c r="F44" s="31" t="n"/>
+      <c r="G44" s="31" t="n"/>
+      <c r="H44" s="32" t="n"/>
+      <c r="I44" s="29" t="n"/>
+      <c r="T44" s="33">
         <f>IF(30&lt;=SUM('1 Matériel'!$E$6:$E$29),30,0)</f>
         <v/>
       </c>
-      <c r="U44" s="31">
+      <c r="U44" s="33">
         <f>IF(T44=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T44)+1)</f>
         <v/>
       </c>
-      <c r="V44" s="31">
+      <c r="V44" s="33">
         <f>IF(U44="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U44)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="45" hidden="1" ht="27" customHeight="1">
-      <c r="A45" s="7">
+    <row r="45" hidden="1" ht="40" customHeight="1">
+      <c r="A45" s="28">
         <f>IF(OR(T45=0,V45=1),"",T45-COUNTIF(V$15:V45,1))</f>
         <v/>
       </c>
-      <c r="B45" s="27" t="n"/>
-      <c r="C45" s="27" t="n"/>
-      <c r="D45" s="28">
+      <c r="B45" s="29" t="n"/>
+      <c r="C45" s="30">
         <f>IF(T45=0,"",IF(V45=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U45)),INDEX('1 Matériel'!$C$6:$C$29,U45)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U45)&gt;1,"  ("&amp;(T45-INDEX('1 Matériel'!$F$6:$F$29,U45)+INDEX('1 Matériel'!$E$6:$E$29,U45))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U45)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E45" s="29" t="n"/>
-      <c r="F45" s="29" t="n"/>
-      <c r="G45" s="29" t="n"/>
-      <c r="H45" s="29" t="n"/>
-      <c r="I45" s="30" t="n"/>
-      <c r="J45" s="30" t="n"/>
-      <c r="K45" s="27" t="n"/>
-      <c r="L45" s="30" t="n"/>
-      <c r="T45" s="31">
+      <c r="D45" s="31" t="n"/>
+      <c r="E45" s="31" t="n"/>
+      <c r="F45" s="31" t="n"/>
+      <c r="G45" s="31" t="n"/>
+      <c r="H45" s="32" t="n"/>
+      <c r="I45" s="29" t="n"/>
+      <c r="T45" s="33">
         <f>IF(31&lt;=SUM('1 Matériel'!$E$6:$E$29),31,0)</f>
         <v/>
       </c>
-      <c r="U45" s="31">
+      <c r="U45" s="33">
         <f>IF(T45=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T45)+1)</f>
         <v/>
       </c>
-      <c r="V45" s="31">
+      <c r="V45" s="33">
         <f>IF(U45="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U45)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="46" hidden="1" ht="27" customHeight="1">
-      <c r="A46" s="7">
+    <row r="46" hidden="1" ht="40" customHeight="1">
+      <c r="A46" s="28">
         <f>IF(OR(T46=0,V46=1),"",T46-COUNTIF(V$15:V46,1))</f>
         <v/>
       </c>
-      <c r="B46" s="27" t="n"/>
-      <c r="C46" s="27" t="n"/>
-      <c r="D46" s="28">
+      <c r="B46" s="29" t="n"/>
+      <c r="C46" s="30">
         <f>IF(T46=0,"",IF(V46=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U46)),INDEX('1 Matériel'!$C$6:$C$29,U46)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U46)&gt;1,"  ("&amp;(T46-INDEX('1 Matériel'!$F$6:$F$29,U46)+INDEX('1 Matériel'!$E$6:$E$29,U46))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U46)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E46" s="29" t="n"/>
-      <c r="F46" s="29" t="n"/>
-      <c r="G46" s="29" t="n"/>
-      <c r="H46" s="29" t="n"/>
-      <c r="I46" s="30" t="n"/>
-      <c r="J46" s="30" t="n"/>
-      <c r="K46" s="27" t="n"/>
-      <c r="L46" s="30" t="n"/>
-      <c r="T46" s="31">
+      <c r="D46" s="31" t="n"/>
+      <c r="E46" s="31" t="n"/>
+      <c r="F46" s="31" t="n"/>
+      <c r="G46" s="31" t="n"/>
+      <c r="H46" s="32" t="n"/>
+      <c r="I46" s="29" t="n"/>
+      <c r="T46" s="33">
         <f>IF(32&lt;=SUM('1 Matériel'!$E$6:$E$29),32,0)</f>
         <v/>
       </c>
-      <c r="U46" s="31">
+      <c r="U46" s="33">
         <f>IF(T46=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T46)+1)</f>
         <v/>
       </c>
-      <c r="V46" s="31">
+      <c r="V46" s="33">
         <f>IF(U46="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U46)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="47" hidden="1" ht="27" customHeight="1">
-      <c r="A47" s="7">
+    <row r="47" hidden="1" ht="40" customHeight="1">
+      <c r="A47" s="28">
         <f>IF(OR(T47=0,V47=1),"",T47-COUNTIF(V$15:V47,1))</f>
         <v/>
       </c>
-      <c r="B47" s="27" t="n"/>
-      <c r="C47" s="27" t="n"/>
-      <c r="D47" s="28">
+      <c r="B47" s="29" t="n"/>
+      <c r="C47" s="30">
         <f>IF(T47=0,"",IF(V47=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U47)),INDEX('1 Matériel'!$C$6:$C$29,U47)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U47)&gt;1,"  ("&amp;(T47-INDEX('1 Matériel'!$F$6:$F$29,U47)+INDEX('1 Matériel'!$E$6:$E$29,U47))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U47)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E47" s="29" t="n"/>
-      <c r="F47" s="29" t="n"/>
-      <c r="G47" s="29" t="n"/>
-      <c r="H47" s="29" t="n"/>
-      <c r="I47" s="30" t="n"/>
-      <c r="J47" s="30" t="n"/>
-      <c r="K47" s="27" t="n"/>
-      <c r="L47" s="30" t="n"/>
-      <c r="T47" s="31">
+      <c r="D47" s="31" t="n"/>
+      <c r="E47" s="31" t="n"/>
+      <c r="F47" s="31" t="n"/>
+      <c r="G47" s="31" t="n"/>
+      <c r="H47" s="32" t="n"/>
+      <c r="I47" s="29" t="n"/>
+      <c r="T47" s="33">
         <f>IF(33&lt;=SUM('1 Matériel'!$E$6:$E$29),33,0)</f>
         <v/>
       </c>
-      <c r="U47" s="31">
+      <c r="U47" s="33">
         <f>IF(T47=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T47)+1)</f>
         <v/>
       </c>
-      <c r="V47" s="31">
+      <c r="V47" s="33">
         <f>IF(U47="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U47)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="48" hidden="1" ht="27" customHeight="1">
-      <c r="A48" s="7">
+    <row r="48" hidden="1" ht="40" customHeight="1">
+      <c r="A48" s="28">
         <f>IF(OR(T48=0,V48=1),"",T48-COUNTIF(V$15:V48,1))</f>
         <v/>
       </c>
-      <c r="B48" s="27" t="n"/>
-      <c r="C48" s="27" t="n"/>
-      <c r="D48" s="28">
+      <c r="B48" s="29" t="n"/>
+      <c r="C48" s="30">
         <f>IF(T48=0,"",IF(V48=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U48)),INDEX('1 Matériel'!$C$6:$C$29,U48)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U48)&gt;1,"  ("&amp;(T48-INDEX('1 Matériel'!$F$6:$F$29,U48)+INDEX('1 Matériel'!$E$6:$E$29,U48))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U48)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E48" s="29" t="n"/>
-      <c r="F48" s="29" t="n"/>
-      <c r="G48" s="29" t="n"/>
-      <c r="H48" s="29" t="n"/>
-      <c r="I48" s="30" t="n"/>
-      <c r="J48" s="30" t="n"/>
-      <c r="K48" s="27" t="n"/>
-      <c r="L48" s="30" t="n"/>
-      <c r="T48" s="31">
+      <c r="D48" s="31" t="n"/>
+      <c r="E48" s="31" t="n"/>
+      <c r="F48" s="31" t="n"/>
+      <c r="G48" s="31" t="n"/>
+      <c r="H48" s="32" t="n"/>
+      <c r="I48" s="29" t="n"/>
+      <c r="T48" s="33">
         <f>IF(34&lt;=SUM('1 Matériel'!$E$6:$E$29),34,0)</f>
         <v/>
       </c>
-      <c r="U48" s="31">
+      <c r="U48" s="33">
         <f>IF(T48=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T48)+1)</f>
         <v/>
       </c>
-      <c r="V48" s="31">
+      <c r="V48" s="33">
         <f>IF(U48="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U48)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="49" hidden="1" ht="27" customHeight="1">
-      <c r="A49" s="7">
+    <row r="49" hidden="1" ht="40" customHeight="1">
+      <c r="A49" s="28">
         <f>IF(OR(T49=0,V49=1),"",T49-COUNTIF(V$15:V49,1))</f>
         <v/>
       </c>
-      <c r="B49" s="27" t="n"/>
-      <c r="C49" s="27" t="n"/>
-      <c r="D49" s="28">
+      <c r="B49" s="29" t="n"/>
+      <c r="C49" s="30">
         <f>IF(T49=0,"",IF(V49=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U49)),INDEX('1 Matériel'!$C$6:$C$29,U49)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U49)&gt;1,"  ("&amp;(T49-INDEX('1 Matériel'!$F$6:$F$29,U49)+INDEX('1 Matériel'!$E$6:$E$29,U49))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U49)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E49" s="29" t="n"/>
-      <c r="F49" s="29" t="n"/>
-      <c r="G49" s="29" t="n"/>
-      <c r="H49" s="29" t="n"/>
-      <c r="I49" s="30" t="n"/>
-      <c r="J49" s="30" t="n"/>
-      <c r="K49" s="27" t="n"/>
-      <c r="L49" s="30" t="n"/>
-      <c r="T49" s="31">
+      <c r="D49" s="31" t="n"/>
+      <c r="E49" s="31" t="n"/>
+      <c r="F49" s="31" t="n"/>
+      <c r="G49" s="31" t="n"/>
+      <c r="H49" s="32" t="n"/>
+      <c r="I49" s="29" t="n"/>
+      <c r="T49" s="33">
         <f>IF(35&lt;=SUM('1 Matériel'!$E$6:$E$29),35,0)</f>
         <v/>
       </c>
-      <c r="U49" s="31">
+      <c r="U49" s="33">
         <f>IF(T49=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T49)+1)</f>
         <v/>
       </c>
-      <c r="V49" s="31">
+      <c r="V49" s="33">
         <f>IF(U49="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U49)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="50" hidden="1" ht="27" customHeight="1">
-      <c r="A50" s="7">
+    <row r="50" hidden="1" ht="40" customHeight="1">
+      <c r="A50" s="28">
         <f>IF(OR(T50=0,V50=1),"",T50-COUNTIF(V$15:V50,1))</f>
         <v/>
       </c>
-      <c r="B50" s="27" t="n"/>
-      <c r="C50" s="27" t="n"/>
-      <c r="D50" s="28">
+      <c r="B50" s="29" t="n"/>
+      <c r="C50" s="30">
         <f>IF(T50=0,"",IF(V50=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U50)),INDEX('1 Matériel'!$C$6:$C$29,U50)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U50)&gt;1,"  ("&amp;(T50-INDEX('1 Matériel'!$F$6:$F$29,U50)+INDEX('1 Matériel'!$E$6:$E$29,U50))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U50)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E50" s="29" t="n"/>
-      <c r="F50" s="29" t="n"/>
-      <c r="G50" s="29" t="n"/>
-      <c r="H50" s="29" t="n"/>
-      <c r="I50" s="30" t="n"/>
-      <c r="J50" s="30" t="n"/>
-      <c r="K50" s="27" t="n"/>
-      <c r="L50" s="30" t="n"/>
-      <c r="T50" s="31">
+      <c r="D50" s="31" t="n"/>
+      <c r="E50" s="31" t="n"/>
+      <c r="F50" s="31" t="n"/>
+      <c r="G50" s="31" t="n"/>
+      <c r="H50" s="32" t="n"/>
+      <c r="I50" s="29" t="n"/>
+      <c r="T50" s="33">
         <f>IF(36&lt;=SUM('1 Matériel'!$E$6:$E$29),36,0)</f>
         <v/>
       </c>
-      <c r="U50" s="31">
+      <c r="U50" s="33">
         <f>IF(T50=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T50)+1)</f>
         <v/>
       </c>
-      <c r="V50" s="31">
+      <c r="V50" s="33">
         <f>IF(U50="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U50)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="51" hidden="1" ht="27" customHeight="1">
-      <c r="A51" s="7">
+    <row r="51" hidden="1" ht="40" customHeight="1">
+      <c r="A51" s="28">
         <f>IF(OR(T51=0,V51=1),"",T51-COUNTIF(V$15:V51,1))</f>
         <v/>
       </c>
-      <c r="B51" s="27" t="n"/>
-      <c r="C51" s="27" t="n"/>
-      <c r="D51" s="28">
+      <c r="B51" s="29" t="n"/>
+      <c r="C51" s="30">
         <f>IF(T51=0,"",IF(V51=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U51)),INDEX('1 Matériel'!$C$6:$C$29,U51)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U51)&gt;1,"  ("&amp;(T51-INDEX('1 Matériel'!$F$6:$F$29,U51)+INDEX('1 Matériel'!$E$6:$E$29,U51))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U51)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E51" s="29" t="n"/>
-      <c r="F51" s="29" t="n"/>
-      <c r="G51" s="29" t="n"/>
-      <c r="H51" s="29" t="n"/>
-      <c r="I51" s="30" t="n"/>
-      <c r="J51" s="30" t="n"/>
-      <c r="K51" s="27" t="n"/>
-      <c r="L51" s="30" t="n"/>
-      <c r="T51" s="31">
+      <c r="D51" s="31" t="n"/>
+      <c r="E51" s="31" t="n"/>
+      <c r="F51" s="31" t="n"/>
+      <c r="G51" s="31" t="n"/>
+      <c r="H51" s="32" t="n"/>
+      <c r="I51" s="29" t="n"/>
+      <c r="T51" s="33">
         <f>IF(37&lt;=SUM('1 Matériel'!$E$6:$E$29),37,0)</f>
         <v/>
       </c>
-      <c r="U51" s="31">
+      <c r="U51" s="33">
         <f>IF(T51=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T51)+1)</f>
         <v/>
       </c>
-      <c r="V51" s="31">
+      <c r="V51" s="33">
         <f>IF(U51="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U51)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="52" hidden="1" ht="27" customHeight="1">
-      <c r="A52" s="7">
+    <row r="52" hidden="1" ht="40" customHeight="1">
+      <c r="A52" s="28">
         <f>IF(OR(T52=0,V52=1),"",T52-COUNTIF(V$15:V52,1))</f>
         <v/>
       </c>
-      <c r="B52" s="27" t="n"/>
-      <c r="C52" s="27" t="n"/>
-      <c r="D52" s="28">
+      <c r="B52" s="29" t="n"/>
+      <c r="C52" s="30">
         <f>IF(T52=0,"",IF(V52=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U52)),INDEX('1 Matériel'!$C$6:$C$29,U52)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U52)&gt;1,"  ("&amp;(T52-INDEX('1 Matériel'!$F$6:$F$29,U52)+INDEX('1 Matériel'!$E$6:$E$29,U52))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U52)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E52" s="29" t="n"/>
-      <c r="F52" s="29" t="n"/>
-      <c r="G52" s="29" t="n"/>
-      <c r="H52" s="29" t="n"/>
-      <c r="I52" s="30" t="n"/>
-      <c r="J52" s="30" t="n"/>
-      <c r="K52" s="27" t="n"/>
-      <c r="L52" s="30" t="n"/>
-      <c r="T52" s="31">
+      <c r="D52" s="31" t="n"/>
+      <c r="E52" s="31" t="n"/>
+      <c r="F52" s="31" t="n"/>
+      <c r="G52" s="31" t="n"/>
+      <c r="H52" s="32" t="n"/>
+      <c r="I52" s="29" t="n"/>
+      <c r="T52" s="33">
         <f>IF(38&lt;=SUM('1 Matériel'!$E$6:$E$29),38,0)</f>
         <v/>
       </c>
-      <c r="U52" s="31">
+      <c r="U52" s="33">
         <f>IF(T52=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T52)+1)</f>
         <v/>
       </c>
-      <c r="V52" s="31">
+      <c r="V52" s="33">
         <f>IF(U52="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U52)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="53" hidden="1" ht="27" customHeight="1">
-      <c r="A53" s="7">
+    <row r="53" hidden="1" ht="40" customHeight="1">
+      <c r="A53" s="28">
         <f>IF(OR(T53=0,V53=1),"",T53-COUNTIF(V$15:V53,1))</f>
         <v/>
       </c>
-      <c r="B53" s="27" t="n"/>
-      <c r="C53" s="27" t="n"/>
-      <c r="D53" s="28">
+      <c r="B53" s="29" t="n"/>
+      <c r="C53" s="30">
         <f>IF(T53=0,"",IF(V53=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U53)),INDEX('1 Matériel'!$C$6:$C$29,U53)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U53)&gt;1,"  ("&amp;(T53-INDEX('1 Matériel'!$F$6:$F$29,U53)+INDEX('1 Matériel'!$E$6:$E$29,U53))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U53)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E53" s="29" t="n"/>
-      <c r="F53" s="29" t="n"/>
-      <c r="G53" s="29" t="n"/>
-      <c r="H53" s="29" t="n"/>
-      <c r="I53" s="30" t="n"/>
-      <c r="J53" s="30" t="n"/>
-      <c r="K53" s="27" t="n"/>
-      <c r="L53" s="30" t="n"/>
-      <c r="T53" s="31">
+      <c r="D53" s="31" t="n"/>
+      <c r="E53" s="31" t="n"/>
+      <c r="F53" s="31" t="n"/>
+      <c r="G53" s="31" t="n"/>
+      <c r="H53" s="32" t="n"/>
+      <c r="I53" s="29" t="n"/>
+      <c r="T53" s="33">
         <f>IF(39&lt;=SUM('1 Matériel'!$E$6:$E$29),39,0)</f>
         <v/>
       </c>
-      <c r="U53" s="31">
+      <c r="U53" s="33">
         <f>IF(T53=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T53)+1)</f>
         <v/>
       </c>
-      <c r="V53" s="31">
+      <c r="V53" s="33">
         <f>IF(U53="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U53)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="54" hidden="1" ht="27" customHeight="1">
-      <c r="A54" s="7">
+    <row r="54" hidden="1" ht="40" customHeight="1">
+      <c r="A54" s="28">
         <f>IF(OR(T54=0,V54=1),"",T54-COUNTIF(V$15:V54,1))</f>
         <v/>
       </c>
-      <c r="B54" s="27" t="n"/>
-      <c r="C54" s="27" t="n"/>
-      <c r="D54" s="28">
+      <c r="B54" s="29" t="n"/>
+      <c r="C54" s="30">
         <f>IF(T54=0,"",IF(V54=1,UPPER(INDEX('1 Matériel'!$C$6:$C$29,U54)),INDEX('1 Matériel'!$C$6:$C$29,U54)&amp;IF(INDEX('1 Matériel'!$E$6:$E$29,U54)&gt;1,"  ("&amp;(T54-INDEX('1 Matériel'!$F$6:$F$29,U54)+INDEX('1 Matériel'!$E$6:$E$29,U54))&amp;"/"&amp;INDEX('1 Matériel'!$E$6:$E$29,U54)&amp;")","")))</f>
         <v/>
       </c>
-      <c r="E54" s="29" t="n"/>
-      <c r="F54" s="29" t="n"/>
-      <c r="G54" s="29" t="n"/>
-      <c r="H54" s="29" t="n"/>
-      <c r="I54" s="30" t="n"/>
-      <c r="J54" s="30" t="n"/>
-      <c r="K54" s="27" t="n"/>
-      <c r="L54" s="30" t="n"/>
-      <c r="T54" s="31">
+      <c r="D54" s="31" t="n"/>
+      <c r="E54" s="31" t="n"/>
+      <c r="F54" s="31" t="n"/>
+      <c r="G54" s="31" t="n"/>
+      <c r="H54" s="32" t="n"/>
+      <c r="I54" s="29" t="n"/>
+      <c r="T54" s="33">
         <f>IF(40&lt;=SUM('1 Matériel'!$E$6:$E$29),40,0)</f>
         <v/>
       </c>
-      <c r="U54" s="31">
+      <c r="U54" s="33">
         <f>IF(T54=0,"",COUNTIF('1 Matériel'!$F$6:$F$29,"&lt;"&amp;T54)+1)</f>
         <v/>
       </c>
-      <c r="V54" s="31">
+      <c r="V54" s="33">
         <f>IF(U54="","",IF(INDEX('1 Matériel'!$B$6:$B$29,U54)="Oui",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1"/>
     <row r="56" ht="18" customHeight="1"/>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
-        <is>
-          <t>COLISAGE</t>
-        </is>
-      </c>
-      <c r="B57" s="1" t="n"/>
-      <c r="C57" s="1" t="n"/>
-      <c r="D57" s="1" t="n"/>
-      <c r="E57" s="1" t="n"/>
-      <c r="F57" s="1" t="n"/>
-      <c r="G57" s="1" t="n"/>
-      <c r="H57" s="1" t="n"/>
-      <c r="I57" s="1" t="n"/>
-      <c r="J57" s="1" t="n"/>
-      <c r="K57" s="1" t="n"/>
-      <c r="L57" s="1" t="n"/>
-    </row>
-    <row r="58" ht="26" customHeight="1">
-      <c r="A58" s="25" t="inlineStr">
+    <row r="57" ht="38" customHeight="1">
+      <c r="A57" s="34" t="inlineStr">
+        <is>
+          <t>NOMBRE DE SERRAGES EFFECTUÉS</t>
+        </is>
+      </c>
+      <c r="B57" s="35" t="n"/>
+      <c r="C57" s="35" t="n"/>
+      <c r="D57" s="36" t="n"/>
+      <c r="E57" s="37" t="n"/>
+    </row>
+    <row r="58" ht="18" customHeight="1"/>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="23" t="inlineStr">
+        <is>
+          <t>COLISAGE (ensemble des items)</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="n"/>
+      <c r="C59" s="1" t="n"/>
+      <c r="D59" s="1" t="n"/>
+      <c r="E59" s="1" t="n"/>
+      <c r="F59" s="1" t="n"/>
+      <c r="G59" s="1" t="n"/>
+      <c r="H59" s="1" t="n"/>
+      <c r="I59" s="1" t="n"/>
+    </row>
+    <row r="60" ht="34" customHeight="1">
+      <c r="A60" s="26" t="inlineStr">
         <is>
           <t>Colis</t>
         </is>
       </c>
-      <c r="B58" s="32" t="n"/>
-      <c r="C58" s="25" t="inlineStr">
+      <c r="B60" s="38" t="n"/>
+      <c r="C60" s="26" t="inlineStr">
         <is>
           <t>Type de colisage</t>
         </is>
       </c>
-      <c r="D58" s="25" t="inlineStr">
-        <is>
-          <t>Contenu (items de la liste)</t>
-        </is>
-      </c>
-      <c r="E58" s="25" t="inlineStr">
+      <c r="D60" s="26" t="inlineStr">
         <is>
           <t>Longueur
 (cm)</t>
         </is>
       </c>
-      <c r="F58" s="25" t="inlineStr">
+      <c r="E60" s="26" t="inlineStr">
         <is>
           <t>Largeur
 (cm)</t>
         </is>
       </c>
-      <c r="G58" s="25" t="inlineStr">
+      <c r="F60" s="26" t="inlineStr">
         <is>
           <t>Hauteur
 (cm)</t>
         </is>
       </c>
-      <c r="H58" s="25" t="inlineStr">
+      <c r="G60" s="26" t="inlineStr">
         <is>
           <t>Poids
 (kg)</t>
         </is>
       </c>
-      <c r="I58" s="25" t="inlineStr">
+      <c r="H60" s="26" t="inlineStr">
         <is>
           <t>Volume
 (m³)</t>
         </is>
       </c>
-      <c r="J58" s="25" t="inlineStr">
+      <c r="I60" s="26" t="inlineStr">
         <is>
           <t>Remarques</t>
         </is>
       </c>
-      <c r="K58" s="32" t="n"/>
-    </row>
-    <row r="59" ht="17" customHeight="1">
-      <c r="A59" s="33" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B59" s="34" t="n"/>
-      <c r="C59" s="35" t="n"/>
-      <c r="D59" s="36">
-        <f t="array" ref="D59">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A59,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E59" s="37" t="n"/>
-      <c r="F59" s="37" t="n"/>
-      <c r="G59" s="37" t="n"/>
-      <c r="H59" s="38" t="n"/>
-      <c r="I59" s="39">
-        <f>IF(COUNT(E59:G59)=3,E59*F59*G59/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J59" s="40" t="n"/>
-      <c r="K59" s="34" t="n"/>
-    </row>
-    <row r="60" ht="17" customHeight="1">
-      <c r="A60" s="33" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B60" s="34" t="n"/>
-      <c r="C60" s="35" t="n"/>
-      <c r="D60" s="36">
-        <f t="array" ref="D60">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A60,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E60" s="37" t="n"/>
-      <c r="F60" s="37" t="n"/>
-      <c r="G60" s="37" t="n"/>
-      <c r="H60" s="38" t="n"/>
-      <c r="I60" s="39">
-        <f>IF(COUNT(E60:G60)=3,E60*F60*G60/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J60" s="40" t="n"/>
-      <c r="K60" s="34" t="n"/>
-    </row>
-    <row r="61" ht="17" customHeight="1">
-      <c r="A61" s="33" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B61" s="34" t="n"/>
-      <c r="C61" s="35" t="n"/>
-      <c r="D61" s="36">
-        <f t="array" ref="D61">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A61,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E61" s="37" t="n"/>
-      <c r="F61" s="37" t="n"/>
-      <c r="G61" s="37" t="n"/>
-      <c r="H61" s="38" t="n"/>
-      <c r="I61" s="39">
-        <f>IF(COUNT(E61:G61)=3,E61*F61*G61/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J61" s="40" t="n"/>
-      <c r="K61" s="34" t="n"/>
-    </row>
-    <row r="62" ht="17" customHeight="1">
-      <c r="A62" s="33" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="B62" s="34" t="n"/>
-      <c r="C62" s="35" t="n"/>
-      <c r="D62" s="36">
-        <f t="array" ref="D62">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A62,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E62" s="37" t="n"/>
-      <c r="F62" s="37" t="n"/>
-      <c r="G62" s="37" t="n"/>
-      <c r="H62" s="38" t="n"/>
-      <c r="I62" s="39">
-        <f>IF(COUNT(E62:G62)=3,E62*F62*G62/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J62" s="40" t="n"/>
-      <c r="K62" s="34" t="n"/>
-    </row>
-    <row r="63" ht="17" customHeight="1">
-      <c r="A63" s="33" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B63" s="34" t="n"/>
-      <c r="C63" s="35" t="n"/>
-      <c r="D63" s="36">
-        <f t="array" ref="D63">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A63,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E63" s="37" t="n"/>
-      <c r="F63" s="37" t="n"/>
-      <c r="G63" s="37" t="n"/>
-      <c r="H63" s="38" t="n"/>
-      <c r="I63" s="39">
-        <f>IF(COUNT(E63:G63)=3,E63*F63*G63/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J63" s="40" t="n"/>
-      <c r="K63" s="34" t="n"/>
-    </row>
-    <row r="64" ht="17" customHeight="1">
-      <c r="A64" s="33" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="B64" s="34" t="n"/>
-      <c r="C64" s="35" t="n"/>
-      <c r="D64" s="36">
-        <f t="array" ref="D64">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A64,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E64" s="37" t="n"/>
-      <c r="F64" s="37" t="n"/>
-      <c r="G64" s="37" t="n"/>
-      <c r="H64" s="38" t="n"/>
-      <c r="I64" s="39">
-        <f>IF(COUNT(E64:G64)=3,E64*F64*G64/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J64" s="40" t="n"/>
-      <c r="K64" s="34" t="n"/>
-    </row>
-    <row r="65" ht="17" customHeight="1">
-      <c r="A65" s="33" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B65" s="34" t="n"/>
-      <c r="C65" s="35" t="n"/>
-      <c r="D65" s="36">
-        <f t="array" ref="D65">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A65,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E65" s="37" t="n"/>
-      <c r="F65" s="37" t="n"/>
-      <c r="G65" s="37" t="n"/>
-      <c r="H65" s="38" t="n"/>
-      <c r="I65" s="39">
-        <f>IF(COUNT(E65:G65)=3,E65*F65*G65/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J65" s="40" t="n"/>
-      <c r="K65" s="34" t="n"/>
-    </row>
-    <row r="66" ht="17" customHeight="1">
-      <c r="A66" s="33" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B66" s="34" t="n"/>
-      <c r="C66" s="35" t="n"/>
-      <c r="D66" s="36">
-        <f t="array" ref="D66">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A66,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E66" s="37" t="n"/>
-      <c r="F66" s="37" t="n"/>
-      <c r="G66" s="37" t="n"/>
-      <c r="H66" s="38" t="n"/>
-      <c r="I66" s="39">
-        <f>IF(COUNT(E66:G66)=3,E66*F66*G66/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J66" s="40" t="n"/>
-      <c r="K66" s="34" t="n"/>
-    </row>
-    <row r="67" ht="17" customHeight="1">
-      <c r="A67" s="33" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="B67" s="34" t="n"/>
-      <c r="C67" s="35" t="n"/>
-      <c r="D67" s="36">
-        <f t="array" ref="D67">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A67,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E67" s="37" t="n"/>
-      <c r="F67" s="37" t="n"/>
-      <c r="G67" s="37" t="n"/>
-      <c r="H67" s="38" t="n"/>
-      <c r="I67" s="39">
-        <f>IF(COUNT(E67:G67)=3,E67*F67*G67/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J67" s="40" t="n"/>
-      <c r="K67" s="34" t="n"/>
-    </row>
-    <row r="68" ht="17" customHeight="1">
-      <c r="A68" s="33" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B68" s="34" t="n"/>
-      <c r="C68" s="35" t="n"/>
-      <c r="D68" s="36">
-        <f t="array" ref="D68">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A68,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E68" s="37" t="n"/>
-      <c r="F68" s="37" t="n"/>
-      <c r="G68" s="37" t="n"/>
-      <c r="H68" s="38" t="n"/>
-      <c r="I68" s="39">
-        <f>IF(COUNT(E68:G68)=3,E68*F68*G68/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="J68" s="40" t="n"/>
-      <c r="K68" s="34" t="n"/>
-    </row>
-    <row r="69" ht="17" customHeight="1">
-      <c r="A69" s="33" t="inlineStr">
-        <is>
-          <t>Vrac</t>
-        </is>
-      </c>
-      <c r="B69" s="34" t="n"/>
-      <c r="C69" s="41" t="inlineStr">
-        <is>
-          <t>Vrac</t>
-        </is>
-      </c>
-      <c r="D69" s="36">
-        <f t="array" ref="D69">_xlfn.TEXTJOIN(", ",TRUE,IF($L$15:$L$54=$A69,$A$15:$A$54,""))</f>
-        <v/>
-      </c>
-      <c r="E69" s="34" t="n"/>
-      <c r="F69" s="34" t="n"/>
-      <c r="G69" s="34" t="n"/>
-      <c r="H69" s="38" t="n"/>
-      <c r="I69" s="34" t="n"/>
-      <c r="J69" s="34" t="n"/>
-      <c r="K69" s="34" t="n"/>
-    </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="42">
-        <f>"TOTAL  ·  "&amp;COUNTA(C59:C68)&amp;" colis  ·  "&amp;COUNT($A$15:$A$54)&amp;" outil(s)"</f>
-        <v/>
-      </c>
-      <c r="B70" s="43" t="n"/>
-      <c r="C70" s="43" t="n"/>
-      <c r="D70" s="43" t="n"/>
-      <c r="E70" s="43" t="n"/>
-      <c r="F70" s="43" t="n"/>
-      <c r="G70" s="43" t="n"/>
-      <c r="H70" s="44">
-        <f>SUM(H59:H69)</f>
-        <v/>
-      </c>
-      <c r="I70" s="45">
-        <f>SUM(I59:I68)</f>
-        <v/>
-      </c>
-      <c r="J70" s="46" t="n"/>
-      <c r="K70" s="46" t="n"/>
-    </row>
-    <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="47" t="inlineStr">
-        <is>
-          <t>NOMBRE DE SERRAGES EFFECTUÉS</t>
-        </is>
-      </c>
-      <c r="B72" s="34" t="n"/>
-      <c r="C72" s="34" t="n"/>
-      <c r="D72" s="34" t="n"/>
-      <c r="E72" s="37" t="n"/>
-      <c r="F72" s="40" t="n"/>
+    </row>
+    <row r="61" ht="36" customHeight="1">
+      <c r="A61" s="39" t="inlineStr">
+        <is>
+          <t>Colis 1</t>
+        </is>
+      </c>
+      <c r="B61" s="40" t="n"/>
+      <c r="C61" s="41" t="n"/>
+      <c r="D61" s="42" t="n"/>
+      <c r="E61" s="42" t="n"/>
+      <c r="F61" s="42" t="n"/>
+      <c r="G61" s="43" t="n"/>
+      <c r="H61" s="44">
+        <f>IF(COUNT(D61:F61)=3,D61*E61*F61/1000000,"")</f>
+        <v/>
+      </c>
+      <c r="I61" s="45" t="n"/>
+    </row>
+    <row r="62" ht="36" customHeight="1">
+      <c r="A62" s="39" t="inlineStr">
+        <is>
+          <t>Colis 2</t>
+        </is>
+      </c>
+      <c r="B62" s="40" t="n"/>
+      <c r="C62" s="41" t="n"/>
+      <c r="D62" s="42" t="n"/>
+      <c r="E62" s="42" t="n"/>
+      <c r="F62" s="42" t="n"/>
+      <c r="G62" s="43" t="n"/>
+      <c r="H62" s="44">
+        <f>IF(COUNT(D62:F62)=3,D62*E62*F62/1000000,"")</f>
+        <v/>
+      </c>
+      <c r="I62" s="45" t="n"/>
+    </row>
+    <row r="63" ht="36" customHeight="1">
+      <c r="A63" s="39" t="inlineStr">
+        <is>
+          <t>Colis 3</t>
+        </is>
+      </c>
+      <c r="B63" s="40" t="n"/>
+      <c r="C63" s="41" t="n"/>
+      <c r="D63" s="42" t="n"/>
+      <c r="E63" s="42" t="n"/>
+      <c r="F63" s="42" t="n"/>
+      <c r="G63" s="43" t="n"/>
+      <c r="H63" s="44">
+        <f>IF(COUNT(D63:F63)=3,D63*E63*F63/1000000,"")</f>
+        <v/>
+      </c>
+      <c r="I63" s="45" t="n"/>
+    </row>
+    <row r="64" ht="36" customHeight="1">
+      <c r="A64" s="39" t="inlineStr">
+        <is>
+          <t>Colis 4</t>
+        </is>
+      </c>
+      <c r="B64" s="40" t="n"/>
+      <c r="C64" s="41" t="n"/>
+      <c r="D64" s="42" t="n"/>
+      <c r="E64" s="42" t="n"/>
+      <c r="F64" s="42" t="n"/>
+      <c r="G64" s="43" t="n"/>
+      <c r="H64" s="44">
+        <f>IF(COUNT(D64:F64)=3,D64*E64*F64/1000000,"")</f>
+        <v/>
+      </c>
+      <c r="I64" s="45" t="n"/>
+    </row>
+    <row r="65" ht="36" customHeight="1">
+      <c r="A65" s="39" t="inlineStr">
+        <is>
+          <t>Colis 5</t>
+        </is>
+      </c>
+      <c r="B65" s="40" t="n"/>
+      <c r="C65" s="41" t="n"/>
+      <c r="D65" s="42" t="n"/>
+      <c r="E65" s="42" t="n"/>
+      <c r="F65" s="42" t="n"/>
+      <c r="G65" s="43" t="n"/>
+      <c r="H65" s="44">
+        <f>IF(COUNT(D65:F65)=3,D65*E65*F65/1000000,"")</f>
+        <v/>
+      </c>
+      <c r="I65" s="45" t="n"/>
+    </row>
+    <row r="66" ht="36" customHeight="1">
+      <c r="A66" s="39" t="inlineStr">
+        <is>
+          <t>Colis 6</t>
+        </is>
+      </c>
+      <c r="B66" s="40" t="n"/>
+      <c r="C66" s="41" t="n"/>
+      <c r="D66" s="42" t="n"/>
+      <c r="E66" s="42" t="n"/>
+      <c r="F66" s="42" t="n"/>
+      <c r="G66" s="43" t="n"/>
+      <c r="H66" s="44">
+        <f>IF(COUNT(D66:F66)=3,D66*E66*F66/1000000,"")</f>
+        <v/>
+      </c>
+      <c r="I66" s="45" t="n"/>
+    </row>
+    <row r="67" ht="28" customHeight="1">
+      <c r="A67" s="46">
+        <f>"TOTAL  ·  "&amp;COUNTA(C61:C66)&amp;" colis"</f>
+        <v/>
+      </c>
+      <c r="B67" s="47" t="n"/>
+      <c r="C67" s="47" t="n"/>
+      <c r="D67" s="48" t="n"/>
+      <c r="E67" s="48" t="n"/>
+      <c r="F67" s="48" t="n"/>
+      <c r="G67" s="49">
+        <f>SUM(G61:G66)</f>
+        <v/>
+      </c>
+      <c r="H67" s="50">
+        <f>SUM(H61:H66)</f>
+        <v/>
+      </c>
+      <c r="I67" s="48" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A14:V54">
@@ -3293,65 +3009,44 @@
     <filterColumn colId="20" hiddenButton="1" showButton="0"/>
     <filterColumn colId="21" hiddenButton="1" showButton="0"/>
   </autoFilter>
-  <mergeCells count="56">
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J64:K64"/>
+  <mergeCells count="35">
+    <mergeCell ref="D9:G9"/>
     <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="G6:I6"/>
     <mergeCell ref="A60:B60"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="J67:K67"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="J59:K59"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A12:L12"/>
-    <mergeCell ref="J60:K60"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="A57:L57"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="F1:L1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="J68:K68"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A65:B65"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="E13:I13"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="E1:I1"/>
     <mergeCell ref="A66:B66"/>
-    <mergeCell ref="J65:K65"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="J58:K58"/>
-    <mergeCell ref="E9:I9"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="A70:G70"/>
-    <mergeCell ref="J63:K63"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="J66:K66"/>
-    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A59:I59"/>
     <mergeCell ref="A62:B62"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="A11:L11"/>
-    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A11:I11"/>
     <mergeCell ref="A63:B63"/>
-    <mergeCell ref="E72:F72"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="J62:K62"/>
-    <mergeCell ref="F2:L2"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J61:K61"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H8:I8"/>
   </mergeCells>
-  <conditionalFormatting sqref="A15:L54">
+  <conditionalFormatting sqref="A15:I54">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
       <formula>$V15=1</formula>
     </cfRule>
@@ -3359,21 +3054,9 @@
       <formula>$T15&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="13">
-    <dataValidation sqref="I15:I54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
+  <dataValidations count="7">
+    <dataValidation sqref="H15:H54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$Q$2:$Q$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="J15:J54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$G$2:$G$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="L15:L54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$K$2:$K$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="C59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$J$2:$J$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="C60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$J$2:$J$12</formula1>
     </dataValidation>
     <dataValidation sqref="C61" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$J$2:$J$12</formula1>
@@ -3393,12 +3076,6 @@
     <dataValidation sqref="C66" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$J$2:$J$12</formula1>
     </dataValidation>
-    <dataValidation sqref="C67" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$J$2:$J$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="C68" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$J$2:$J$12</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3410,6 +3087,9 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="58" min="0" max="16383" man="1"/>
+  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -3440,366 +3120,366 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="48" t="inlineStr">
+      <c r="A1" s="51" t="inlineStr">
         <is>
           <t>Contact Enedril</t>
         </is>
       </c>
-      <c r="B1" s="48" t="inlineStr">
+      <c r="B1" s="51" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="D1" s="48" t="inlineStr">
+      <c r="D1" s="51" t="inlineStr">
         <is>
           <t>Incoterm</t>
         </is>
       </c>
-      <c r="E1" s="48" t="inlineStr">
+      <c r="E1" s="51" t="inlineStr">
         <is>
           <t>Validité</t>
         </is>
       </c>
-      <c r="F1" s="48" t="inlineStr">
+      <c r="F1" s="51" t="inlineStr">
         <is>
           <t>Règlement</t>
         </is>
       </c>
-      <c r="G1" s="48" t="inlineStr">
+      <c r="G1" s="51" t="inlineStr">
         <is>
           <t>Oui / Non</t>
         </is>
       </c>
-      <c r="H1" s="49" t="n">
+      <c r="H1" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="J1" s="48" t="inlineStr">
+      <c r="J1" s="51" t="inlineStr">
         <is>
           <t>Support de colisage</t>
         </is>
       </c>
-      <c r="K1" s="48" t="inlineStr">
+      <c r="K1" s="51" t="inlineStr">
         <is>
           <t>N° de colis</t>
         </is>
       </c>
-      <c r="L1" s="48" t="inlineStr">
+      <c r="L1" s="51" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="M1" s="48" t="inlineStr">
+      <c r="M1" s="51" t="inlineStr">
         <is>
           <t>Mode transport</t>
         </is>
       </c>
-      <c r="N1" s="48" t="inlineStr">
+      <c r="N1" s="51" t="inlineStr">
         <is>
           <t>Mode forfait</t>
         </is>
       </c>
-      <c r="P1" s="48" t="inlineStr">
+      <c r="P1" s="51" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="Q1" s="48" t="inlineStr">
+      <c r="Q1" s="51" t="inlineStr">
         <is>
           <t>Test / Taille</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="50" t="inlineStr">
+      <c r="A2" s="53" t="inlineStr">
         <is>
           <t>Fabien JACQUOT</t>
         </is>
       </c>
-      <c r="B2" s="50" t="inlineStr">
+      <c r="B2" s="53" t="inlineStr">
         <is>
           <t>fjacquot@enedril.fr</t>
         </is>
       </c>
-      <c r="D2" s="50" t="inlineStr">
+      <c r="D2" s="53" t="inlineStr">
         <is>
           <t>EXW Lons</t>
         </is>
       </c>
-      <c r="E2" s="50" t="inlineStr">
+      <c r="E2" s="53" t="inlineStr">
         <is>
           <t>15 jours / 15 days</t>
         </is>
       </c>
-      <c r="F2" s="50" t="inlineStr">
+      <c r="F2" s="53" t="inlineStr">
         <is>
           <t>30 jours date de facture / 30 days invoice date</t>
         </is>
       </c>
-      <c r="G2" s="50" t="inlineStr">
+      <c r="G2" s="53" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="H2" s="51" t="inlineStr">
+      <c r="H2" s="54" t="inlineStr">
         <is>
           <t>← langue du devis : 1 = français, 2 = anglais</t>
         </is>
       </c>
-      <c r="J2" s="50" t="inlineStr">
+      <c r="J2" s="53" t="inlineStr">
         <is>
           <t>Palette</t>
         </is>
       </c>
-      <c r="K2" s="50" t="inlineStr">
+      <c r="K2" s="53" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L2" s="50" t="inlineStr">
+      <c r="L2" s="53" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="M2" s="50" t="inlineStr">
+      <c r="M2" s="53" t="inlineStr">
         <is>
           <t>Coût réel +15 %</t>
         </is>
       </c>
-      <c r="N2" s="50" t="inlineStr">
+      <c r="N2" s="53" t="inlineStr">
         <is>
           <t>Forfait calculé (S + O + UC)</t>
         </is>
       </c>
-      <c r="P2" s="50" t="inlineStr">
+      <c r="P2" s="53" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="Q2" s="50" t="inlineStr">
+      <c r="Q2" s="53" t="inlineStr">
         <is>
           <t>Taille OK</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="53" t="inlineStr">
         <is>
           <t>Alexis ESTINES</t>
         </is>
       </c>
-      <c r="B3" s="50" t="inlineStr">
+      <c r="B3" s="53" t="inlineStr">
         <is>
           <t>aestines@enedril.fr</t>
         </is>
       </c>
-      <c r="D3" s="50" t="inlineStr">
+      <c r="D3" s="53" t="inlineStr">
         <is>
           <t>FCA Lons</t>
         </is>
       </c>
-      <c r="E3" s="50" t="inlineStr">
+      <c r="E3" s="53" t="inlineStr">
         <is>
           <t>30 jours / 30 days</t>
         </is>
       </c>
-      <c r="F3" s="50" t="inlineStr">
+      <c r="F3" s="53" t="inlineStr">
         <is>
           <t>30 jours fin de mois / 30 days end of month</t>
         </is>
       </c>
-      <c r="G3" s="50" t="inlineStr">
+      <c r="G3" s="53" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="J3" s="50" t="inlineStr">
+      <c r="J3" s="53" t="inlineStr">
         <is>
           <t>Fishing basket</t>
         </is>
       </c>
-      <c r="K3" s="50" t="inlineStr">
+      <c r="K3" s="53" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="L3" s="50" t="inlineStr">
+      <c r="L3" s="53" t="inlineStr">
         <is>
           <t>€/jour</t>
         </is>
       </c>
-      <c r="M3" s="50" t="inlineStr">
+      <c r="M3" s="53" t="inlineStr">
         <is>
           <t>Forfait</t>
         </is>
       </c>
-      <c r="N3" s="50" t="inlineStr">
+      <c r="N3" s="53" t="inlineStr">
         <is>
           <t>Forfait global</t>
         </is>
       </c>
-      <c r="P3" s="50" t="inlineStr">
+      <c r="P3" s="53" t="inlineStr">
         <is>
           <t>En cours</t>
         </is>
       </c>
-      <c r="Q3" s="50" t="inlineStr">
+      <c r="Q3" s="53" t="inlineStr">
         <is>
           <t>Test OK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="53" t="inlineStr">
         <is>
           <t>Paul HYNDERICK</t>
         </is>
       </c>
-      <c r="B4" s="50" t="inlineStr">
+      <c r="B4" s="53" t="inlineStr">
         <is>
           <t>phynderick@enedril.fr</t>
         </is>
       </c>
-      <c r="D4" s="50" t="inlineStr">
+      <c r="D4" s="53" t="inlineStr">
         <is>
           <t>DAP</t>
         </is>
       </c>
-      <c r="E4" s="50" t="inlineStr">
+      <c r="E4" s="53" t="inlineStr">
         <is>
           <t>60 jours / 60 days</t>
         </is>
       </c>
-      <c r="F4" s="50" t="inlineStr">
+      <c r="F4" s="53" t="inlineStr">
         <is>
           <t>45 jours fin de mois / 45 days end of month</t>
         </is>
       </c>
-      <c r="J4" s="50" t="inlineStr">
+      <c r="J4" s="53" t="inlineStr">
         <is>
           <t>Caisse</t>
         </is>
       </c>
-      <c r="K4" s="50" t="inlineStr">
+      <c r="K4" s="53" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="L4" s="50" t="inlineStr">
+      <c r="L4" s="53" t="inlineStr">
         <is>
           <t>€/jour/pers</t>
         </is>
       </c>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="N4" s="53" t="inlineStr">
         <is>
           <t>Forfait par jour</t>
         </is>
       </c>
-      <c r="Q4" s="50" t="inlineStr">
+      <c r="Q4" s="53" t="inlineStr">
         <is>
           <t>Taille + test OK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="50" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Céline CARDONA</t>
         </is>
       </c>
-      <c r="B5" s="50" t="inlineStr">
+      <c r="B5" s="53" t="inlineStr">
         <is>
           <t>ccardona@enedril.fr</t>
         </is>
       </c>
-      <c r="D5" s="50" t="inlineStr">
+      <c r="D5" s="53" t="inlineStr">
         <is>
           <t>DDP</t>
         </is>
       </c>
-      <c r="E5" s="50" t="inlineStr">
+      <c r="E5" s="53" t="inlineStr">
         <is>
           <t>90 jours / 90 days</t>
         </is>
       </c>
-      <c r="F5" s="50" t="inlineStr">
+      <c r="F5" s="53" t="inlineStr">
         <is>
           <t>À la commande / Upon order</t>
         </is>
       </c>
-      <c r="J5" s="50" t="inlineStr">
+      <c r="J5" s="53" t="inlineStr">
         <is>
           <t>Vrac</t>
         </is>
       </c>
-      <c r="K5" s="50" t="inlineStr">
+      <c r="K5" s="53" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="L5" s="53" t="inlineStr">
         <is>
           <t>€/pers</t>
         </is>
       </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="Q5" s="53" t="inlineStr">
         <is>
           <t>À contrôler</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="50" t="inlineStr">
+      <c r="A6" s="53" t="inlineStr">
         <is>
           <t>Koen MONDELAERS</t>
         </is>
       </c>
-      <c r="B6" s="50" t="inlineStr">
+      <c r="B6" s="53" t="inlineStr">
         <is>
           <t>kmondelaers@enedril.fr</t>
         </is>
       </c>
-      <c r="D6" s="50" t="inlineStr">
+      <c r="D6" s="53" t="inlineStr">
         <is>
           <t>FOB</t>
         </is>
       </c>
-      <c r="K6" s="50" t="inlineStr">
+      <c r="K6" s="53" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="L6" s="50" t="inlineStr">
+      <c r="L6" s="53" t="inlineStr">
         <is>
           <t>€/unité</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="50" t="inlineStr">
+      <c r="A7" s="53" t="inlineStr">
         <is>
           <t>Luigi LIBERATORE</t>
         </is>
       </c>
-      <c r="B7" s="50" t="inlineStr">
+      <c r="B7" s="53" t="inlineStr">
         <is>
           <t>lliberatore@enedril.fr</t>
         </is>
       </c>
-      <c r="K7" s="50" t="inlineStr">
+      <c r="K7" s="53" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="K8" s="50" t="inlineStr">
+      <c r="K8" s="53" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="K9" s="50" t="inlineStr">
+      <c r="K9" s="53" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
@@ -3811,21 +3491,21 @@
           <t>Pour ajouter un contact, une validité, etc. : écrire à la suite dans la colonne (les listes déroulantes lisent les 12 premières lignes).</t>
         </is>
       </c>
-      <c r="K10" s="50" t="inlineStr">
+      <c r="K10" s="53" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="K11" s="50" t="inlineStr">
+      <c r="K11" s="53" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="K12" s="50" t="inlineStr">
+      <c r="K12" s="53" t="inlineStr">
         <is>
           <t>Vrac</t>
         </is>

</xml_diff>

<commit_message>
Tool list : descriptions sans gras, 3 colis
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Tool_List_Enedril_2027.xlsx
+++ b/devis_2027/Tool_List_Enedril_2027.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Tool List'!$A$14:$V$54</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'2 Tool List'!$A$1:$I$67</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'2 Tool List'!$A$1:$I$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="#,##0.0 &quot;kg&quot;"/>
     <numFmt numFmtId="169" formatCode="0.000 &quot;m³&quot;"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -157,7 +157,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="000B1B2E"/>
       <sz val="13"/>
     </font>
@@ -188,11 +187,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0008203F"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="000B1B2E"/>
       <sz val="13"/>
     </font>
     <font>
@@ -387,25 +381,25 @@
     <xf numFmtId="167" fontId="23" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="28" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="29" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="29" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1368,7 +1362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V67"/>
+  <dimension ref="A1:V64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2906,79 +2900,25 @@
       </c>
       <c r="I63" s="45" t="n"/>
     </row>
-    <row r="64" ht="36" customHeight="1">
-      <c r="A64" s="39" t="inlineStr">
-        <is>
-          <t>Colis 4</t>
-        </is>
-      </c>
-      <c r="B64" s="40" t="n"/>
-      <c r="C64" s="41" t="n"/>
-      <c r="D64" s="42" t="n"/>
-      <c r="E64" s="42" t="n"/>
-      <c r="F64" s="42" t="n"/>
-      <c r="G64" s="43" t="n"/>
-      <c r="H64" s="44">
-        <f>IF(COUNT(D64:F64)=3,D64*E64*F64/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="I64" s="45" t="n"/>
-    </row>
-    <row r="65" ht="36" customHeight="1">
-      <c r="A65" s="39" t="inlineStr">
-        <is>
-          <t>Colis 5</t>
-        </is>
-      </c>
-      <c r="B65" s="40" t="n"/>
-      <c r="C65" s="41" t="n"/>
-      <c r="D65" s="42" t="n"/>
-      <c r="E65" s="42" t="n"/>
-      <c r="F65" s="42" t="n"/>
-      <c r="G65" s="43" t="n"/>
-      <c r="H65" s="44">
-        <f>IF(COUNT(D65:F65)=3,D65*E65*F65/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="I65" s="45" t="n"/>
-    </row>
-    <row r="66" ht="36" customHeight="1">
-      <c r="A66" s="39" t="inlineStr">
-        <is>
-          <t>Colis 6</t>
-        </is>
-      </c>
-      <c r="B66" s="40" t="n"/>
-      <c r="C66" s="41" t="n"/>
-      <c r="D66" s="42" t="n"/>
-      <c r="E66" s="42" t="n"/>
-      <c r="F66" s="42" t="n"/>
-      <c r="G66" s="43" t="n"/>
-      <c r="H66" s="44">
-        <f>IF(COUNT(D66:F66)=3,D66*E66*F66/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="I66" s="45" t="n"/>
-    </row>
-    <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="46">
-        <f>"TOTAL  ·  "&amp;COUNTA(C61:C66)&amp;" colis"</f>
-        <v/>
-      </c>
-      <c r="B67" s="47" t="n"/>
-      <c r="C67" s="47" t="n"/>
-      <c r="D67" s="48" t="n"/>
-      <c r="E67" s="48" t="n"/>
-      <c r="F67" s="48" t="n"/>
-      <c r="G67" s="49">
-        <f>SUM(G61:G66)</f>
-        <v/>
-      </c>
-      <c r="H67" s="50">
-        <f>SUM(H61:H66)</f>
-        <v/>
-      </c>
-      <c r="I67" s="48" t="n"/>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="46">
+        <f>"TOTAL  ·  "&amp;COUNTA(C61:C63)&amp;" colis"</f>
+        <v/>
+      </c>
+      <c r="B64" s="47" t="n"/>
+      <c r="C64" s="47" t="n"/>
+      <c r="D64" s="48" t="n"/>
+      <c r="E64" s="48" t="n"/>
+      <c r="F64" s="48" t="n"/>
+      <c r="G64" s="49">
+        <f>SUM(G61:G63)</f>
+        <v/>
+      </c>
+      <c r="H64" s="50">
+        <f>SUM(H61:H63)</f>
+        <v/>
+      </c>
+      <c r="I64" s="48" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A14:V54">
@@ -3009,9 +2949,8 @@
     <filterColumn colId="20" hiddenButton="1" showButton="0"/>
     <filterColumn colId="21" hiddenButton="1" showButton="0"/>
   </autoFilter>
-  <mergeCells count="35">
+  <mergeCells count="32">
     <mergeCell ref="D9:G9"/>
-    <mergeCell ref="A64:B64"/>
     <mergeCell ref="A60:B60"/>
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="H10:I10"/>
@@ -3023,11 +2962,9 @@
     <mergeCell ref="A61:B61"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A65:B65"/>
     <mergeCell ref="D57:E57"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A66:B66"/>
     <mergeCell ref="D10:G10"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A13:C13"/>
@@ -3036,8 +2973,8 @@
     <mergeCell ref="E2:I2"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A67:C67"/>
     <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A64:C64"/>
     <mergeCell ref="A59:I59"/>
     <mergeCell ref="A62:B62"/>
     <mergeCell ref="A11:I11"/>
@@ -3054,7 +2991,7 @@
       <formula>$T15&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="7">
+  <dataValidations count="4">
     <dataValidation sqref="H15:H54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$Q$2:$Q$12</formula1>
     </dataValidation>
@@ -3065,15 +3002,6 @@
       <formula1>=Listes!$J$2:$J$12</formula1>
     </dataValidation>
     <dataValidation sqref="C63" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$J$2:$J$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="C64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$J$2:$J$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="C65" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
-      <formula1>=Listes!$J$2:$J$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="C66" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$J$2:$J$12</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>